<commit_message>
Rename sheets: Rooms -> Clearances, Types -> Shop Drawings
</commit_message>
<xml_diff>
--- a/WPH_Room_Register.xlsx
+++ b/WPH_Room_Register.xlsx
@@ -8,15 +8,15 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rooms" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Types" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clearances" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shop Drawings" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fields" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Rooms'!$A$1:$M$554</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Clearances'!$A$1:$M$554</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
@@ -577,7 +577,7 @@
     <row r="5" ht="15" customHeight="1" s="11">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>1. Edit the Rooms sheet (per-room data: clearances, remarks) or the Types sheet (per-typology data: shop drawing status). Use the drop-down lists.</t>
+          <t>1. Edit the Clearances sheet (per-room data: clearances, remarks) or the Shop Drawings sheet (per-typology data: shop drawing status). Use the drop-down lists.</t>
         </is>
       </c>
     </row>
@@ -608,21 +608,21 @@
     <row r="10" ht="15" customHeight="1" s="11">
       <c r="A10" s="13" t="inlineStr">
         <is>
-          <t>• Types sheet = default per room type (e.g. ID shop drawing status of K01C applies to every K01C room).</t>
+          <t>• Shop Drawings sheet = default per room type (e.g. ID shop drawing status of K01C applies to every K01C room).</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="11">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>• Rooms sheet = per room. If a column with the same header exists in Rooms and is filled, it overrides the Types value for that room only.</t>
+          <t>• Clearances sheet = per room. If a column with the same header exists in Clearances and is filled, it overrides the Shop Drawings value for that room only.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="11">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>• Room counts and percentages are calculated automatically by the page from the Rooms sheet. Do not type them.</t>
+          <t>• Room counts and percentages are calculated automatically by the page from the Clearances sheet. Do not type them.</t>
         </is>
       </c>
     </row>
@@ -639,7 +639,7 @@
     <row r="15" ht="15" customHeight="1" s="11">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>1. Add a new column to Rooms (per room) or Types (per type) with a clear header, e.g. "Snagging Status".</t>
+          <t>1. Add a new column to Clearances (per room) or Shop Drawings (per type) with a clear header, e.g. "Snagging Status".</t>
         </is>
       </c>
     </row>
@@ -726,6 +726,7 @@
         </is>
       </c>
     </row>
+    <row r="29"/>
     <row r="30">
       <c r="A30" s="20" t="inlineStr">
         <is>
@@ -736,7 +737,7 @@
     <row r="31">
       <c r="A31" s="21" t="inlineStr">
         <is>
-          <t>Fixed information is locked. Cells you can update are shaded light yellow: Rooms (clearances, dates, remarks), Types (drawing ref, revision, statuses, dates), Config (data last updated, updated by). Spare columns to the right of Rooms/Types and spare rows below Fields/Lists are open for adding new information. Filtering and sorting are allowed on Rooms and Types. To change locked cells: Review &gt; Unprotect Sheet (password held by the Technical Department).</t>
+          <t>Fixed information is locked. Cells you can update are shaded light yellow: Clearances (clearances, dates, remarks), Shop Drawings (drawing ref, revision, statuses, dates), Config (data last updated, updated by). Spare columns to the right of Clearances/Shop Drawings and spare rows below Fields/Lists are open for adding new information. Filtering and sorting are allowed on Clearances and Shop Drawings. To change locked cells: Review &gt; Unprotect Sheet (password held by the Technical Department).</t>
         </is>
       </c>
     </row>
@@ -39834,19 +39835,19 @@
         </is>
       </c>
       <c r="C2" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A2,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A2,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D2" s="17">
-        <f>C2/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C2/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E2" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A2,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A2,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F2" s="17">
-        <f>E2/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E2/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G2" s="10">
@@ -39854,7 +39855,7 @@
         <v/>
       </c>
       <c r="H2" s="17">
-        <f>G2/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G2/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -39870,19 +39871,19 @@
         </is>
       </c>
       <c r="C3" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A3,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A3,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D3" s="17">
-        <f>C3/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C3/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E3" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A3,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A3,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F3" s="17">
-        <f>E3/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E3/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G3" s="10">
@@ -39890,7 +39891,7 @@
         <v/>
       </c>
       <c r="H3" s="17">
-        <f>G3/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G3/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -39906,19 +39907,19 @@
         </is>
       </c>
       <c r="C4" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A4,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A4,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D4" s="17">
-        <f>C4/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C4/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E4" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A4,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A4,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F4" s="17">
-        <f>E4/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E4/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G4" s="10">
@@ -39926,7 +39927,7 @@
         <v/>
       </c>
       <c r="H4" s="17">
-        <f>G4/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G4/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -39942,19 +39943,19 @@
         </is>
       </c>
       <c r="C5" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A5,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A5,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D5" s="17">
-        <f>C5/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C5/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A5,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A5,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F5" s="17">
-        <f>E5/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E5/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -39962,7 +39963,7 @@
         <v/>
       </c>
       <c r="H5" s="17">
-        <f>G5/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G5/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -39978,19 +39979,19 @@
         </is>
       </c>
       <c r="C6" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A6,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A6,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D6" s="17">
-        <f>C6/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C6/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E6" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A6,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A6,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F6" s="17">
-        <f>E6/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E6/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G6" s="10">
@@ -39998,7 +39999,7 @@
         <v/>
       </c>
       <c r="H6" s="17">
-        <f>G6/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G6/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -40014,19 +40015,19 @@
         </is>
       </c>
       <c r="C7" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A7,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A7,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D7" s="17">
-        <f>C7/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C7/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A7,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A7,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F7" s="17">
-        <f>E7/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E7/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -40034,7 +40035,7 @@
         <v/>
       </c>
       <c r="H7" s="17">
-        <f>G7/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G7/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -40050,19 +40051,19 @@
         </is>
       </c>
       <c r="C8" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A8,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A8,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D8" s="17">
-        <f>C8/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C8/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E8" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A8,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A8,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F8" s="17">
-        <f>E8/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E8/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G8" s="10">
@@ -40070,7 +40071,7 @@
         <v/>
       </c>
       <c r="H8" s="17">
-        <f>G8/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G8/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -40086,19 +40087,19 @@
         </is>
       </c>
       <c r="C9" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A9,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A9,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D9" s="17">
-        <f>C9/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C9/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A9,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A9,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F9" s="17">
-        <f>E9/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E9/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -40106,7 +40107,7 @@
         <v/>
       </c>
       <c r="H9" s="17">
-        <f>G9/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G9/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -40122,19 +40123,19 @@
         </is>
       </c>
       <c r="C10" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A10,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A10,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D10" s="17">
-        <f>C10/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C10/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E10" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A10,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A10,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F10" s="17">
-        <f>E10/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E10/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G10" s="10">
@@ -40142,7 +40143,7 @@
         <v/>
       </c>
       <c r="H10" s="17">
-        <f>G10/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G10/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -40158,19 +40159,19 @@
         </is>
       </c>
       <c r="C11" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A11,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A11,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D11" s="17">
-        <f>C11/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C11/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A11,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A11,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F11" s="17">
-        <f>E11/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E11/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -40178,7 +40179,7 @@
         <v/>
       </c>
       <c r="H11" s="17">
-        <f>G11/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G11/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -40194,19 +40195,19 @@
         </is>
       </c>
       <c r="C12" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A12,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A12,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D12" s="17">
-        <f>C12/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C12/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E12" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A12,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A12,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F12" s="17">
-        <f>E12/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E12/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G12" s="10">
@@ -40214,7 +40215,7 @@
         <v/>
       </c>
       <c r="H12" s="17">
-        <f>G12/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G12/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -40230,19 +40231,19 @@
         </is>
       </c>
       <c r="C13" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A13,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A13,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D13" s="17">
-        <f>C13/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C13/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A13,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A13,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F13" s="17">
-        <f>E13/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E13/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -40250,7 +40251,7 @@
         <v/>
       </c>
       <c r="H13" s="17">
-        <f>G13/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G13/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -40266,19 +40267,19 @@
         </is>
       </c>
       <c r="C14" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A14,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A14,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D14" s="17">
-        <f>C14/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C14/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E14" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A14,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A14,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F14" s="17">
-        <f>E14/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E14/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G14" s="10">
@@ -40286,7 +40287,7 @@
         <v/>
       </c>
       <c r="H14" s="17">
-        <f>G14/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G14/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -40302,19 +40303,19 @@
         </is>
       </c>
       <c r="C15" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A15,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A15,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D15" s="17">
-        <f>C15/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C15/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A15,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A15,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F15" s="17">
-        <f>E15/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E15/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G15" s="10">
@@ -40322,7 +40323,7 @@
         <v/>
       </c>
       <c r="H15" s="17">
-        <f>G15/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G15/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -40338,19 +40339,19 @@
         </is>
       </c>
       <c r="C16" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A16,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A16,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D16" s="17">
-        <f>C16/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C16/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E16" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A16,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A16,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F16" s="17">
-        <f>E16/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E16/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G16" s="10">
@@ -40358,7 +40359,7 @@
         <v/>
       </c>
       <c r="H16" s="17">
-        <f>G16/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G16/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -40374,19 +40375,19 @@
         </is>
       </c>
       <c r="C17" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A17,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A17,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D17" s="17">
-        <f>C17/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C17/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A17,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A17,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F17" s="17">
-        <f>E17/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E17/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G17" s="10">
@@ -40394,7 +40395,7 @@
         <v/>
       </c>
       <c r="H17" s="17">
-        <f>G17/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G17/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -40410,19 +40411,19 @@
         </is>
       </c>
       <c r="C18" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A18,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A18,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D18" s="17">
-        <f>C18/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C18/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E18" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A18,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A18,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F18" s="17">
-        <f>E18/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E18/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G18" s="10">
@@ -40430,7 +40431,7 @@
         <v/>
       </c>
       <c r="H18" s="17">
-        <f>G18/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G18/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -40446,19 +40447,19 @@
         </is>
       </c>
       <c r="C19" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A19,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A19,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D19" s="17">
-        <f>C19/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C19/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A19,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A19,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F19" s="17">
-        <f>E19/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E19/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G19" s="10">
@@ -40466,7 +40467,7 @@
         <v/>
       </c>
       <c r="H19" s="17">
-        <f>G19/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G19/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -40482,19 +40483,19 @@
         </is>
       </c>
       <c r="C20" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A20,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A20,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D20" s="17">
-        <f>C20/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C20/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E20" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A20,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A20,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F20" s="17">
-        <f>E20/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E20/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G20" s="10">
@@ -40502,7 +40503,7 @@
         <v/>
       </c>
       <c r="H20" s="17">
-        <f>G20/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G20/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -40518,19 +40519,19 @@
         </is>
       </c>
       <c r="C21" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A21,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A21,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D21" s="17">
-        <f>C21/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C21/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A21,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A21,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F21" s="17">
-        <f>E21/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E21/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G21" s="10">
@@ -40538,7 +40539,7 @@
         <v/>
       </c>
       <c r="H21" s="17">
-        <f>G21/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G21/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -40554,19 +40555,19 @@
         </is>
       </c>
       <c r="C22" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A22,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A22,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D22" s="17">
-        <f>C22/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C22/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E22" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A22,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A22,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F22" s="17">
-        <f>E22/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E22/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G22" s="10">
@@ -40574,7 +40575,7 @@
         <v/>
       </c>
       <c r="H22" s="17">
-        <f>G22/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G22/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -40590,19 +40591,19 @@
         </is>
       </c>
       <c r="C23" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A23,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A23,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D23" s="17">
-        <f>C23/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C23/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E23" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A23,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A23,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F23" s="17">
-        <f>E23/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E23/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G23" s="10">
@@ -40610,7 +40611,7 @@
         <v/>
       </c>
       <c r="H23" s="17">
-        <f>G23/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G23/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -40626,19 +40627,19 @@
         </is>
       </c>
       <c r="C24" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A24,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A24,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D24" s="17">
-        <f>C24/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C24/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E24" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A24,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A24,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F24" s="17">
-        <f>E24/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E24/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G24" s="10">
@@ -40646,7 +40647,7 @@
         <v/>
       </c>
       <c r="H24" s="17">
-        <f>G24/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G24/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -40662,19 +40663,19 @@
         </is>
       </c>
       <c r="C25" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A25,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A25,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D25" s="17">
-        <f>C25/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C25/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E25" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A25,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A25,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F25" s="17">
-        <f>E25/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E25/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G25" s="10">
@@ -40682,7 +40683,7 @@
         <v/>
       </c>
       <c r="H25" s="17">
-        <f>G25/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G25/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -40698,19 +40699,19 @@
         </is>
       </c>
       <c r="C26" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A26,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A26,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D26" s="17">
-        <f>C26/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C26/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E26" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A26,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A26,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F26" s="17">
-        <f>E26/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E26/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G26" s="10">
@@ -40718,7 +40719,7 @@
         <v/>
       </c>
       <c r="H26" s="17">
-        <f>G26/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G26/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -40734,19 +40735,19 @@
         </is>
       </c>
       <c r="C27" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A27,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A27,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D27" s="17">
-        <f>C27/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C27/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E27" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A27,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A27,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F27" s="17">
-        <f>E27/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E27/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G27" s="10">
@@ -40754,7 +40755,7 @@
         <v/>
       </c>
       <c r="H27" s="17">
-        <f>G27/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G27/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -40770,19 +40771,19 @@
         </is>
       </c>
       <c r="C28" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A28,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A28,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D28" s="17">
-        <f>C28/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C28/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E28" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A28,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A28,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F28" s="17">
-        <f>E28/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E28/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G28" s="10">
@@ -40790,7 +40791,7 @@
         <v/>
       </c>
       <c r="H28" s="17">
-        <f>G28/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G28/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -40806,19 +40807,19 @@
         </is>
       </c>
       <c r="C29" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A29,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A29,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D29" s="17">
-        <f>C29/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C29/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E29" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A29,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A29,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F29" s="17">
-        <f>E29/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E29/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G29" s="10">
@@ -40826,7 +40827,7 @@
         <v/>
       </c>
       <c r="H29" s="17">
-        <f>G29/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G29/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -40842,19 +40843,19 @@
         </is>
       </c>
       <c r="C30" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A30,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A30,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D30" s="17">
-        <f>C30/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C30/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E30" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A30,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A30,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F30" s="17">
-        <f>E30/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E30/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G30" s="10">
@@ -40862,7 +40863,7 @@
         <v/>
       </c>
       <c r="H30" s="17">
-        <f>G30/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G30/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -40878,19 +40879,19 @@
         </is>
       </c>
       <c r="C31" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A31,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A31,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D31" s="17">
-        <f>C31/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C31/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E31" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A31,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A31,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F31" s="17">
-        <f>E31/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E31/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G31" s="10">
@@ -40898,7 +40899,7 @@
         <v/>
       </c>
       <c r="H31" s="17">
-        <f>G31/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G31/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -40914,19 +40915,19 @@
         </is>
       </c>
       <c r="C32" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A32,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A32,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D32" s="17">
-        <f>C32/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C32/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E32" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A32,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A32,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F32" s="17">
-        <f>E32/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E32/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G32" s="10">
@@ -40934,7 +40935,7 @@
         <v/>
       </c>
       <c r="H32" s="17">
-        <f>G32/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G32/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -40950,19 +40951,19 @@
         </is>
       </c>
       <c r="C33" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A33,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A33,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D33" s="17">
-        <f>C33/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C33/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E33" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A33,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A33,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F33" s="17">
-        <f>E33/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E33/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G33" s="10">
@@ -40970,7 +40971,7 @@
         <v/>
       </c>
       <c r="H33" s="17">
-        <f>G33/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G33/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -40986,19 +40987,19 @@
         </is>
       </c>
       <c r="C34" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A34,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A34,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D34" s="17">
-        <f>C34/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C34/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E34" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A34,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A34,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F34" s="17">
-        <f>E34/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E34/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G34" s="10">
@@ -41006,7 +41007,7 @@
         <v/>
       </c>
       <c r="H34" s="17">
-        <f>G34/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G34/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -41022,19 +41023,19 @@
         </is>
       </c>
       <c r="C35" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A35,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A35,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D35" s="17">
-        <f>C35/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C35/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E35" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A35,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A35,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F35" s="17">
-        <f>E35/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E35/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G35" s="10">
@@ -41042,7 +41043,7 @@
         <v/>
       </c>
       <c r="H35" s="17">
-        <f>G35/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G35/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -41058,19 +41059,19 @@
         </is>
       </c>
       <c r="C36" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A36,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A36,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D36" s="17">
-        <f>C36/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C36/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E36" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A36,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A36,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F36" s="17">
-        <f>E36/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E36/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G36" s="10">
@@ -41078,7 +41079,7 @@
         <v/>
       </c>
       <c r="H36" s="17">
-        <f>G36/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G36/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -41094,19 +41095,19 @@
         </is>
       </c>
       <c r="C37" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A37,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A37,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D37" s="17">
-        <f>C37/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C37/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E37" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A37,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A37,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F37" s="17">
-        <f>E37/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E37/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G37" s="10">
@@ -41114,7 +41115,7 @@
         <v/>
       </c>
       <c r="H37" s="17">
-        <f>G37/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G37/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -41130,19 +41131,19 @@
         </is>
       </c>
       <c r="C38" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A38,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A38,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D38" s="17">
-        <f>C38/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C38/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E38" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A38,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A38,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F38" s="17">
-        <f>E38/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E38/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G38" s="10">
@@ -41150,7 +41151,7 @@
         <v/>
       </c>
       <c r="H38" s="17">
-        <f>G38/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G38/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -41166,19 +41167,19 @@
         </is>
       </c>
       <c r="C39" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A39,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A39,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D39" s="17">
-        <f>C39/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C39/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E39" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A39,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A39,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F39" s="17">
-        <f>E39/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E39/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G39" s="10">
@@ -41186,7 +41187,7 @@
         <v/>
       </c>
       <c r="H39" s="17">
-        <f>G39/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G39/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -41202,19 +41203,19 @@
         </is>
       </c>
       <c r="C40" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A40,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A40,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D40" s="17">
-        <f>C40/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C40/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E40" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A40,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A40,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F40" s="17">
-        <f>E40/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E40/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G40" s="10">
@@ -41222,7 +41223,7 @@
         <v/>
       </c>
       <c r="H40" s="17">
-        <f>G40/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G40/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -41238,19 +41239,19 @@
         </is>
       </c>
       <c r="C41" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A41,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A41,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D41" s="17">
-        <f>C41/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C41/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E41" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A41,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A41,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F41" s="17">
-        <f>E41/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E41/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G41" s="10">
@@ -41258,7 +41259,7 @@
         <v/>
       </c>
       <c r="H41" s="17">
-        <f>G41/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G41/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -41274,19 +41275,19 @@
         </is>
       </c>
       <c r="C42" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A42,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A42,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D42" s="17">
-        <f>C42/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C42/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E42" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A42,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A42,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F42" s="17">
-        <f>E42/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E42/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G42" s="10">
@@ -41294,7 +41295,7 @@
         <v/>
       </c>
       <c r="H42" s="17">
-        <f>G42/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G42/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -41310,19 +41311,19 @@
         </is>
       </c>
       <c r="C43" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A43,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A43,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D43" s="17">
-        <f>C43/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C43/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E43" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A43,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A43,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F43" s="17">
-        <f>E43/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E43/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G43" s="10">
@@ -41330,7 +41331,7 @@
         <v/>
       </c>
       <c r="H43" s="17">
-        <f>G43/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G43/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -41346,19 +41347,19 @@
         </is>
       </c>
       <c r="C44" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A44,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A44,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D44" s="17">
-        <f>C44/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C44/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E44" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A44,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A44,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F44" s="17">
-        <f>E44/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E44/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G44" s="10">
@@ -41366,7 +41367,7 @@
         <v/>
       </c>
       <c r="H44" s="17">
-        <f>G44/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G44/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -41382,19 +41383,19 @@
         </is>
       </c>
       <c r="C45" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A45,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A45,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D45" s="17">
-        <f>C45/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C45/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E45" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A45,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A45,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F45" s="17">
-        <f>E45/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E45/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G45" s="10">
@@ -41402,7 +41403,7 @@
         <v/>
       </c>
       <c r="H45" s="17">
-        <f>G45/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G45/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -41418,19 +41419,19 @@
         </is>
       </c>
       <c r="C46" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A46,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A46,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D46" s="17">
-        <f>C46/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C46/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E46" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A46,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A46,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F46" s="17">
-        <f>E46/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E46/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G46" s="10">
@@ -41438,7 +41439,7 @@
         <v/>
       </c>
       <c r="H46" s="17">
-        <f>G46/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G46/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -41454,19 +41455,19 @@
         </is>
       </c>
       <c r="C47" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A47,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A47,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D47" s="17">
-        <f>C47/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C47/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E47" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A47,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A47,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F47" s="17">
-        <f>E47/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E47/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G47" s="10">
@@ -41474,7 +41475,7 @@
         <v/>
       </c>
       <c r="H47" s="17">
-        <f>G47/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G47/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -41490,19 +41491,19 @@
         </is>
       </c>
       <c r="C48" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A48,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A48,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D48" s="17">
-        <f>C48/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C48/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E48" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A48,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A48,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F48" s="17">
-        <f>E48/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E48/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G48" s="10">
@@ -41510,7 +41511,7 @@
         <v/>
       </c>
       <c r="H48" s="17">
-        <f>G48/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G48/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -41526,19 +41527,19 @@
         </is>
       </c>
       <c r="C49" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A49,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A49,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D49" s="17">
-        <f>C49/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C49/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E49" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A49,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A49,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F49" s="17">
-        <f>E49/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E49/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G49" s="10">
@@ -41546,7 +41547,7 @@
         <v/>
       </c>
       <c r="H49" s="17">
-        <f>G49/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G49/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -41562,19 +41563,19 @@
         </is>
       </c>
       <c r="C50" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A50,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A50,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D50" s="17">
-        <f>C50/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C50/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E50" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A50,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A50,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F50" s="17">
-        <f>E50/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E50/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G50" s="10">
@@ -41582,7 +41583,7 @@
         <v/>
       </c>
       <c r="H50" s="17">
-        <f>G50/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G50/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -41598,19 +41599,19 @@
         </is>
       </c>
       <c r="C51" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A51,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A51,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D51" s="17">
-        <f>C51/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C51/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E51" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A51,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A51,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F51" s="17">
-        <f>E51/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E51/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G51" s="10">
@@ -41618,7 +41619,7 @@
         <v/>
       </c>
       <c r="H51" s="17">
-        <f>G51/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G51/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -41634,19 +41635,19 @@
         </is>
       </c>
       <c r="C52" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A52,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A52,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D52" s="17">
-        <f>C52/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C52/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E52" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A52,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A52,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F52" s="17">
-        <f>E52/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E52/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G52" s="10">
@@ -41654,7 +41655,7 @@
         <v/>
       </c>
       <c r="H52" s="17">
-        <f>G52/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G52/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -41670,19 +41671,19 @@
         </is>
       </c>
       <c r="C53" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A53,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A53,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D53" s="17">
-        <f>C53/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C53/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E53" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A53,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A53,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F53" s="17">
-        <f>E53/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E53/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G53" s="10">
@@ -41690,7 +41691,7 @@
         <v/>
       </c>
       <c r="H53" s="17">
-        <f>G53/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G53/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -41706,19 +41707,19 @@
         </is>
       </c>
       <c r="C54" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A54,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A54,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D54" s="17">
-        <f>C54/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C54/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E54" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A54,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A54,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F54" s="17">
-        <f>E54/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E54/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G54" s="10">
@@ -41726,7 +41727,7 @@
         <v/>
       </c>
       <c r="H54" s="17">
-        <f>G54/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G54/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -41742,19 +41743,19 @@
         </is>
       </c>
       <c r="C55" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A55,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A55,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D55" s="17">
-        <f>C55/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C55/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E55" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A55,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A55,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F55" s="17">
-        <f>E55/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E55/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G55" s="10">
@@ -41762,7 +41763,7 @@
         <v/>
       </c>
       <c r="H55" s="17">
-        <f>G55/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G55/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -41778,19 +41779,19 @@
         </is>
       </c>
       <c r="C56" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A56,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A56,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D56" s="17">
-        <f>C56/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C56/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E56" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A56,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A56,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F56" s="17">
-        <f>E56/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E56/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G56" s="10">
@@ -41798,7 +41799,7 @@
         <v/>
       </c>
       <c r="H56" s="17">
-        <f>G56/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G56/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -41814,19 +41815,19 @@
         </is>
       </c>
       <c r="C57" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A57,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A57,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D57" s="17">
-        <f>C57/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C57/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E57" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A57,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A57,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F57" s="17">
-        <f>E57/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E57/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G57" s="10">
@@ -41834,7 +41835,7 @@
         <v/>
       </c>
       <c r="H57" s="17">
-        <f>G57/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G57/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -41850,19 +41851,19 @@
         </is>
       </c>
       <c r="C58" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A58,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A58,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D58" s="17">
-        <f>C58/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C58/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E58" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A58,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A58,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F58" s="17">
-        <f>E58/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E58/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G58" s="10">
@@ -41870,7 +41871,7 @@
         <v/>
       </c>
       <c r="H58" s="17">
-        <f>G58/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G58/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -41886,19 +41887,19 @@
         </is>
       </c>
       <c r="C59" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A59,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A59,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D59" s="17">
-        <f>C59/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C59/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E59" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A59,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A59,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F59" s="17">
-        <f>E59/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E59/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G59" s="10">
@@ -41906,7 +41907,7 @@
         <v/>
       </c>
       <c r="H59" s="17">
-        <f>G59/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G59/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -41922,19 +41923,19 @@
         </is>
       </c>
       <c r="C60" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A60,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A60,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D60" s="17">
-        <f>C60/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C60/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E60" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A60,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A60,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F60" s="17">
-        <f>E60/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E60/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G60" s="10">
@@ -41942,7 +41943,7 @@
         <v/>
       </c>
       <c r="H60" s="17">
-        <f>G60/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G60/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -41958,19 +41959,19 @@
         </is>
       </c>
       <c r="C61" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A61,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A61,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D61" s="17">
-        <f>C61/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C61/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E61" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A61,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A61,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F61" s="17">
-        <f>E61/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E61/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G61" s="10">
@@ -41978,7 +41979,7 @@
         <v/>
       </c>
       <c r="H61" s="17">
-        <f>G61/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G61/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>
@@ -41994,19 +41995,19 @@
         </is>
       </c>
       <c r="C62" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A62,Rooms!$B:$B,"Tower A")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A62,Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="D62" s="17">
-        <f>C62/COUNTIF(Rooms!$B:$B,"Tower A")</f>
+        <f>C62/COUNTIF(Clearances!$B:$B,"Tower A")</f>
         <v/>
       </c>
       <c r="E62" s="10">
-        <f>COUNTIFS(Rooms!$E:$E,$A62,Rooms!$B:$B,"Tower B")</f>
+        <f>COUNTIFS(Clearances!$E:$E,$A62,Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="F62" s="17">
-        <f>E62/COUNTIF(Rooms!$B:$B,"Tower B")</f>
+        <f>E62/COUNTIF(Clearances!$B:$B,"Tower B")</f>
         <v/>
       </c>
       <c r="G62" s="10">
@@ -42014,7 +42015,7 @@
         <v/>
       </c>
       <c r="H62" s="17">
-        <f>G62/(COUNTA(Rooms!$A:$A)-1)</f>
+        <f>G62/(COUNTA(Clearances!$A:$A)-1)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Rename DSA Room Tag column to Room Tag
</commit_message>
<xml_diff>
--- a/WPH_Room_Register.xlsx
+++ b/WPH_Room_Register.xlsx
@@ -691,7 +691,7 @@
     <row r="23" ht="15" customHeight="1" s="11">
       <c r="A23" s="13" t="inlineStr">
         <is>
-          <t>The DSA room tag from the drawings (e.g. AL02G03) is kept in the column "DSA Room Tag" for cross-reference.</t>
+          <t>The room tag from the DSA typology drawings (e.g. AL02G03) is kept in the column "Room Tag" for cross-reference.</t>
         </is>
       </c>
     </row>
@@ -790,7 +790,7 @@
       </c>
       <c r="D1" s="15" t="inlineStr">
         <is>
-          <t>DSA Room Tag</t>
+          <t>Room Tag</t>
         </is>
       </c>
       <c r="E1" s="15" t="inlineStr">
@@ -38549,12 +38549,12 @@
     <row r="32" ht="15" customHeight="1" s="11">
       <c r="A32" s="10" t="inlineStr">
         <is>
-          <t>DSA Room Tag</t>
+          <t>Room Tag</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>DSA room tag (drawing)</t>
+          <t>Room tag</t>
         </is>
       </c>
       <c r="C32" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Add coordination sketch: light green when sketch provided, dark green for official approval
</commit_message>
<xml_diff>
--- a/WPH_Room_Register.xlsx
+++ b/WPH_Room_Register.xlsx
@@ -24,9 +24,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="dd\-mmm\-yyyy"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="dd-mmm-yyyy"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -148,7 +149,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -229,6 +230,13 @@
       <alignment horizontal="general" vertical="bottom"/>
       <protection locked="0" hidden="0"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -238,7 +246,7 @@
     <cellStyle name="Currency [0]" xfId="4" builtinId="7"/>
     <cellStyle name="Percent" xfId="5" builtinId="5"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="9">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -296,6 +304,13 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00BFECCB"/>
         </patternFill>
       </fill>
     </dxf>
@@ -544,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A31"/>
+  <dimension ref="A1:A34"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="130" customWidth="1" style="10" min="1" max="1"/>
@@ -726,7 +741,6 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
     <row r="30">
       <c r="A30" s="20" t="inlineStr">
         <is>
@@ -738,6 +752,20 @@
       <c r="A31" s="21" t="inlineStr">
         <is>
           <t>Fixed information is locked. Cells you can update are shaded light yellow: Clearances (clearances, dates, remarks), Shop Drawings (drawing ref, revision, statuses, dates), Config (data last updated, updated by). Spare columns to the right of Clearances/Shop Drawings and spare rows below Fields/Lists are open for adding new information. Filtering and sorting are allowed on Clearances and Shop Drawings. To change locked cells: Review &gt; Unprotect Sheet (password held by the Technical Department).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="20" t="inlineStr">
+        <is>
+          <t>COORDINATION SKETCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="21" t="inlineStr">
+        <is>
+          <t>Shop Drawings sheet, columns R-S: set "Provided" (with date) when the MEP/ELV-ID coordination sketch for that room type is issued. While the official MEP/ELV shop drawing is not yet approved, the sketch is treated as mitigating it: the QR page shows that item in LIGHT GREEN ("Sketch provided"). Once the official shop drawing is A/B approved it shows in DARK GREEN ("Approved"), regardless of the sketch.</t>
         </is>
       </c>
     </row>
@@ -34656,6 +34684,8 @@
     <col width="24" customWidth="1" style="10" min="5" max="5"/>
     <col width="14" customWidth="1" style="10" min="6" max="6"/>
     <col width="17" customWidth="1" style="10" min="7" max="17"/>
+    <col width="20" customWidth="1" style="11" min="18" max="18"/>
+    <col width="20" customWidth="1" style="11" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="33.75" customHeight="1" s="11">
@@ -34744,8 +34774,16 @@
           <t>ELV SD - ICT GRMS Lighting Control</t>
         </is>
       </c>
-      <c r="R1" s="22" t="n"/>
-      <c r="S1" s="22" t="n"/>
+      <c r="R1" s="15" t="inlineStr">
+        <is>
+          <t>Coordination Sketch</t>
+        </is>
+      </c>
+      <c r="S1" s="15" t="inlineStr">
+        <is>
+          <t>Coordination Sketch Date</t>
+        </is>
+      </c>
       <c r="T1" s="22" t="n"/>
       <c r="U1" s="22" t="n"/>
       <c r="V1" s="22" t="n"/>
@@ -34790,8 +34828,8 @@
       <c r="O2" s="23" t="n"/>
       <c r="P2" s="23" t="n"/>
       <c r="Q2" s="23" t="n"/>
-      <c r="R2" s="22" t="n"/>
-      <c r="S2" s="22" t="n"/>
+      <c r="R2" s="23" t="n"/>
+      <c r="S2" s="27" t="n"/>
       <c r="T2" s="22" t="n"/>
       <c r="U2" s="22" t="n"/>
       <c r="V2" s="22" t="n"/>
@@ -34836,8 +34874,8 @@
       <c r="O3" s="23" t="n"/>
       <c r="P3" s="23" t="n"/>
       <c r="Q3" s="23" t="n"/>
-      <c r="R3" s="22" t="n"/>
-      <c r="S3" s="22" t="n"/>
+      <c r="R3" s="23" t="n"/>
+      <c r="S3" s="27" t="n"/>
       <c r="T3" s="22" t="n"/>
       <c r="U3" s="22" t="n"/>
       <c r="V3" s="22" t="n"/>
@@ -34932,8 +34970,8 @@
           <t>A - Approved</t>
         </is>
       </c>
-      <c r="R4" s="22" t="n"/>
-      <c r="S4" s="22" t="n"/>
+      <c r="R4" s="23" t="n"/>
+      <c r="S4" s="27" t="n"/>
       <c r="T4" s="22" t="n"/>
       <c r="U4" s="22" t="n"/>
       <c r="V4" s="22" t="n"/>
@@ -34978,8 +35016,8 @@
       <c r="O5" s="23" t="n"/>
       <c r="P5" s="23" t="n"/>
       <c r="Q5" s="23" t="n"/>
-      <c r="R5" s="22" t="n"/>
-      <c r="S5" s="22" t="n"/>
+      <c r="R5" s="23" t="n"/>
+      <c r="S5" s="27" t="n"/>
       <c r="T5" s="22" t="n"/>
       <c r="U5" s="22" t="n"/>
       <c r="V5" s="22" t="n"/>
@@ -35024,8 +35062,8 @@
       <c r="O6" s="23" t="n"/>
       <c r="P6" s="23" t="n"/>
       <c r="Q6" s="23" t="n"/>
-      <c r="R6" s="22" t="n"/>
-      <c r="S6" s="22" t="n"/>
+      <c r="R6" s="23" t="n"/>
+      <c r="S6" s="27" t="n"/>
       <c r="T6" s="22" t="n"/>
       <c r="U6" s="22" t="n"/>
       <c r="V6" s="22" t="n"/>
@@ -35070,8 +35108,8 @@
       <c r="O7" s="23" t="n"/>
       <c r="P7" s="23" t="n"/>
       <c r="Q7" s="23" t="n"/>
-      <c r="R7" s="22" t="n"/>
-      <c r="S7" s="22" t="n"/>
+      <c r="R7" s="23" t="n"/>
+      <c r="S7" s="27" t="n"/>
       <c r="T7" s="22" t="n"/>
       <c r="U7" s="22" t="n"/>
       <c r="V7" s="22" t="n"/>
@@ -35116,8 +35154,8 @@
       <c r="O8" s="23" t="n"/>
       <c r="P8" s="23" t="n"/>
       <c r="Q8" s="23" t="n"/>
-      <c r="R8" s="22" t="n"/>
-      <c r="S8" s="22" t="n"/>
+      <c r="R8" s="23" t="n"/>
+      <c r="S8" s="27" t="n"/>
       <c r="T8" s="22" t="n"/>
       <c r="U8" s="22" t="n"/>
       <c r="V8" s="22" t="n"/>
@@ -35162,8 +35200,8 @@
       <c r="O9" s="23" t="n"/>
       <c r="P9" s="23" t="n"/>
       <c r="Q9" s="23" t="n"/>
-      <c r="R9" s="22" t="n"/>
-      <c r="S9" s="22" t="n"/>
+      <c r="R9" s="23" t="n"/>
+      <c r="S9" s="27" t="n"/>
       <c r="T9" s="22" t="n"/>
       <c r="U9" s="22" t="n"/>
       <c r="V9" s="22" t="n"/>
@@ -35208,8 +35246,8 @@
       <c r="O10" s="23" t="n"/>
       <c r="P10" s="23" t="n"/>
       <c r="Q10" s="23" t="n"/>
-      <c r="R10" s="22" t="n"/>
-      <c r="S10" s="22" t="n"/>
+      <c r="R10" s="23" t="n"/>
+      <c r="S10" s="27" t="n"/>
       <c r="T10" s="22" t="n"/>
       <c r="U10" s="22" t="n"/>
       <c r="V10" s="22" t="n"/>
@@ -35254,8 +35292,8 @@
       <c r="O11" s="23" t="n"/>
       <c r="P11" s="23" t="n"/>
       <c r="Q11" s="23" t="n"/>
-      <c r="R11" s="22" t="n"/>
-      <c r="S11" s="22" t="n"/>
+      <c r="R11" s="23" t="n"/>
+      <c r="S11" s="27" t="n"/>
       <c r="T11" s="22" t="n"/>
       <c r="U11" s="22" t="n"/>
       <c r="V11" s="22" t="n"/>
@@ -35300,8 +35338,8 @@
       <c r="O12" s="23" t="n"/>
       <c r="P12" s="23" t="n"/>
       <c r="Q12" s="23" t="n"/>
-      <c r="R12" s="22" t="n"/>
-      <c r="S12" s="22" t="n"/>
+      <c r="R12" s="23" t="n"/>
+      <c r="S12" s="27" t="n"/>
       <c r="T12" s="22" t="n"/>
       <c r="U12" s="22" t="n"/>
       <c r="V12" s="22" t="n"/>
@@ -35346,8 +35384,8 @@
       <c r="O13" s="23" t="n"/>
       <c r="P13" s="23" t="n"/>
       <c r="Q13" s="23" t="n"/>
-      <c r="R13" s="22" t="n"/>
-      <c r="S13" s="22" t="n"/>
+      <c r="R13" s="23" t="n"/>
+      <c r="S13" s="27" t="n"/>
       <c r="T13" s="22" t="n"/>
       <c r="U13" s="22" t="n"/>
       <c r="V13" s="22" t="n"/>
@@ -35392,8 +35430,8 @@
       <c r="O14" s="23" t="n"/>
       <c r="P14" s="23" t="n"/>
       <c r="Q14" s="23" t="n"/>
-      <c r="R14" s="22" t="n"/>
-      <c r="S14" s="22" t="n"/>
+      <c r="R14" s="23" t="n"/>
+      <c r="S14" s="27" t="n"/>
       <c r="T14" s="22" t="n"/>
       <c r="U14" s="22" t="n"/>
       <c r="V14" s="22" t="n"/>
@@ -35438,8 +35476,8 @@
       <c r="O15" s="23" t="n"/>
       <c r="P15" s="23" t="n"/>
       <c r="Q15" s="23" t="n"/>
-      <c r="R15" s="22" t="n"/>
-      <c r="S15" s="22" t="n"/>
+      <c r="R15" s="23" t="n"/>
+      <c r="S15" s="27" t="n"/>
       <c r="T15" s="22" t="n"/>
       <c r="U15" s="22" t="n"/>
       <c r="V15" s="22" t="n"/>
@@ -35484,8 +35522,8 @@
       <c r="O16" s="23" t="n"/>
       <c r="P16" s="23" t="n"/>
       <c r="Q16" s="23" t="n"/>
-      <c r="R16" s="22" t="n"/>
-      <c r="S16" s="22" t="n"/>
+      <c r="R16" s="23" t="n"/>
+      <c r="S16" s="27" t="n"/>
       <c r="T16" s="22" t="n"/>
       <c r="U16" s="22" t="n"/>
       <c r="V16" s="22" t="n"/>
@@ -35530,8 +35568,8 @@
       <c r="O17" s="23" t="n"/>
       <c r="P17" s="23" t="n"/>
       <c r="Q17" s="23" t="n"/>
-      <c r="R17" s="22" t="n"/>
-      <c r="S17" s="22" t="n"/>
+      <c r="R17" s="23" t="n"/>
+      <c r="S17" s="27" t="n"/>
       <c r="T17" s="22" t="n"/>
       <c r="U17" s="22" t="n"/>
       <c r="V17" s="22" t="n"/>
@@ -35576,8 +35614,8 @@
       <c r="O18" s="23" t="n"/>
       <c r="P18" s="23" t="n"/>
       <c r="Q18" s="23" t="n"/>
-      <c r="R18" s="22" t="n"/>
-      <c r="S18" s="22" t="n"/>
+      <c r="R18" s="23" t="n"/>
+      <c r="S18" s="27" t="n"/>
       <c r="T18" s="22" t="n"/>
       <c r="U18" s="22" t="n"/>
       <c r="V18" s="22" t="n"/>
@@ -35622,8 +35660,8 @@
       <c r="O19" s="23" t="n"/>
       <c r="P19" s="23" t="n"/>
       <c r="Q19" s="23" t="n"/>
-      <c r="R19" s="22" t="n"/>
-      <c r="S19" s="22" t="n"/>
+      <c r="R19" s="23" t="n"/>
+      <c r="S19" s="27" t="n"/>
       <c r="T19" s="22" t="n"/>
       <c r="U19" s="22" t="n"/>
       <c r="V19" s="22" t="n"/>
@@ -35668,8 +35706,8 @@
       <c r="O20" s="23" t="n"/>
       <c r="P20" s="23" t="n"/>
       <c r="Q20" s="23" t="n"/>
-      <c r="R20" s="22" t="n"/>
-      <c r="S20" s="22" t="n"/>
+      <c r="R20" s="23" t="n"/>
+      <c r="S20" s="27" t="n"/>
       <c r="T20" s="22" t="n"/>
       <c r="U20" s="22" t="n"/>
       <c r="V20" s="22" t="n"/>
@@ -35714,8 +35752,8 @@
       <c r="O21" s="23" t="n"/>
       <c r="P21" s="23" t="n"/>
       <c r="Q21" s="23" t="n"/>
-      <c r="R21" s="22" t="n"/>
-      <c r="S21" s="22" t="n"/>
+      <c r="R21" s="23" t="n"/>
+      <c r="S21" s="27" t="n"/>
       <c r="T21" s="22" t="n"/>
       <c r="U21" s="22" t="n"/>
       <c r="V21" s="22" t="n"/>
@@ -35760,8 +35798,8 @@
       <c r="O22" s="23" t="n"/>
       <c r="P22" s="23" t="n"/>
       <c r="Q22" s="23" t="n"/>
-      <c r="R22" s="22" t="n"/>
-      <c r="S22" s="22" t="n"/>
+      <c r="R22" s="23" t="n"/>
+      <c r="S22" s="27" t="n"/>
       <c r="T22" s="22" t="n"/>
       <c r="U22" s="22" t="n"/>
       <c r="V22" s="22" t="n"/>
@@ -35806,8 +35844,8 @@
       <c r="O23" s="23" t="n"/>
       <c r="P23" s="23" t="n"/>
       <c r="Q23" s="23" t="n"/>
-      <c r="R23" s="22" t="n"/>
-      <c r="S23" s="22" t="n"/>
+      <c r="R23" s="23" t="n"/>
+      <c r="S23" s="27" t="n"/>
       <c r="T23" s="22" t="n"/>
       <c r="U23" s="22" t="n"/>
       <c r="V23" s="22" t="n"/>
@@ -35852,8 +35890,8 @@
       <c r="O24" s="23" t="n"/>
       <c r="P24" s="23" t="n"/>
       <c r="Q24" s="23" t="n"/>
-      <c r="R24" s="22" t="n"/>
-      <c r="S24" s="22" t="n"/>
+      <c r="R24" s="23" t="n"/>
+      <c r="S24" s="27" t="n"/>
       <c r="T24" s="22" t="n"/>
       <c r="U24" s="22" t="n"/>
       <c r="V24" s="22" t="n"/>
@@ -35898,8 +35936,8 @@
       <c r="O25" s="23" t="n"/>
       <c r="P25" s="23" t="n"/>
       <c r="Q25" s="23" t="n"/>
-      <c r="R25" s="22" t="n"/>
-      <c r="S25" s="22" t="n"/>
+      <c r="R25" s="23" t="n"/>
+      <c r="S25" s="27" t="n"/>
       <c r="T25" s="22" t="n"/>
       <c r="U25" s="22" t="n"/>
       <c r="V25" s="22" t="n"/>
@@ -35944,8 +35982,8 @@
       <c r="O26" s="23" t="n"/>
       <c r="P26" s="23" t="n"/>
       <c r="Q26" s="23" t="n"/>
-      <c r="R26" s="22" t="n"/>
-      <c r="S26" s="22" t="n"/>
+      <c r="R26" s="23" t="n"/>
+      <c r="S26" s="27" t="n"/>
       <c r="T26" s="22" t="n"/>
       <c r="U26" s="22" t="n"/>
       <c r="V26" s="22" t="n"/>
@@ -35990,8 +36028,8 @@
       <c r="O27" s="23" t="n"/>
       <c r="P27" s="23" t="n"/>
       <c r="Q27" s="23" t="n"/>
-      <c r="R27" s="22" t="n"/>
-      <c r="S27" s="22" t="n"/>
+      <c r="R27" s="23" t="n"/>
+      <c r="S27" s="27" t="n"/>
       <c r="T27" s="22" t="n"/>
       <c r="U27" s="22" t="n"/>
       <c r="V27" s="22" t="n"/>
@@ -36036,8 +36074,8 @@
       <c r="O28" s="23" t="n"/>
       <c r="P28" s="23" t="n"/>
       <c r="Q28" s="23" t="n"/>
-      <c r="R28" s="22" t="n"/>
-      <c r="S28" s="22" t="n"/>
+      <c r="R28" s="23" t="n"/>
+      <c r="S28" s="27" t="n"/>
       <c r="T28" s="22" t="n"/>
       <c r="U28" s="22" t="n"/>
       <c r="V28" s="22" t="n"/>
@@ -36082,8 +36120,8 @@
       <c r="O29" s="23" t="n"/>
       <c r="P29" s="23" t="n"/>
       <c r="Q29" s="23" t="n"/>
-      <c r="R29" s="22" t="n"/>
-      <c r="S29" s="22" t="n"/>
+      <c r="R29" s="23" t="n"/>
+      <c r="S29" s="27" t="n"/>
       <c r="T29" s="22" t="n"/>
       <c r="U29" s="22" t="n"/>
       <c r="V29" s="22" t="n"/>
@@ -36128,8 +36166,8 @@
       <c r="O30" s="23" t="n"/>
       <c r="P30" s="23" t="n"/>
       <c r="Q30" s="23" t="n"/>
-      <c r="R30" s="22" t="n"/>
-      <c r="S30" s="22" t="n"/>
+      <c r="R30" s="23" t="n"/>
+      <c r="S30" s="27" t="n"/>
       <c r="T30" s="22" t="n"/>
       <c r="U30" s="22" t="n"/>
       <c r="V30" s="22" t="n"/>
@@ -36174,8 +36212,8 @@
       <c r="O31" s="23" t="n"/>
       <c r="P31" s="23" t="n"/>
       <c r="Q31" s="23" t="n"/>
-      <c r="R31" s="22" t="n"/>
-      <c r="S31" s="22" t="n"/>
+      <c r="R31" s="23" t="n"/>
+      <c r="S31" s="27" t="n"/>
       <c r="T31" s="22" t="n"/>
       <c r="U31" s="22" t="n"/>
       <c r="V31" s="22" t="n"/>
@@ -36220,8 +36258,8 @@
       <c r="O32" s="23" t="n"/>
       <c r="P32" s="23" t="n"/>
       <c r="Q32" s="23" t="n"/>
-      <c r="R32" s="22" t="n"/>
-      <c r="S32" s="22" t="n"/>
+      <c r="R32" s="23" t="n"/>
+      <c r="S32" s="27" t="n"/>
       <c r="T32" s="22" t="n"/>
       <c r="U32" s="22" t="n"/>
       <c r="V32" s="22" t="n"/>
@@ -36266,8 +36304,8 @@
       <c r="O33" s="23" t="n"/>
       <c r="P33" s="23" t="n"/>
       <c r="Q33" s="23" t="n"/>
-      <c r="R33" s="22" t="n"/>
-      <c r="S33" s="22" t="n"/>
+      <c r="R33" s="23" t="n"/>
+      <c r="S33" s="27" t="n"/>
       <c r="T33" s="22" t="n"/>
       <c r="U33" s="22" t="n"/>
       <c r="V33" s="22" t="n"/>
@@ -36312,8 +36350,8 @@
       <c r="O34" s="23" t="n"/>
       <c r="P34" s="23" t="n"/>
       <c r="Q34" s="23" t="n"/>
-      <c r="R34" s="22" t="n"/>
-      <c r="S34" s="22" t="n"/>
+      <c r="R34" s="23" t="n"/>
+      <c r="S34" s="27" t="n"/>
       <c r="T34" s="22" t="n"/>
       <c r="U34" s="22" t="n"/>
       <c r="V34" s="22" t="n"/>
@@ -36358,8 +36396,8 @@
       <c r="O35" s="23" t="n"/>
       <c r="P35" s="23" t="n"/>
       <c r="Q35" s="23" t="n"/>
-      <c r="R35" s="22" t="n"/>
-      <c r="S35" s="22" t="n"/>
+      <c r="R35" s="23" t="n"/>
+      <c r="S35" s="27" t="n"/>
       <c r="T35" s="22" t="n"/>
       <c r="U35" s="22" t="n"/>
       <c r="V35" s="22" t="n"/>
@@ -36404,8 +36442,8 @@
       <c r="O36" s="23" t="n"/>
       <c r="P36" s="23" t="n"/>
       <c r="Q36" s="23" t="n"/>
-      <c r="R36" s="22" t="n"/>
-      <c r="S36" s="22" t="n"/>
+      <c r="R36" s="23" t="n"/>
+      <c r="S36" s="27" t="n"/>
       <c r="T36" s="22" t="n"/>
       <c r="U36" s="22" t="n"/>
       <c r="V36" s="22" t="n"/>
@@ -36450,8 +36488,8 @@
       <c r="O37" s="23" t="n"/>
       <c r="P37" s="23" t="n"/>
       <c r="Q37" s="23" t="n"/>
-      <c r="R37" s="22" t="n"/>
-      <c r="S37" s="22" t="n"/>
+      <c r="R37" s="23" t="n"/>
+      <c r="S37" s="27" t="n"/>
       <c r="T37" s="22" t="n"/>
       <c r="U37" s="22" t="n"/>
       <c r="V37" s="22" t="n"/>
@@ -36496,8 +36534,8 @@
       <c r="O38" s="23" t="n"/>
       <c r="P38" s="23" t="n"/>
       <c r="Q38" s="23" t="n"/>
-      <c r="R38" s="22" t="n"/>
-      <c r="S38" s="22" t="n"/>
+      <c r="R38" s="23" t="n"/>
+      <c r="S38" s="27" t="n"/>
       <c r="T38" s="22" t="n"/>
       <c r="U38" s="22" t="n"/>
       <c r="V38" s="22" t="n"/>
@@ -36542,8 +36580,8 @@
       <c r="O39" s="23" t="n"/>
       <c r="P39" s="23" t="n"/>
       <c r="Q39" s="23" t="n"/>
-      <c r="R39" s="22" t="n"/>
-      <c r="S39" s="22" t="n"/>
+      <c r="R39" s="23" t="n"/>
+      <c r="S39" s="27" t="n"/>
       <c r="T39" s="22" t="n"/>
       <c r="U39" s="22" t="n"/>
       <c r="V39" s="22" t="n"/>
@@ -36588,8 +36626,8 @@
       <c r="O40" s="23" t="n"/>
       <c r="P40" s="23" t="n"/>
       <c r="Q40" s="23" t="n"/>
-      <c r="R40" s="22" t="n"/>
-      <c r="S40" s="22" t="n"/>
+      <c r="R40" s="23" t="n"/>
+      <c r="S40" s="27" t="n"/>
       <c r="T40" s="22" t="n"/>
       <c r="U40" s="22" t="n"/>
       <c r="V40" s="22" t="n"/>
@@ -36634,8 +36672,8 @@
       <c r="O41" s="23" t="n"/>
       <c r="P41" s="23" t="n"/>
       <c r="Q41" s="23" t="n"/>
-      <c r="R41" s="22" t="n"/>
-      <c r="S41" s="22" t="n"/>
+      <c r="R41" s="23" t="n"/>
+      <c r="S41" s="27" t="n"/>
       <c r="T41" s="22" t="n"/>
       <c r="U41" s="22" t="n"/>
       <c r="V41" s="22" t="n"/>
@@ -36680,8 +36718,8 @@
       <c r="O42" s="23" t="n"/>
       <c r="P42" s="23" t="n"/>
       <c r="Q42" s="23" t="n"/>
-      <c r="R42" s="22" t="n"/>
-      <c r="S42" s="22" t="n"/>
+      <c r="R42" s="23" t="n"/>
+      <c r="S42" s="27" t="n"/>
       <c r="T42" s="22" t="n"/>
       <c r="U42" s="22" t="n"/>
       <c r="V42" s="22" t="n"/>
@@ -36726,8 +36764,8 @@
       <c r="O43" s="23" t="n"/>
       <c r="P43" s="23" t="n"/>
       <c r="Q43" s="23" t="n"/>
-      <c r="R43" s="22" t="n"/>
-      <c r="S43" s="22" t="n"/>
+      <c r="R43" s="23" t="n"/>
+      <c r="S43" s="27" t="n"/>
       <c r="T43" s="22" t="n"/>
       <c r="U43" s="22" t="n"/>
       <c r="V43" s="22" t="n"/>
@@ -36772,8 +36810,8 @@
       <c r="O44" s="23" t="n"/>
       <c r="P44" s="23" t="n"/>
       <c r="Q44" s="23" t="n"/>
-      <c r="R44" s="22" t="n"/>
-      <c r="S44" s="22" t="n"/>
+      <c r="R44" s="23" t="n"/>
+      <c r="S44" s="27" t="n"/>
       <c r="T44" s="22" t="n"/>
       <c r="U44" s="22" t="n"/>
       <c r="V44" s="22" t="n"/>
@@ -36818,8 +36856,8 @@
       <c r="O45" s="23" t="n"/>
       <c r="P45" s="23" t="n"/>
       <c r="Q45" s="23" t="n"/>
-      <c r="R45" s="22" t="n"/>
-      <c r="S45" s="22" t="n"/>
+      <c r="R45" s="23" t="n"/>
+      <c r="S45" s="27" t="n"/>
       <c r="T45" s="22" t="n"/>
       <c r="U45" s="22" t="n"/>
       <c r="V45" s="22" t="n"/>
@@ -36864,8 +36902,8 @@
       <c r="O46" s="23" t="n"/>
       <c r="P46" s="23" t="n"/>
       <c r="Q46" s="23" t="n"/>
-      <c r="R46" s="22" t="n"/>
-      <c r="S46" s="22" t="n"/>
+      <c r="R46" s="23" t="n"/>
+      <c r="S46" s="27" t="n"/>
       <c r="T46" s="22" t="n"/>
       <c r="U46" s="22" t="n"/>
       <c r="V46" s="22" t="n"/>
@@ -36910,8 +36948,8 @@
       <c r="O47" s="23" t="n"/>
       <c r="P47" s="23" t="n"/>
       <c r="Q47" s="23" t="n"/>
-      <c r="R47" s="22" t="n"/>
-      <c r="S47" s="22" t="n"/>
+      <c r="R47" s="23" t="n"/>
+      <c r="S47" s="27" t="n"/>
       <c r="T47" s="22" t="n"/>
       <c r="U47" s="22" t="n"/>
       <c r="V47" s="22" t="n"/>
@@ -36956,8 +36994,8 @@
       <c r="O48" s="23" t="n"/>
       <c r="P48" s="23" t="n"/>
       <c r="Q48" s="23" t="n"/>
-      <c r="R48" s="22" t="n"/>
-      <c r="S48" s="22" t="n"/>
+      <c r="R48" s="23" t="n"/>
+      <c r="S48" s="27" t="n"/>
       <c r="T48" s="22" t="n"/>
       <c r="U48" s="22" t="n"/>
       <c r="V48" s="22" t="n"/>
@@ -37002,8 +37040,8 @@
       <c r="O49" s="23" t="n"/>
       <c r="P49" s="23" t="n"/>
       <c r="Q49" s="23" t="n"/>
-      <c r="R49" s="22" t="n"/>
-      <c r="S49" s="22" t="n"/>
+      <c r="R49" s="23" t="n"/>
+      <c r="S49" s="27" t="n"/>
       <c r="T49" s="22" t="n"/>
       <c r="U49" s="22" t="n"/>
       <c r="V49" s="22" t="n"/>
@@ -37048,8 +37086,8 @@
       <c r="O50" s="23" t="n"/>
       <c r="P50" s="23" t="n"/>
       <c r="Q50" s="23" t="n"/>
-      <c r="R50" s="22" t="n"/>
-      <c r="S50" s="22" t="n"/>
+      <c r="R50" s="23" t="n"/>
+      <c r="S50" s="27" t="n"/>
       <c r="T50" s="22" t="n"/>
       <c r="U50" s="22" t="n"/>
       <c r="V50" s="22" t="n"/>
@@ -37094,8 +37132,8 @@
       <c r="O51" s="23" t="n"/>
       <c r="P51" s="23" t="n"/>
       <c r="Q51" s="23" t="n"/>
-      <c r="R51" s="22" t="n"/>
-      <c r="S51" s="22" t="n"/>
+      <c r="R51" s="23" t="n"/>
+      <c r="S51" s="27" t="n"/>
       <c r="T51" s="22" t="n"/>
       <c r="U51" s="22" t="n"/>
       <c r="V51" s="22" t="n"/>
@@ -37140,8 +37178,8 @@
       <c r="O52" s="23" t="n"/>
       <c r="P52" s="23" t="n"/>
       <c r="Q52" s="23" t="n"/>
-      <c r="R52" s="22" t="n"/>
-      <c r="S52" s="22" t="n"/>
+      <c r="R52" s="23" t="n"/>
+      <c r="S52" s="27" t="n"/>
       <c r="T52" s="22" t="n"/>
       <c r="U52" s="22" t="n"/>
       <c r="V52" s="22" t="n"/>
@@ -37186,8 +37224,8 @@
       <c r="O53" s="23" t="n"/>
       <c r="P53" s="23" t="n"/>
       <c r="Q53" s="23" t="n"/>
-      <c r="R53" s="22" t="n"/>
-      <c r="S53" s="22" t="n"/>
+      <c r="R53" s="23" t="n"/>
+      <c r="S53" s="27" t="n"/>
       <c r="T53" s="22" t="n"/>
       <c r="U53" s="22" t="n"/>
       <c r="V53" s="22" t="n"/>
@@ -37232,8 +37270,8 @@
       <c r="O54" s="23" t="n"/>
       <c r="P54" s="23" t="n"/>
       <c r="Q54" s="23" t="n"/>
-      <c r="R54" s="22" t="n"/>
-      <c r="S54" s="22" t="n"/>
+      <c r="R54" s="23" t="n"/>
+      <c r="S54" s="27" t="n"/>
       <c r="T54" s="22" t="n"/>
       <c r="U54" s="22" t="n"/>
       <c r="V54" s="22" t="n"/>
@@ -37278,8 +37316,8 @@
       <c r="O55" s="23" t="n"/>
       <c r="P55" s="23" t="n"/>
       <c r="Q55" s="23" t="n"/>
-      <c r="R55" s="22" t="n"/>
-      <c r="S55" s="22" t="n"/>
+      <c r="R55" s="23" t="n"/>
+      <c r="S55" s="27" t="n"/>
       <c r="T55" s="22" t="n"/>
       <c r="U55" s="22" t="n"/>
       <c r="V55" s="22" t="n"/>
@@ -37324,8 +37362,8 @@
       <c r="O56" s="23" t="n"/>
       <c r="P56" s="23" t="n"/>
       <c r="Q56" s="23" t="n"/>
-      <c r="R56" s="22" t="n"/>
-      <c r="S56" s="22" t="n"/>
+      <c r="R56" s="23" t="n"/>
+      <c r="S56" s="27" t="n"/>
       <c r="T56" s="22" t="n"/>
       <c r="U56" s="22" t="n"/>
       <c r="V56" s="22" t="n"/>
@@ -37370,8 +37408,8 @@
       <c r="O57" s="23" t="n"/>
       <c r="P57" s="23" t="n"/>
       <c r="Q57" s="23" t="n"/>
-      <c r="R57" s="22" t="n"/>
-      <c r="S57" s="22" t="n"/>
+      <c r="R57" s="23" t="n"/>
+      <c r="S57" s="27" t="n"/>
       <c r="T57" s="22" t="n"/>
       <c r="U57" s="22" t="n"/>
       <c r="V57" s="22" t="n"/>
@@ -37416,8 +37454,8 @@
       <c r="O58" s="23" t="n"/>
       <c r="P58" s="23" t="n"/>
       <c r="Q58" s="23" t="n"/>
-      <c r="R58" s="22" t="n"/>
-      <c r="S58" s="22" t="n"/>
+      <c r="R58" s="23" t="n"/>
+      <c r="S58" s="27" t="n"/>
       <c r="T58" s="22" t="n"/>
       <c r="U58" s="22" t="n"/>
       <c r="V58" s="22" t="n"/>
@@ -37462,8 +37500,8 @@
       <c r="O59" s="23" t="n"/>
       <c r="P59" s="23" t="n"/>
       <c r="Q59" s="23" t="n"/>
-      <c r="R59" s="22" t="n"/>
-      <c r="S59" s="22" t="n"/>
+      <c r="R59" s="23" t="n"/>
+      <c r="S59" s="27" t="n"/>
       <c r="T59" s="22" t="n"/>
       <c r="U59" s="22" t="n"/>
       <c r="V59" s="22" t="n"/>
@@ -37508,8 +37546,8 @@
       <c r="O60" s="23" t="n"/>
       <c r="P60" s="23" t="n"/>
       <c r="Q60" s="23" t="n"/>
-      <c r="R60" s="22" t="n"/>
-      <c r="S60" s="22" t="n"/>
+      <c r="R60" s="23" t="n"/>
+      <c r="S60" s="27" t="n"/>
       <c r="T60" s="22" t="n"/>
       <c r="U60" s="22" t="n"/>
       <c r="V60" s="22" t="n"/>
@@ -37554,8 +37592,8 @@
       <c r="O61" s="23" t="n"/>
       <c r="P61" s="23" t="n"/>
       <c r="Q61" s="23" t="n"/>
-      <c r="R61" s="22" t="n"/>
-      <c r="S61" s="22" t="n"/>
+      <c r="R61" s="23" t="n"/>
+      <c r="S61" s="27" t="n"/>
       <c r="T61" s="22" t="n"/>
       <c r="U61" s="22" t="n"/>
       <c r="V61" s="22" t="n"/>
@@ -37600,8 +37638,8 @@
       <c r="O62" s="23" t="n"/>
       <c r="P62" s="23" t="n"/>
       <c r="Q62" s="23" t="n"/>
-      <c r="R62" s="22" t="n"/>
-      <c r="S62" s="22" t="n"/>
+      <c r="R62" s="23" t="n"/>
+      <c r="S62" s="27" t="n"/>
       <c r="T62" s="22" t="n"/>
       <c r="U62" s="22" t="n"/>
       <c r="V62" s="22" t="n"/>
@@ -37632,7 +37670,12 @@
       <formula>LEFT(E2,3)="D -"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
+  <conditionalFormatting sqref="R2:R62">
+    <cfRule type="expression" priority="5" dxfId="8">
+      <formula>R2="Provided"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="4">
     <dataValidation sqref="E2:E62 G2:Q62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>Lists!$A$2:$A$30</formula1>
       <formula2>0</formula2>
@@ -37641,6 +37684,10 @@
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
+    <dataValidation sqref="R2:R62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Provided,Not Provided"</formula1>
+    </dataValidation>
+    <dataValidation sqref="S2:S62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date"/>
   </dataValidations>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -37654,7 +37701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F260"/>
+  <dimension ref="A1:F262"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="10" min="1" max="1"/>
@@ -38597,12 +38644,64 @@
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="11">
-      <c r="E34" s="10" t="n"/>
-      <c r="F34" s="10" t="n"/>
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t>Coordination Sketch</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="inlineStr">
+        <is>
+          <t>Coordination sketch (MEP/ELV with ID)</t>
+        </is>
+      </c>
+      <c r="C34" s="10" t="inlineStr">
+        <is>
+          <t>Coordination sketch</t>
+        </is>
+      </c>
+      <c r="D34" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="E34" s="10" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F34" s="10" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="11">
-      <c r="E35" s="10" t="n"/>
-      <c r="F35" s="10" t="n"/>
+      <c r="A35" s="10" t="inlineStr">
+        <is>
+          <t>Coordination Sketch Date</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>Sketch date</t>
+        </is>
+      </c>
+      <c r="C35" s="10" t="inlineStr">
+        <is>
+          <t>Coordination sketch</t>
+        </is>
+      </c>
+      <c r="D35" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="E35" s="10" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F35" s="10" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="11">
       <c r="E36" s="10" t="n"/>
@@ -39743,6 +39842,22 @@
       <c r="D260" s="22" t="n"/>
       <c r="E260" s="22" t="n"/>
       <c r="F260" s="22" t="n"/>
+    </row>
+    <row r="261">
+      <c r="A261" s="28" t="n"/>
+      <c r="B261" s="28" t="n"/>
+      <c r="C261" s="28" t="n"/>
+      <c r="D261" s="28" t="n"/>
+      <c r="E261" s="28" t="n"/>
+      <c r="F261" s="28" t="n"/>
+    </row>
+    <row r="262">
+      <c r="A262" s="28" t="n"/>
+      <c r="B262" s="28" t="n"/>
+      <c r="C262" s="28" t="n"/>
+      <c r="D262" s="28" t="n"/>
+      <c r="E262" s="28" t="n"/>
+      <c r="F262" s="28" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="1" password="D6EA"/>

</xml_diff>

<commit_message>
Status codes A/B/UR/C/TBS with colours from Lists; sketch shown as Coordinated
</commit_message>
<xml_diff>
--- a/WPH_Room_Register.xlsx
+++ b/WPH_Room_Register.xlsx
@@ -96,7 +96,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -112,6 +112,31 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF9E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0000B050"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BFBFBF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B6E3A3"/>
       </patternFill>
     </fill>
   </fills>
@@ -149,7 +174,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -237,6 +262,21 @@
       <alignment horizontal="general" vertical="bottom"/>
       <protection locked="0" hidden="0"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -246,7 +286,7 @@
     <cellStyle name="Currency [0]" xfId="4" builtinId="7"/>
     <cellStyle name="Percent" xfId="5" builtinId="5"/>
   </cellStyles>
-  <dxfs count="9">
+  <dxfs count="14">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -311,6 +351,57 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00BFECCB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00FFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="0000B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00000000"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00FFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00000000"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00BFBFBF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00B6E3A3"/>
         </patternFill>
       </fill>
     </dxf>
@@ -559,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A34"/>
+  <dimension ref="A1:A37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="130" customWidth="1" style="10" min="1" max="1"/>
@@ -766,6 +857,20 @@
       <c r="A34" s="21" t="inlineStr">
         <is>
           <t>Shop Drawings sheet, columns R-S: set "Provided" (with date) when the MEP/ELV-ID coordination sketch for that room type is issued. While the official MEP/ELV shop drawing is not yet approved, the sketch is treated as mitigating it: the QR page shows that item in LIGHT GREEN ("Sketch provided"). Once the official shop drawing is A/B approved it shows in DARK GREEN ("Approved"), regardless of the sketch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="20" t="inlineStr">
+        <is>
+          <t>STATUS CODES (Shop Drawings sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="21" t="inlineStr">
+        <is>
+          <t>A / B = Approved / Approved as Noted (dark green)  |  UR = Under Review (amber)  |  C = Revise &amp; Resubmit (red)  |  TBS = To Be Submitted (grey). Codes, colours and meanings are defined in the Lists sheet and are used by both Excel and the QR pages. When the Coordination Sketch is "Provided", every MEP/ELV item that is not A/B is shown as "Coordinated" (light green); A/B approvals always show dark green.</t>
         </is>
       </c>
     </row>
@@ -34909,7 +35014,7 @@
       <c r="D4" s="23" t="n"/>
       <c r="E4" s="25" t="inlineStr">
         <is>
-          <t>A - Approved</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F4" s="24" t="n">
@@ -34917,57 +35022,57 @@
       </c>
       <c r="G4" s="25" t="inlineStr">
         <is>
-          <t>A - Approved</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H4" s="25" t="inlineStr">
         <is>
-          <t>A - Approved</t>
+          <t>A</t>
         </is>
       </c>
       <c r="I4" s="25" t="inlineStr">
         <is>
-          <t>A - Approved</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J4" s="25" t="inlineStr">
         <is>
-          <t>A - Approved</t>
+          <t>A</t>
         </is>
       </c>
       <c r="K4" s="25" t="inlineStr">
         <is>
-          <t>A - Approved</t>
+          <t>A</t>
         </is>
       </c>
       <c r="L4" s="25" t="inlineStr">
         <is>
-          <t>A - Approved</t>
+          <t>A</t>
         </is>
       </c>
       <c r="M4" s="25" t="inlineStr">
         <is>
-          <t>A - Approved</t>
+          <t>A</t>
         </is>
       </c>
       <c r="N4" s="25" t="inlineStr">
         <is>
-          <t>A - Approved</t>
+          <t>A</t>
         </is>
       </c>
       <c r="O4" s="25" t="inlineStr">
         <is>
-          <t>A - Approved</t>
+          <t>A</t>
         </is>
       </c>
       <c r="P4" s="25" t="inlineStr">
         <is>
-          <t>A - Approved</t>
+          <t>A</t>
         </is>
       </c>
       <c r="Q4" s="25" t="inlineStr">
         <is>
-          <t>A - Approved</t>
+          <t>A</t>
         </is>
       </c>
       <c r="R4" s="23" t="n"/>
@@ -37656,28 +37761,31 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="1" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="0" password="D6EA"/>
-  <conditionalFormatting sqref="E2:Q62">
-    <cfRule type="expression" rank="0" priority="2" equalAverage="0" aboveAverage="0" dxfId="5" text="" percent="0" bottom="0">
-      <formula>LEFT(E2,3)="A -"</formula>
+  <conditionalFormatting sqref="E2:E62 G2:Q62">
+    <cfRule type="expression" priority="1" dxfId="9">
+      <formula>UPPER(E2)="A"</formula>
     </cfRule>
-    <cfRule type="expression" rank="0" priority="3" equalAverage="0" aboveAverage="0" dxfId="5" text="" percent="0" bottom="0">
-      <formula>LEFT(E2,3)="B -"</formula>
+    <cfRule type="expression" priority="2" dxfId="9">
+      <formula>UPPER(E2)="B"</formula>
     </cfRule>
-    <cfRule type="expression" rank="0" priority="4" equalAverage="0" aboveAverage="0" dxfId="6" text="" percent="0" bottom="0">
-      <formula>LEFT(E2,3)="C -"</formula>
+    <cfRule type="expression" priority="3" dxfId="10">
+      <formula>UPPER(E2)="UR"</formula>
     </cfRule>
-    <cfRule type="expression" rank="0" priority="5" equalAverage="0" aboveAverage="0" dxfId="7" text="" percent="0" bottom="0">
-      <formula>LEFT(E2,3)="D -"</formula>
+    <cfRule type="expression" priority="4" dxfId="11">
+      <formula>UPPER(E2)="C"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="12">
+      <formula>UPPER(E2)="TBS"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R2:R62">
-    <cfRule type="expression" priority="5" dxfId="8">
+    <cfRule type="expression" priority="6" dxfId="13">
       <formula>R2="Provided"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation sqref="E2:E62 G2:Q62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
-      <formula1>Lists!$A$2:$A$30</formula1>
+    <dataValidation sqref="E2:E62 G2:Q62" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Use A, B, UR, C or TBS" type="list" errorStyle="stop" operator="between">
+      <formula1>Lists!$A$2:$A$6</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation sqref="F2:F62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date" errorStyle="stop" operator="between">
@@ -42172,8 +42280,8 @@
   <cols>
     <col width="30" customWidth="1" style="10" min="1" max="1"/>
     <col width="12" customWidth="1" style="10" min="2" max="2"/>
-    <col width="45" customWidth="1" style="10" min="3" max="3"/>
-    <col width="4" customWidth="1" style="10" min="4" max="4"/>
+    <col width="60" customWidth="1" style="10" min="3" max="3"/>
+    <col width="14" customWidth="1" style="10" min="4" max="4"/>
     <col width="22" customWidth="1" style="10" min="5" max="5"/>
     <col width="12" customWidth="1" style="10" min="6" max="6"/>
   </cols>
@@ -42194,7 +42302,11 @@
           <t>Meaning</t>
         </is>
       </c>
-      <c r="D1" s="15" t="n"/>
+      <c r="D1" s="15" t="inlineStr">
+        <is>
+          <t>Counts as</t>
+        </is>
+      </c>
       <c r="E1" s="15" t="inlineStr">
         <is>
           <t>Clearance</t>
@@ -42209,17 +42321,22 @@
     <row r="2" ht="15" customHeight="1" s="11">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>A - Approved</t>
-        </is>
-      </c>
-      <c r="B2" s="10" t="inlineStr">
-        <is>
-          <t>green</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B2" s="29" t="inlineStr">
+        <is>
+          <t>#00B050</t>
         </is>
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>Code A</t>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="E2" s="10" t="inlineStr">
@@ -42236,17 +42353,22 @@
     <row r="3" ht="15" customHeight="1" s="11">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>B - Approved as Noted</t>
-        </is>
-      </c>
-      <c r="B3" s="10" t="inlineStr">
-        <is>
-          <t>green</t>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B3" s="29" t="inlineStr">
+        <is>
+          <t>#00B050</t>
         </is>
       </c>
       <c r="C3" s="10" t="inlineStr">
         <is>
-          <t>Code B</t>
+          <t>Approved as Noted</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="E3" s="10" t="inlineStr">
@@ -42263,17 +42385,22 @@
     <row r="4" ht="15" customHeight="1" s="11">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>C - Revise &amp; Resubmit</t>
-        </is>
-      </c>
-      <c r="B4" s="10" t="inlineStr">
-        <is>
-          <t>amber</t>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="B4" s="30" t="inlineStr">
+        <is>
+          <t>#FFC000</t>
         </is>
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>Code C</t>
+          <t>Under Review</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>review</t>
         </is>
       </c>
       <c r="E4" s="10" t="inlineStr">
@@ -42290,17 +42417,22 @@
     <row r="5" ht="15" customHeight="1" s="11">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>D - Rejected</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>red</t>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B5" s="31" t="inlineStr">
+        <is>
+          <t>#FF0000</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>Code D</t>
+          <t>Code C - Revise &amp; Resubmit</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>revise</t>
         </is>
       </c>
       <c r="E5" s="10" t="inlineStr">
@@ -42317,17 +42449,22 @@
     <row r="6" ht="15" customHeight="1" s="11">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>Under Review</t>
-        </is>
-      </c>
-      <c r="B6" s="10" t="inlineStr">
-        <is>
-          <t>blue</t>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="B6" s="32" t="inlineStr">
+        <is>
+          <t>#BFBFBF</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>Submitted, awaiting consultant</t>
+          <t>To Be Submitted</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>pending</t>
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr">
@@ -42344,48 +42481,36 @@
     <row r="7" ht="15" customHeight="1" s="11">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>In Preparation</t>
-        </is>
-      </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>grey</t>
+          <t>Coordinated</t>
+        </is>
+      </c>
+      <c r="B7" s="33" t="inlineStr">
+        <is>
+          <t>#B6E3A3</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>Being prepared by BUJV / subcontractor</t>
+          <t>Coordination sketch provided (shown instead of a non-approved MEP/ELV status)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>coordinated</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="11">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>Not Submitted</t>
-        </is>
-      </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>grey</t>
-        </is>
-      </c>
+      <c r="A8" s="28" t="n"/>
+      <c r="B8" s="28" t="n"/>
+      <c r="C8" s="22" t="n"/>
+      <c r="D8" s="22" t="n"/>
     </row>
     <row r="9" ht="15" customHeight="1" s="11">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>grey</t>
-        </is>
-      </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>Not applicable</t>
-        </is>
-      </c>
+      <c r="A9" s="28" t="n"/>
+      <c r="B9" s="28" t="n"/>
+      <c r="C9" s="28" t="n"/>
+      <c r="D9" s="22" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="22" t="n"/>

</xml_diff>

<commit_message>
Exact status colours; Excel rules show Coordinated unless A/B; keep user edits (F03 sketch, F02 TBS)
</commit_message>
<xml_diff>
--- a/WPH_Room_Register.xlsx
+++ b/WPH_Room_Register.xlsx
@@ -96,7 +96,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -139,6 +139,11 @@
         <fgColor rgb="00B6E3A3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B5E6A2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -174,7 +179,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -277,6 +282,9 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -286,7 +294,7 @@
     <cellStyle name="Currency [0]" xfId="4" builtinId="7"/>
     <cellStyle name="Percent" xfId="5" builtinId="5"/>
   </cellStyles>
-  <dxfs count="14">
+  <dxfs count="20">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -402,6 +410,55 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00B6E3A3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="0000B050"/>
+          <bgColor rgb="0000B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC000"/>
+          <bgColor rgb="00FFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FF0000"/>
+          <bgColor rgb="00FF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00BFBFBF"/>
+          <bgColor rgb="00BFBFBF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="200" formatCode="General;General;General;&quot;Coordinated&quot;"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00B5E6A2"/>
+          <bgColor rgb="00B5E6A2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00B5E6A2"/>
+          <bgColor rgb="00B5E6A2"/>
         </patternFill>
       </fill>
     </dxf>
@@ -34978,7 +35035,11 @@
       <c r="N3" s="23" t="n"/>
       <c r="O3" s="23" t="n"/>
       <c r="P3" s="23" t="n"/>
-      <c r="Q3" s="23" t="n"/>
+      <c r="Q3" s="23" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="R3" s="23" t="n"/>
       <c r="S3" s="27" t="n"/>
       <c r="T3" s="22" t="n"/>
@@ -35012,70 +35073,26 @@
         </is>
       </c>
       <c r="D4" s="23" t="n"/>
-      <c r="E4" s="25" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
+      <c r="E4" s="25" t="n"/>
       <c r="F4" s="24" t="n">
         <v>46301</v>
       </c>
-      <c r="G4" s="25" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="H4" s="25" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="I4" s="25" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="J4" s="25" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="K4" s="25" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L4" s="25" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="M4" s="25" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="N4" s="25" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="O4" s="25" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="P4" s="25" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="Q4" s="25" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="R4" s="23" t="n"/>
+      <c r="G4" s="25" t="n"/>
+      <c r="H4" s="25" t="n"/>
+      <c r="I4" s="25" t="n"/>
+      <c r="J4" s="25" t="n"/>
+      <c r="K4" s="25" t="n"/>
+      <c r="L4" s="25" t="n"/>
+      <c r="M4" s="25" t="n"/>
+      <c r="N4" s="25" t="n"/>
+      <c r="O4" s="25" t="n"/>
+      <c r="P4" s="25" t="n"/>
+      <c r="Q4" s="25" t="n"/>
+      <c r="R4" s="23" t="inlineStr">
+        <is>
+          <t>Provided</t>
+        </is>
+      </c>
       <c r="S4" s="27" t="n"/>
       <c r="T4" s="22" t="n"/>
       <c r="U4" s="22" t="n"/>
@@ -37761,26 +37778,46 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="1" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="0" password="D6EA"/>
-  <conditionalFormatting sqref="E2:E62 G2:Q62">
-    <cfRule type="expression" priority="1" dxfId="9">
-      <formula>UPPER(E2)="A"</formula>
+  <conditionalFormatting sqref="E2:E62">
+    <cfRule type="expression" priority="1" dxfId="14" stopIfTrue="1">
+      <formula>TRIM(UPPER(E2))="A"</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="9">
-      <formula>UPPER(E2)="B"</formula>
+    <cfRule type="expression" priority="2" dxfId="14" stopIfTrue="1">
+      <formula>TRIM(UPPER(E2))="B"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" dxfId="10">
-      <formula>UPPER(E2)="UR"</formula>
+    <cfRule type="expression" priority="3" dxfId="15" stopIfTrue="1">
+      <formula>TRIM(UPPER(E2))="UR"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" dxfId="11">
-      <formula>UPPER(E2)="C"</formula>
+    <cfRule type="expression" priority="4" dxfId="16" stopIfTrue="1">
+      <formula>TRIM(UPPER(E2))="C"</formula>
     </cfRule>
-    <cfRule type="expression" priority="5" dxfId="12">
-      <formula>UPPER(E2)="TBS"</formula>
+    <cfRule type="expression" priority="5" dxfId="17" stopIfTrue="1">
+      <formula>TRIM(UPPER(E2))="TBS"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:Q62">
+    <cfRule type="expression" priority="6" dxfId="14" stopIfTrue="1">
+      <formula>TRIM(UPPER(G2))="A"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="7" dxfId="14" stopIfTrue="1">
+      <formula>TRIM(UPPER(G2))="B"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" dxfId="18" stopIfTrue="1">
+      <formula>TRIM($R2)="Provided"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="9" dxfId="15" stopIfTrue="1">
+      <formula>TRIM(UPPER(G2))="UR"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="10" dxfId="16" stopIfTrue="1">
+      <formula>TRIM(UPPER(G2))="C"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="11" dxfId="17" stopIfTrue="1">
+      <formula>TRIM(UPPER(G2))="TBS"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R2:R62">
-    <cfRule type="expression" priority="6" dxfId="13">
-      <formula>R2="Provided"</formula>
+    <cfRule type="expression" priority="12" dxfId="19" stopIfTrue="1">
+      <formula>TRIM(R2)="Provided"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
@@ -42334,7 +42371,7 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="10" t="inlineStr">
         <is>
           <t>approved</t>
         </is>
@@ -42366,7 +42403,7 @@
           <t>Approved as Noted</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="10" t="inlineStr">
         <is>
           <t>approved</t>
         </is>
@@ -42398,7 +42435,7 @@
           <t>Under Review</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>review</t>
         </is>
@@ -42430,7 +42467,7 @@
           <t>Code C - Revise &amp; Resubmit</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="10" t="inlineStr">
         <is>
           <t>revise</t>
         </is>
@@ -42462,7 +42499,7 @@
           <t>To Be Submitted</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>pending</t>
         </is>
@@ -42484,9 +42521,9 @@
           <t>Coordinated</t>
         </is>
       </c>
-      <c r="B7" s="33" t="inlineStr">
-        <is>
-          <t>#B6E3A3</t>
+      <c r="B7" s="34" t="inlineStr">
+        <is>
+          <t>#B5E6A2</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
@@ -42494,7 +42531,7 @@
           <t>Coordination sketch provided (shown instead of a non-approved MEP/ELV status)</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="10" t="inlineStr">
         <is>
           <t>coordinated</t>
         </is>

</xml_diff>

<commit_message>
Rename Room Tag to Design Room Tag
</commit_message>
<xml_diff>
--- a/WPH_Room_Register.xlsx
+++ b/WPH_Room_Register.xlsx
@@ -25,11 +25,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="dd\-mmm\-yyyy"/>
     <numFmt numFmtId="166" formatCode="dd-mmm-yyyy"/>
-    <numFmt numFmtId="167" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -811,7 +810,7 @@
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>The room tag from the DSA typology drawings (e.g. AL02G03) is kept in the column "Room Tag" for cross-reference.</t>
+          <t>The design room tag from the DSA typology drawings (e.g. AL02G03) is kept in the column "Design Room Tag" for cross-reference.</t>
         </is>
       </c>
     </row>
@@ -846,6 +845,7 @@
         </is>
       </c>
     </row>
+    <row r="29"/>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
@@ -860,6 +860,7 @@
         </is>
       </c>
     </row>
+    <row r="32"/>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
@@ -874,6 +875,7 @@
         </is>
       </c>
     </row>
+    <row r="35"/>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
@@ -936,7 +938,7 @@
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>Room Tag</t>
+          <t>Design Room Tag</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
@@ -39562,12 +39564,12 @@
     <row r="17" ht="15" customHeight="1">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Room Tag</t>
+          <t>Design Room Tag</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Room tag</t>
+          <t>Design room tag</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -40005,8 +40007,6 @@
           <t>ID SD Reference</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
       <c r="D32" t="n">
         <v>99</v>
       </c>
@@ -40027,8 +40027,6 @@
           <t>ID SD Revision</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr"/>
-      <c r="C33" t="inlineStr"/>
       <c r="D33" t="n">
         <v>99</v>
       </c>
@@ -40049,8 +40047,6 @@
           <t>ID SD Status Date</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr"/>
-      <c r="C34" t="inlineStr"/>
       <c r="D34" t="n">
         <v>99</v>
       </c>
@@ -40071,8 +40067,6 @@
           <t>Coordination Sketch Date</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr"/>
-      <c r="C35" t="inlineStr"/>
       <c r="D35" t="n">
         <v>99</v>
       </c>
@@ -40093,8 +40087,6 @@
           <t>MEP SD - Drainage Network Rev</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr"/>
-      <c r="C36" t="inlineStr"/>
       <c r="D36" t="n">
         <v>99</v>
       </c>
@@ -40115,8 +40107,6 @@
           <t>MEP SD - Water Supply Network Rev</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr"/>
-      <c r="C37" t="inlineStr"/>
       <c r="D37" t="n">
         <v>99</v>
       </c>
@@ -40137,8 +40127,6 @@
           <t>MEP SD - Chilled Water Network Rev</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr"/>
-      <c r="C38" t="inlineStr"/>
       <c r="D38" t="n">
         <v>99</v>
       </c>
@@ -40159,8 +40147,6 @@
           <t>MEP SD - Fire Fighting Network Rev</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr"/>
-      <c r="C39" t="inlineStr"/>
       <c r="D39" t="n">
         <v>99</v>
       </c>
@@ -40181,8 +40167,6 @@
           <t>MEP SD - AC System Rev</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr"/>
-      <c r="C40" t="inlineStr"/>
       <c r="D40" t="n">
         <v>99</v>
       </c>
@@ -40203,8 +40187,6 @@
           <t>MEP SD - Ventilation System Rev</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr"/>
-      <c r="C41" t="inlineStr"/>
       <c r="D41" t="n">
         <v>99</v>
       </c>
@@ -40225,8 +40207,6 @@
           <t>MEP SD - CDP System Rev</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr"/>
-      <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
         <v>99</v>
       </c>
@@ -40247,8 +40227,6 @@
           <t>MEP SD - Small Power Rev</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr"/>
-      <c r="C43" t="inlineStr"/>
       <c r="D43" t="n">
         <v>99</v>
       </c>
@@ -40269,8 +40247,6 @@
           <t>MEP SD - Lighting Rev</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr"/>
-      <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
         <v>99</v>
       </c>
@@ -40291,8 +40267,6 @@
           <t>ELV SD - ICT System GRMS Rev</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr"/>
-      <c r="C45" t="inlineStr"/>
       <c r="D45" t="n">
         <v>99</v>
       </c>
@@ -40313,8 +40287,6 @@
           <t>ELV SD - ICT GRMS Lighting Control Rev</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr"/>
-      <c r="C46" t="inlineStr"/>
       <c r="D46" t="n">
         <v>99</v>
       </c>

</xml_diff>

<commit_message>
Import MEP/ELV shop drawing status, revisions and sketch from team log (35 non-standard room types)
</commit_message>
<xml_diff>
--- a/WPH_Room_Register.xlsx
+++ b/WPH_Room_Register.xlsx
@@ -845,7 +845,6 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
@@ -860,7 +859,6 @@
         </is>
       </c>
     </row>
-    <row r="32"/>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
@@ -875,7 +873,6 @@
         </is>
       </c>
     </row>
-    <row r="35"/>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
@@ -35007,7 +35004,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-42301</t>
         </is>
       </c>
-      <c r="D2" s="26" t="n"/>
+      <c r="D2" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E2" s="27" t="n"/>
       <c r="F2" s="28" t="n"/>
       <c r="G2" s="29" t="inlineStr">
@@ -35017,27 +35018,83 @@
       </c>
       <c r="H2" s="27" t="n"/>
       <c r="I2" s="28" t="n"/>
-      <c r="J2" s="29" t="n"/>
+      <c r="J2" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K2" s="28" t="n"/>
-      <c r="L2" s="29" t="n"/>
+      <c r="L2" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M2" s="28" t="n"/>
-      <c r="N2" s="29" t="n"/>
+      <c r="N2" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O2" s="28" t="n"/>
-      <c r="P2" s="29" t="n"/>
+      <c r="P2" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q2" s="28" t="n"/>
-      <c r="R2" s="29" t="n"/>
+      <c r="R2" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S2" s="28" t="n"/>
-      <c r="T2" s="29" t="n"/>
+      <c r="T2" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U2" s="28" t="n"/>
-      <c r="V2" s="29" t="n"/>
-      <c r="W2" s="28" t="n"/>
-      <c r="X2" s="29" t="n"/>
+      <c r="V2" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="W2" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="X2" s="29" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="Y2" s="28" t="n"/>
-      <c r="Z2" s="29" t="n"/>
-      <c r="AA2" s="28" t="n"/>
-      <c r="AB2" s="29" t="n"/>
-      <c r="AC2" s="28" t="n"/>
-      <c r="AD2" s="29" t="n"/>
+      <c r="Z2" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="AA2" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="AB2" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AC2" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="AD2" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="AE2" s="10" t="n"/>
       <c r="AF2" s="10" t="n"/>
       <c r="AG2" s="10" t="n"/>
@@ -35070,7 +35127,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-42401</t>
         </is>
       </c>
-      <c r="D3" s="26" t="n"/>
+      <c r="D3" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E3" s="27" t="n"/>
       <c r="F3" s="28" t="n"/>
       <c r="G3" s="29" t="inlineStr">
@@ -35080,29 +35141,105 @@
       </c>
       <c r="H3" s="27" t="n"/>
       <c r="I3" s="28" t="n"/>
-      <c r="J3" s="29" t="n"/>
-      <c r="K3" s="28" t="n"/>
-      <c r="L3" s="29" t="n"/>
-      <c r="M3" s="28" t="n"/>
-      <c r="N3" s="29" t="n"/>
-      <c r="O3" s="28" t="n"/>
-      <c r="P3" s="29" t="n"/>
-      <c r="Q3" s="28" t="n"/>
-      <c r="R3" s="29" t="n"/>
-      <c r="S3" s="28" t="n"/>
-      <c r="T3" s="29" t="n"/>
-      <c r="U3" s="28" t="n"/>
-      <c r="V3" s="29" t="n"/>
-      <c r="W3" s="28" t="n"/>
-      <c r="X3" s="29" t="n"/>
+      <c r="J3" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="K3" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="L3" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="M3" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="N3" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="O3" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="P3" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="Q3" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="R3" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="S3" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="T3" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="U3" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="V3" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="W3" s="28" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="X3" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="Y3" s="28" t="n"/>
-      <c r="Z3" s="29" t="n"/>
-      <c r="AA3" s="28" t="n"/>
-      <c r="AB3" s="29" t="n"/>
-      <c r="AC3" s="28" t="n"/>
+      <c r="Z3" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="AA3" s="28" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="AB3" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AC3" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
       <c r="AD3" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="AE3" s="10" t="n"/>
@@ -35139,7 +35276,7 @@
       </c>
       <c r="D4" s="26" t="inlineStr">
         <is>
-          <t>Not Provided</t>
+          <t>Provided</t>
         </is>
       </c>
       <c r="E4" s="27" t="n"/>
@@ -35155,64 +35292,80 @@
       <c r="I4" s="28" t="n"/>
       <c r="J4" s="29" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>TBS</t>
         </is>
       </c>
       <c r="K4" s="28" t="n"/>
       <c r="L4" s="29" t="inlineStr">
         <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="M4" s="28" t="n"/>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="M4" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
       <c r="N4" s="29" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="O4" s="28" t="n"/>
       <c r="P4" s="29" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>TBS</t>
         </is>
       </c>
       <c r="Q4" s="28" t="n"/>
       <c r="R4" s="29" t="inlineStr">
         <is>
-          <t>UR</t>
+          <t>TBS</t>
         </is>
       </c>
       <c r="S4" s="28" t="n"/>
       <c r="T4" s="29" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>TBS</t>
         </is>
       </c>
       <c r="U4" s="28" t="n"/>
       <c r="V4" s="29" t="inlineStr">
         <is>
-          <t>UR</t>
-        </is>
-      </c>
-      <c r="W4" s="28" t="n"/>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="W4" s="28" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
       <c r="X4" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="Y4" s="28" t="n"/>
       <c r="Z4" s="29" t="inlineStr">
         <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="AA4" s="28" t="n"/>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="AA4" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
       <c r="AB4" s="29" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="AC4" s="28" t="n"/>
+      <c r="AC4" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
       <c r="AD4" s="29" t="inlineStr">
         <is>
           <t>B</t>
@@ -35250,7 +35403,11 @@
           <t>(no drawing number in legend)</t>
         </is>
       </c>
-      <c r="D5" s="26" t="n"/>
+      <c r="D5" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E5" s="27" t="n"/>
       <c r="F5" s="28" t="n"/>
       <c r="G5" s="29" t="inlineStr">
@@ -35260,27 +35417,91 @@
       </c>
       <c r="H5" s="27" t="n"/>
       <c r="I5" s="28" t="n"/>
-      <c r="J5" s="29" t="n"/>
+      <c r="J5" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K5" s="28" t="n"/>
-      <c r="L5" s="29" t="n"/>
-      <c r="M5" s="28" t="n"/>
-      <c r="N5" s="29" t="n"/>
+      <c r="L5" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="M5" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="N5" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="O5" s="28" t="n"/>
-      <c r="P5" s="29" t="n"/>
+      <c r="P5" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q5" s="28" t="n"/>
-      <c r="R5" s="29" t="n"/>
+      <c r="R5" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S5" s="28" t="n"/>
-      <c r="T5" s="29" t="n"/>
+      <c r="T5" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U5" s="28" t="n"/>
-      <c r="V5" s="29" t="n"/>
-      <c r="W5" s="28" t="n"/>
-      <c r="X5" s="29" t="n"/>
-      <c r="Y5" s="28" t="n"/>
-      <c r="Z5" s="29" t="n"/>
-      <c r="AA5" s="28" t="n"/>
-      <c r="AB5" s="29" t="n"/>
-      <c r="AC5" s="28" t="n"/>
-      <c r="AD5" s="29" t="n"/>
+      <c r="V5" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="W5" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="X5" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="Y5" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="Z5" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="AA5" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="AB5" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AC5" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="AD5" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="AE5" s="10" t="n"/>
       <c r="AF5" s="10" t="n"/>
       <c r="AG5" s="10" t="n"/>
@@ -35376,7 +35597,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-42801</t>
         </is>
       </c>
-      <c r="D7" s="26" t="n"/>
+      <c r="D7" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E7" s="27" t="n"/>
       <c r="F7" s="28" t="n"/>
       <c r="G7" s="29" t="inlineStr">
@@ -35386,27 +35611,107 @@
       </c>
       <c r="H7" s="27" t="n"/>
       <c r="I7" s="28" t="n"/>
-      <c r="J7" s="29" t="n"/>
-      <c r="K7" s="28" t="n"/>
-      <c r="L7" s="29" t="n"/>
-      <c r="M7" s="28" t="n"/>
-      <c r="N7" s="29" t="n"/>
-      <c r="O7" s="28" t="n"/>
-      <c r="P7" s="29" t="n"/>
-      <c r="Q7" s="28" t="n"/>
-      <c r="R7" s="29" t="n"/>
-      <c r="S7" s="28" t="n"/>
-      <c r="T7" s="29" t="n"/>
-      <c r="U7" s="28" t="n"/>
-      <c r="V7" s="29" t="n"/>
-      <c r="W7" s="28" t="n"/>
-      <c r="X7" s="29" t="n"/>
+      <c r="J7" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="K7" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="L7" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="M7" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="N7" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="O7" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="P7" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="Q7" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="R7" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="S7" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="T7" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="U7" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="V7" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="W7" s="28" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="X7" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="Y7" s="28" t="n"/>
-      <c r="Z7" s="29" t="n"/>
-      <c r="AA7" s="28" t="n"/>
-      <c r="AB7" s="29" t="n"/>
-      <c r="AC7" s="28" t="n"/>
-      <c r="AD7" s="29" t="n"/>
+      <c r="Z7" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="AA7" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="AB7" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AC7" s="28" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="AD7" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="AE7" s="10" t="n"/>
       <c r="AF7" s="10" t="n"/>
       <c r="AG7" s="10" t="n"/>
@@ -35439,7 +35744,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-42901</t>
         </is>
       </c>
-      <c r="D8" s="26" t="n"/>
+      <c r="D8" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E8" s="27" t="n"/>
       <c r="F8" s="28" t="n"/>
       <c r="G8" s="29" t="inlineStr">
@@ -35449,27 +35758,83 @@
       </c>
       <c r="H8" s="27" t="n"/>
       <c r="I8" s="28" t="n"/>
-      <c r="J8" s="29" t="n"/>
+      <c r="J8" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K8" s="28" t="n"/>
-      <c r="L8" s="29" t="n"/>
+      <c r="L8" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M8" s="28" t="n"/>
-      <c r="N8" s="29" t="n"/>
+      <c r="N8" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O8" s="28" t="n"/>
-      <c r="P8" s="29" t="n"/>
+      <c r="P8" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q8" s="28" t="n"/>
-      <c r="R8" s="29" t="n"/>
+      <c r="R8" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S8" s="28" t="n"/>
-      <c r="T8" s="29" t="n"/>
+      <c r="T8" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U8" s="28" t="n"/>
-      <c r="V8" s="29" t="n"/>
-      <c r="W8" s="28" t="n"/>
-      <c r="X8" s="29" t="n"/>
+      <c r="V8" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="W8" s="28" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="X8" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="Y8" s="28" t="n"/>
-      <c r="Z8" s="29" t="n"/>
-      <c r="AA8" s="28" t="n"/>
-      <c r="AB8" s="29" t="n"/>
-      <c r="AC8" s="28" t="n"/>
-      <c r="AD8" s="29" t="n"/>
+      <c r="Z8" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="AA8" s="28" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="AB8" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AC8" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="AD8" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="AE8" s="10" t="n"/>
       <c r="AF8" s="10" t="n"/>
       <c r="AG8" s="10" t="n"/>
@@ -35502,7 +35867,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-43001</t>
         </is>
       </c>
-      <c r="D9" s="26" t="n"/>
+      <c r="D9" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E9" s="27" t="n"/>
       <c r="F9" s="28" t="n"/>
       <c r="G9" s="29" t="inlineStr">
@@ -35511,28 +35880,116 @@
         </is>
       </c>
       <c r="H9" s="27" t="n"/>
-      <c r="I9" s="28" t="n"/>
-      <c r="J9" s="29" t="n"/>
-      <c r="K9" s="28" t="n"/>
-      <c r="L9" s="29" t="n"/>
-      <c r="M9" s="28" t="n"/>
-      <c r="N9" s="29" t="n"/>
-      <c r="O9" s="28" t="n"/>
-      <c r="P9" s="29" t="n"/>
-      <c r="Q9" s="28" t="n"/>
-      <c r="R9" s="29" t="n"/>
-      <c r="S9" s="28" t="n"/>
-      <c r="T9" s="29" t="n"/>
-      <c r="U9" s="28" t="n"/>
-      <c r="V9" s="29" t="n"/>
-      <c r="W9" s="28" t="n"/>
-      <c r="X9" s="29" t="n"/>
-      <c r="Y9" s="28" t="n"/>
-      <c r="Z9" s="29" t="n"/>
-      <c r="AA9" s="28" t="n"/>
-      <c r="AB9" s="29" t="n"/>
-      <c r="AC9" s="28" t="n"/>
-      <c r="AD9" s="29" t="n"/>
+      <c r="I9" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="J9" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="K9" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="L9" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="M9" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="N9" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="O9" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="P9" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="Q9" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="R9" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="S9" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="T9" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="U9" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="V9" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="W9" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="X9" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="Y9" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="Z9" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AA9" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="AB9" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AC9" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="AD9" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="AE9" s="10" t="n"/>
       <c r="AF9" s="10" t="n"/>
       <c r="AG9" s="10" t="n"/>
@@ -35565,7 +36022,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-43101</t>
         </is>
       </c>
-      <c r="D10" s="26" t="n"/>
+      <c r="D10" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E10" s="27" t="n"/>
       <c r="F10" s="28" t="n"/>
       <c r="G10" s="29" t="inlineStr">
@@ -35575,27 +36036,83 @@
       </c>
       <c r="H10" s="27" t="n"/>
       <c r="I10" s="28" t="n"/>
-      <c r="J10" s="29" t="n"/>
+      <c r="J10" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K10" s="28" t="n"/>
-      <c r="L10" s="29" t="n"/>
+      <c r="L10" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M10" s="28" t="n"/>
-      <c r="N10" s="29" t="n"/>
+      <c r="N10" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O10" s="28" t="n"/>
-      <c r="P10" s="29" t="n"/>
+      <c r="P10" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q10" s="28" t="n"/>
-      <c r="R10" s="29" t="n"/>
+      <c r="R10" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S10" s="28" t="n"/>
-      <c r="T10" s="29" t="n"/>
+      <c r="T10" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U10" s="28" t="n"/>
-      <c r="V10" s="29" t="n"/>
-      <c r="W10" s="28" t="n"/>
-      <c r="X10" s="29" t="n"/>
+      <c r="V10" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="W10" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="X10" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="Y10" s="28" t="n"/>
-      <c r="Z10" s="29" t="n"/>
-      <c r="AA10" s="28" t="n"/>
-      <c r="AB10" s="29" t="n"/>
-      <c r="AC10" s="28" t="n"/>
-      <c r="AD10" s="29" t="n"/>
+      <c r="Z10" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="AA10" s="28" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="AB10" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AC10" s="28" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="AD10" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="AE10" s="10" t="n"/>
       <c r="AF10" s="10" t="n"/>
       <c r="AG10" s="10" t="n"/>
@@ -35628,7 +36145,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-43201</t>
         </is>
       </c>
-      <c r="D11" s="26" t="n"/>
+      <c r="D11" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E11" s="27" t="n"/>
       <c r="F11" s="28" t="n"/>
       <c r="G11" s="29" t="inlineStr">
@@ -35638,27 +36159,79 @@
       </c>
       <c r="H11" s="27" t="n"/>
       <c r="I11" s="28" t="n"/>
-      <c r="J11" s="29" t="n"/>
+      <c r="J11" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K11" s="28" t="n"/>
-      <c r="L11" s="29" t="n"/>
+      <c r="L11" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M11" s="28" t="n"/>
-      <c r="N11" s="29" t="n"/>
+      <c r="N11" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O11" s="28" t="n"/>
-      <c r="P11" s="29" t="n"/>
+      <c r="P11" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q11" s="28" t="n"/>
-      <c r="R11" s="29" t="n"/>
+      <c r="R11" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S11" s="28" t="n"/>
-      <c r="T11" s="29" t="n"/>
+      <c r="T11" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U11" s="28" t="n"/>
-      <c r="V11" s="29" t="n"/>
+      <c r="V11" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W11" s="28" t="n"/>
-      <c r="X11" s="29" t="n"/>
+      <c r="X11" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y11" s="28" t="n"/>
-      <c r="Z11" s="29" t="n"/>
-      <c r="AA11" s="28" t="n"/>
-      <c r="AB11" s="29" t="n"/>
-      <c r="AC11" s="28" t="n"/>
-      <c r="AD11" s="29" t="n"/>
+      <c r="Z11" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="AA11" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="AB11" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AC11" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="AD11" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="AE11" s="10" t="n"/>
       <c r="AF11" s="10" t="n"/>
       <c r="AG11" s="10" t="n"/>
@@ -35691,7 +36264,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-43301</t>
         </is>
       </c>
-      <c r="D12" s="26" t="n"/>
+      <c r="D12" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E12" s="27" t="n"/>
       <c r="F12" s="28" t="n"/>
       <c r="G12" s="29" t="inlineStr">
@@ -35700,28 +36277,112 @@
         </is>
       </c>
       <c r="H12" s="27" t="n"/>
-      <c r="I12" s="28" t="n"/>
-      <c r="J12" s="29" t="n"/>
-      <c r="K12" s="28" t="n"/>
-      <c r="L12" s="29" t="n"/>
-      <c r="M12" s="28" t="n"/>
-      <c r="N12" s="29" t="n"/>
-      <c r="O12" s="28" t="n"/>
-      <c r="P12" s="29" t="n"/>
-      <c r="Q12" s="28" t="n"/>
-      <c r="R12" s="29" t="n"/>
-      <c r="S12" s="28" t="n"/>
-      <c r="T12" s="29" t="n"/>
-      <c r="U12" s="28" t="n"/>
-      <c r="V12" s="29" t="n"/>
-      <c r="W12" s="28" t="n"/>
-      <c r="X12" s="29" t="n"/>
+      <c r="I12" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="J12" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K12" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="L12" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="M12" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="N12" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="O12" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="P12" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="Q12" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="R12" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="S12" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="T12" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="U12" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="V12" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="W12" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="X12" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="Y12" s="28" t="n"/>
-      <c r="Z12" s="29" t="n"/>
-      <c r="AA12" s="28" t="n"/>
-      <c r="AB12" s="29" t="n"/>
-      <c r="AC12" s="28" t="n"/>
-      <c r="AD12" s="29" t="n"/>
+      <c r="Z12" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="AA12" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="AB12" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="AC12" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="AD12" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
       <c r="AE12" s="10" t="n"/>
       <c r="AF12" s="10" t="n"/>
       <c r="AG12" s="10" t="n"/>
@@ -36573,7 +37234,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-41101</t>
         </is>
       </c>
-      <c r="D26" s="26" t="n"/>
+      <c r="D26" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E26" s="27" t="n"/>
       <c r="F26" s="28" t="n"/>
       <c r="G26" s="29" t="inlineStr">
@@ -36583,27 +37248,83 @@
       </c>
       <c r="H26" s="27" t="n"/>
       <c r="I26" s="28" t="n"/>
-      <c r="J26" s="29" t="n"/>
-      <c r="K26" s="28" t="n"/>
-      <c r="L26" s="29" t="n"/>
-      <c r="M26" s="28" t="n"/>
-      <c r="N26" s="29" t="n"/>
+      <c r="J26" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="K26" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="L26" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="M26" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="N26" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="O26" s="28" t="n"/>
-      <c r="P26" s="29" t="n"/>
+      <c r="P26" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q26" s="28" t="n"/>
-      <c r="R26" s="29" t="n"/>
+      <c r="R26" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S26" s="28" t="n"/>
-      <c r="T26" s="29" t="n"/>
+      <c r="T26" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U26" s="28" t="n"/>
-      <c r="V26" s="29" t="n"/>
-      <c r="W26" s="28" t="n"/>
-      <c r="X26" s="29" t="n"/>
+      <c r="V26" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="W26" s="28" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="X26" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="Y26" s="28" t="n"/>
-      <c r="Z26" s="29" t="n"/>
+      <c r="Z26" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA26" s="28" t="n"/>
-      <c r="AB26" s="29" t="n"/>
+      <c r="AB26" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC26" s="28" t="n"/>
-      <c r="AD26" s="29" t="n"/>
+      <c r="AD26" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE26" s="10" t="n"/>
       <c r="AF26" s="10" t="n"/>
       <c r="AG26" s="10" t="n"/>
@@ -36636,7 +37357,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-41201</t>
         </is>
       </c>
-      <c r="D27" s="26" t="n"/>
+      <c r="D27" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E27" s="27" t="n"/>
       <c r="F27" s="28" t="n"/>
       <c r="G27" s="29" t="inlineStr">
@@ -36646,27 +37371,83 @@
       </c>
       <c r="H27" s="27" t="n"/>
       <c r="I27" s="28" t="n"/>
-      <c r="J27" s="29" t="n"/>
-      <c r="K27" s="28" t="n"/>
-      <c r="L27" s="29" t="n"/>
-      <c r="M27" s="28" t="n"/>
-      <c r="N27" s="29" t="n"/>
+      <c r="J27" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="K27" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="L27" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="M27" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="N27" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="O27" s="28" t="n"/>
-      <c r="P27" s="29" t="n"/>
+      <c r="P27" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q27" s="28" t="n"/>
-      <c r="R27" s="29" t="n"/>
+      <c r="R27" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S27" s="28" t="n"/>
-      <c r="T27" s="29" t="n"/>
+      <c r="T27" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U27" s="28" t="n"/>
-      <c r="V27" s="29" t="n"/>
-      <c r="W27" s="28" t="n"/>
-      <c r="X27" s="29" t="n"/>
+      <c r="V27" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="W27" s="28" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="X27" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="Y27" s="28" t="n"/>
-      <c r="Z27" s="29" t="n"/>
+      <c r="Z27" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA27" s="28" t="n"/>
-      <c r="AB27" s="29" t="n"/>
+      <c r="AB27" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC27" s="28" t="n"/>
-      <c r="AD27" s="29" t="n"/>
+      <c r="AD27" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE27" s="10" t="n"/>
       <c r="AF27" s="10" t="n"/>
       <c r="AG27" s="10" t="n"/>
@@ -36699,7 +37480,11 @@
           <t>(no drawing number in legend)</t>
         </is>
       </c>
-      <c r="D28" s="26" t="n"/>
+      <c r="D28" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E28" s="27" t="n"/>
       <c r="F28" s="28" t="n"/>
       <c r="G28" s="29" t="inlineStr">
@@ -36709,27 +37494,75 @@
       </c>
       <c r="H28" s="27" t="n"/>
       <c r="I28" s="28" t="n"/>
-      <c r="J28" s="29" t="n"/>
+      <c r="J28" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K28" s="28" t="n"/>
-      <c r="L28" s="29" t="n"/>
+      <c r="L28" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M28" s="28" t="n"/>
-      <c r="N28" s="29" t="n"/>
+      <c r="N28" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O28" s="28" t="n"/>
-      <c r="P28" s="29" t="n"/>
+      <c r="P28" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q28" s="28" t="n"/>
-      <c r="R28" s="29" t="n"/>
+      <c r="R28" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S28" s="28" t="n"/>
-      <c r="T28" s="29" t="n"/>
+      <c r="T28" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U28" s="28" t="n"/>
-      <c r="V28" s="29" t="n"/>
-      <c r="W28" s="28" t="n"/>
-      <c r="X28" s="29" t="n"/>
+      <c r="V28" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="W28" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="X28" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="Y28" s="28" t="n"/>
-      <c r="Z28" s="29" t="n"/>
+      <c r="Z28" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA28" s="28" t="n"/>
-      <c r="AB28" s="29" t="n"/>
+      <c r="AB28" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC28" s="28" t="n"/>
-      <c r="AD28" s="29" t="n"/>
+      <c r="AD28" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE28" s="10" t="n"/>
       <c r="AF28" s="10" t="n"/>
       <c r="AG28" s="10" t="n"/>
@@ -37329,7 +38162,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-42001</t>
         </is>
       </c>
-      <c r="D38" s="26" t="n"/>
+      <c r="D38" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E38" s="27" t="n"/>
       <c r="F38" s="28" t="n"/>
       <c r="G38" s="29" t="inlineStr">
@@ -37338,28 +38175,108 @@
         </is>
       </c>
       <c r="H38" s="27" t="n"/>
-      <c r="I38" s="28" t="n"/>
-      <c r="J38" s="29" t="n"/>
-      <c r="K38" s="28" t="n"/>
-      <c r="L38" s="29" t="n"/>
-      <c r="M38" s="28" t="n"/>
-      <c r="N38" s="29" t="n"/>
-      <c r="O38" s="28" t="n"/>
-      <c r="P38" s="29" t="n"/>
-      <c r="Q38" s="28" t="n"/>
-      <c r="R38" s="29" t="n"/>
-      <c r="S38" s="28" t="n"/>
-      <c r="T38" s="29" t="n"/>
-      <c r="U38" s="28" t="n"/>
-      <c r="V38" s="29" t="n"/>
-      <c r="W38" s="28" t="n"/>
-      <c r="X38" s="29" t="n"/>
-      <c r="Y38" s="28" t="n"/>
-      <c r="Z38" s="29" t="n"/>
+      <c r="I38" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="J38" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K38" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="L38" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="M38" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="N38" s="29" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="O38" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="P38" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="Q38" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="R38" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="S38" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="T38" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="U38" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="V38" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="W38" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="X38" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="Y38" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="Z38" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="AA38" s="28" t="n"/>
-      <c r="AB38" s="29" t="n"/>
+      <c r="AB38" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC38" s="28" t="n"/>
-      <c r="AD38" s="29" t="n"/>
+      <c r="AD38" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE38" s="10" t="n"/>
       <c r="AF38" s="10" t="n"/>
       <c r="AG38" s="10" t="n"/>
@@ -37392,7 +38309,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-42101</t>
         </is>
       </c>
-      <c r="D39" s="26" t="n"/>
+      <c r="D39" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E39" s="27" t="n"/>
       <c r="F39" s="28" t="n"/>
       <c r="G39" s="29" t="inlineStr">
@@ -37401,28 +38322,104 @@
         </is>
       </c>
       <c r="H39" s="27" t="n"/>
-      <c r="I39" s="28" t="n"/>
-      <c r="J39" s="29" t="n"/>
-      <c r="K39" s="28" t="n"/>
-      <c r="L39" s="29" t="n"/>
-      <c r="M39" s="28" t="n"/>
-      <c r="N39" s="29" t="n"/>
-      <c r="O39" s="28" t="n"/>
-      <c r="P39" s="29" t="n"/>
-      <c r="Q39" s="28" t="n"/>
-      <c r="R39" s="29" t="n"/>
-      <c r="S39" s="28" t="n"/>
-      <c r="T39" s="29" t="n"/>
-      <c r="U39" s="28" t="n"/>
-      <c r="V39" s="29" t="n"/>
-      <c r="W39" s="28" t="n"/>
-      <c r="X39" s="29" t="n"/>
+      <c r="I39" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="J39" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K39" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="L39" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="M39" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="N39" s="29" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="O39" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="P39" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="Q39" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="R39" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="S39" s="28" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="T39" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="U39" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="V39" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="W39" s="28" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="X39" s="29" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="Y39" s="28" t="n"/>
-      <c r="Z39" s="29" t="n"/>
+      <c r="Z39" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA39" s="28" t="n"/>
-      <c r="AB39" s="29" t="n"/>
+      <c r="AB39" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC39" s="28" t="n"/>
-      <c r="AD39" s="29" t="n"/>
+      <c r="AD39" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE39" s="10" t="n"/>
       <c r="AF39" s="10" t="n"/>
       <c r="AG39" s="10" t="n"/>
@@ -37518,7 +38515,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-41501</t>
         </is>
       </c>
-      <c r="D41" s="26" t="n"/>
+      <c r="D41" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E41" s="27" t="n"/>
       <c r="F41" s="28" t="n"/>
       <c r="G41" s="29" t="inlineStr">
@@ -37527,28 +38528,104 @@
         </is>
       </c>
       <c r="H41" s="27" t="n"/>
-      <c r="I41" s="28" t="n"/>
-      <c r="J41" s="29" t="n"/>
-      <c r="K41" s="28" t="n"/>
-      <c r="L41" s="29" t="n"/>
-      <c r="M41" s="28" t="n"/>
-      <c r="N41" s="29" t="n"/>
-      <c r="O41" s="28" t="n"/>
-      <c r="P41" s="29" t="n"/>
-      <c r="Q41" s="28" t="n"/>
-      <c r="R41" s="29" t="n"/>
-      <c r="S41" s="28" t="n"/>
-      <c r="T41" s="29" t="n"/>
-      <c r="U41" s="28" t="n"/>
-      <c r="V41" s="29" t="n"/>
-      <c r="W41" s="28" t="n"/>
-      <c r="X41" s="29" t="n"/>
+      <c r="I41" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="J41" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K41" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="L41" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="M41" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="N41" s="29" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="O41" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="P41" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="Q41" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="R41" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="S41" s="28" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="T41" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="U41" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="V41" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="W41" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="X41" s="29" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="Y41" s="28" t="n"/>
-      <c r="Z41" s="29" t="n"/>
+      <c r="Z41" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA41" s="28" t="n"/>
-      <c r="AB41" s="29" t="n"/>
+      <c r="AB41" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC41" s="28" t="n"/>
-      <c r="AD41" s="29" t="n"/>
+      <c r="AD41" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE41" s="10" t="n"/>
       <c r="AF41" s="10" t="n"/>
       <c r="AG41" s="10" t="n"/>
@@ -37581,7 +38658,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-41701</t>
         </is>
       </c>
-      <c r="D42" s="26" t="n"/>
+      <c r="D42" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E42" s="27" t="n"/>
       <c r="F42" s="28" t="n"/>
       <c r="G42" s="29" t="inlineStr">
@@ -37590,28 +38671,100 @@
         </is>
       </c>
       <c r="H42" s="27" t="n"/>
-      <c r="I42" s="28" t="n"/>
-      <c r="J42" s="29" t="n"/>
-      <c r="K42" s="28" t="n"/>
-      <c r="L42" s="29" t="n"/>
-      <c r="M42" s="28" t="n"/>
-      <c r="N42" s="29" t="n"/>
-      <c r="O42" s="28" t="n"/>
-      <c r="P42" s="29" t="n"/>
-      <c r="Q42" s="28" t="n"/>
-      <c r="R42" s="29" t="n"/>
-      <c r="S42" s="28" t="n"/>
-      <c r="T42" s="29" t="n"/>
-      <c r="U42" s="28" t="n"/>
-      <c r="V42" s="29" t="n"/>
+      <c r="I42" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="J42" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K42" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="L42" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="M42" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="N42" s="29" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="O42" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="P42" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="Q42" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="R42" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="S42" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="T42" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="U42" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="V42" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="W42" s="28" t="n"/>
-      <c r="X42" s="29" t="n"/>
+      <c r="X42" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y42" s="28" t="n"/>
-      <c r="Z42" s="29" t="n"/>
+      <c r="Z42" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA42" s="28" t="n"/>
-      <c r="AB42" s="29" t="n"/>
+      <c r="AB42" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC42" s="28" t="n"/>
-      <c r="AD42" s="29" t="n"/>
+      <c r="AD42" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE42" s="10" t="n"/>
       <c r="AF42" s="10" t="n"/>
       <c r="AG42" s="10" t="n"/>
@@ -37770,7 +38923,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-42201</t>
         </is>
       </c>
-      <c r="D45" s="26" t="n"/>
+      <c r="D45" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E45" s="27" t="n"/>
       <c r="F45" s="28" t="n"/>
       <c r="G45" s="29" t="inlineStr">
@@ -37779,28 +38936,116 @@
         </is>
       </c>
       <c r="H45" s="27" t="n"/>
-      <c r="I45" s="28" t="n"/>
-      <c r="J45" s="29" t="n"/>
-      <c r="K45" s="28" t="n"/>
-      <c r="L45" s="29" t="n"/>
-      <c r="M45" s="28" t="n"/>
-      <c r="N45" s="29" t="n"/>
-      <c r="O45" s="28" t="n"/>
-      <c r="P45" s="29" t="n"/>
-      <c r="Q45" s="28" t="n"/>
-      <c r="R45" s="29" t="n"/>
-      <c r="S45" s="28" t="n"/>
-      <c r="T45" s="29" t="n"/>
-      <c r="U45" s="28" t="n"/>
-      <c r="V45" s="29" t="n"/>
-      <c r="W45" s="28" t="n"/>
-      <c r="X45" s="29" t="n"/>
-      <c r="Y45" s="28" t="n"/>
-      <c r="Z45" s="29" t="n"/>
-      <c r="AA45" s="28" t="n"/>
-      <c r="AB45" s="29" t="n"/>
-      <c r="AC45" s="28" t="n"/>
-      <c r="AD45" s="29" t="n"/>
+      <c r="I45" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="J45" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="K45" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="L45" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="M45" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="N45" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="O45" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="P45" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="Q45" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="R45" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="S45" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="T45" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="U45" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="V45" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="W45" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="X45" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="Y45" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="Z45" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="AA45" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="AB45" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="AC45" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="AD45" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
       <c r="AE45" s="10" t="n"/>
       <c r="AF45" s="10" t="n"/>
       <c r="AG45" s="10" t="n"/>
@@ -37833,7 +39078,11 @@
           <t>(no drawing number in legend)</t>
         </is>
       </c>
-      <c r="D46" s="26" t="n"/>
+      <c r="D46" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E46" s="27" t="n"/>
       <c r="F46" s="28" t="n"/>
       <c r="G46" s="29" t="inlineStr">
@@ -37843,27 +39092,87 @@
       </c>
       <c r="H46" s="27" t="n"/>
       <c r="I46" s="28" t="n"/>
-      <c r="J46" s="29" t="n"/>
+      <c r="J46" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K46" s="28" t="n"/>
-      <c r="L46" s="29" t="n"/>
+      <c r="L46" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M46" s="28" t="n"/>
-      <c r="N46" s="29" t="n"/>
+      <c r="N46" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O46" s="28" t="n"/>
-      <c r="P46" s="29" t="n"/>
+      <c r="P46" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q46" s="28" t="n"/>
-      <c r="R46" s="29" t="n"/>
+      <c r="R46" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S46" s="28" t="n"/>
-      <c r="T46" s="29" t="n"/>
+      <c r="T46" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U46" s="28" t="n"/>
-      <c r="V46" s="29" t="n"/>
-      <c r="W46" s="28" t="n"/>
-      <c r="X46" s="29" t="n"/>
-      <c r="Y46" s="28" t="n"/>
-      <c r="Z46" s="29" t="n"/>
-      <c r="AA46" s="28" t="n"/>
-      <c r="AB46" s="29" t="n"/>
-      <c r="AC46" s="28" t="n"/>
-      <c r="AD46" s="29" t="n"/>
+      <c r="V46" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="W46" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="X46" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="Y46" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="Z46" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="AA46" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="AB46" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="AC46" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="AD46" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
       <c r="AE46" s="10" t="n"/>
       <c r="AF46" s="10" t="n"/>
       <c r="AG46" s="10" t="n"/>
@@ -37896,7 +39205,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-43401</t>
         </is>
       </c>
-      <c r="D47" s="26" t="n"/>
+      <c r="D47" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E47" s="27" t="n"/>
       <c r="F47" s="28" t="n"/>
       <c r="G47" s="29" t="inlineStr">
@@ -37905,28 +39218,116 @@
         </is>
       </c>
       <c r="H47" s="27" t="n"/>
-      <c r="I47" s="28" t="n"/>
-      <c r="J47" s="29" t="n"/>
-      <c r="K47" s="28" t="n"/>
-      <c r="L47" s="29" t="n"/>
-      <c r="M47" s="28" t="n"/>
-      <c r="N47" s="29" t="n"/>
-      <c r="O47" s="28" t="n"/>
-      <c r="P47" s="29" t="n"/>
-      <c r="Q47" s="28" t="n"/>
-      <c r="R47" s="29" t="n"/>
-      <c r="S47" s="28" t="n"/>
-      <c r="T47" s="29" t="n"/>
-      <c r="U47" s="28" t="n"/>
-      <c r="V47" s="29" t="n"/>
-      <c r="W47" s="28" t="n"/>
-      <c r="X47" s="29" t="n"/>
-      <c r="Y47" s="28" t="n"/>
-      <c r="Z47" s="29" t="n"/>
-      <c r="AA47" s="28" t="n"/>
-      <c r="AB47" s="29" t="n"/>
-      <c r="AC47" s="28" t="n"/>
-      <c r="AD47" s="29" t="n"/>
+      <c r="I47" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="J47" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="K47" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="L47" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="M47" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="N47" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="O47" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="P47" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="Q47" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="R47" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="S47" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="T47" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="U47" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="V47" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="W47" s="28" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="X47" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="Y47" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="Z47" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AA47" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="AB47" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AC47" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="AD47" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="AE47" s="10" t="n"/>
       <c r="AF47" s="10" t="n"/>
       <c r="AG47" s="10" t="n"/>
@@ -37959,7 +39360,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-43501</t>
         </is>
       </c>
-      <c r="D48" s="26" t="n"/>
+      <c r="D48" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E48" s="27" t="n"/>
       <c r="F48" s="28" t="n"/>
       <c r="G48" s="29" t="inlineStr">
@@ -37968,28 +39373,112 @@
         </is>
       </c>
       <c r="H48" s="27" t="n"/>
-      <c r="I48" s="28" t="n"/>
-      <c r="J48" s="29" t="n"/>
-      <c r="K48" s="28" t="n"/>
-      <c r="L48" s="29" t="n"/>
-      <c r="M48" s="28" t="n"/>
-      <c r="N48" s="29" t="n"/>
-      <c r="O48" s="28" t="n"/>
-      <c r="P48" s="29" t="n"/>
-      <c r="Q48" s="28" t="n"/>
-      <c r="R48" s="29" t="n"/>
-      <c r="S48" s="28" t="n"/>
-      <c r="T48" s="29" t="n"/>
-      <c r="U48" s="28" t="n"/>
-      <c r="V48" s="29" t="n"/>
-      <c r="W48" s="28" t="n"/>
-      <c r="X48" s="29" t="n"/>
+      <c r="I48" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="J48" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="K48" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="L48" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="M48" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="N48" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="O48" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="P48" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="Q48" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="R48" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="S48" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="T48" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="U48" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="V48" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="W48" s="28" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="X48" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="Y48" s="28" t="n"/>
-      <c r="Z48" s="29" t="n"/>
-      <c r="AA48" s="28" t="n"/>
-      <c r="AB48" s="29" t="n"/>
-      <c r="AC48" s="28" t="n"/>
-      <c r="AD48" s="29" t="n"/>
+      <c r="Z48" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="AA48" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="AB48" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AC48" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="AD48" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="AE48" s="10" t="n"/>
       <c r="AF48" s="10" t="n"/>
       <c r="AG48" s="10" t="n"/>
@@ -38022,7 +39511,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-43601</t>
         </is>
       </c>
-      <c r="D49" s="26" t="n"/>
+      <c r="D49" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E49" s="27" t="n"/>
       <c r="F49" s="28" t="n"/>
       <c r="G49" s="29" t="inlineStr">
@@ -38032,27 +39525,87 @@
       </c>
       <c r="H49" s="27" t="n"/>
       <c r="I49" s="28" t="n"/>
-      <c r="J49" s="29" t="n"/>
+      <c r="J49" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K49" s="28" t="n"/>
-      <c r="L49" s="29" t="n"/>
-      <c r="M49" s="28" t="n"/>
-      <c r="N49" s="29" t="n"/>
+      <c r="L49" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="M49" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="N49" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="O49" s="28" t="n"/>
-      <c r="P49" s="29" t="n"/>
+      <c r="P49" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q49" s="28" t="n"/>
-      <c r="R49" s="29" t="n"/>
+      <c r="R49" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S49" s="28" t="n"/>
-      <c r="T49" s="29" t="n"/>
+      <c r="T49" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U49" s="28" t="n"/>
-      <c r="V49" s="29" t="n"/>
-      <c r="W49" s="28" t="n"/>
-      <c r="X49" s="29" t="n"/>
+      <c r="V49" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="W49" s="28" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="X49" s="29" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="Y49" s="28" t="n"/>
-      <c r="Z49" s="29" t="n"/>
-      <c r="AA49" s="28" t="n"/>
-      <c r="AB49" s="29" t="n"/>
-      <c r="AC49" s="28" t="n"/>
-      <c r="AD49" s="29" t="n"/>
+      <c r="Z49" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="AA49" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="AB49" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AC49" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="AD49" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="AE49" s="10" t="n"/>
       <c r="AF49" s="10" t="n"/>
       <c r="AG49" s="10" t="n"/>
@@ -38085,7 +39638,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-43701</t>
         </is>
       </c>
-      <c r="D50" s="26" t="n"/>
+      <c r="D50" s="26" t="inlineStr">
+        <is>
+          <t>Provided</t>
+        </is>
+      </c>
       <c r="E50" s="27" t="n"/>
       <c r="F50" s="28" t="n"/>
       <c r="G50" s="29" t="inlineStr">
@@ -38094,28 +39651,116 @@
         </is>
       </c>
       <c r="H50" s="27" t="n"/>
-      <c r="I50" s="28" t="n"/>
-      <c r="J50" s="29" t="n"/>
-      <c r="K50" s="28" t="n"/>
-      <c r="L50" s="29" t="n"/>
-      <c r="M50" s="28" t="n"/>
-      <c r="N50" s="29" t="n"/>
-      <c r="O50" s="28" t="n"/>
-      <c r="P50" s="29" t="n"/>
-      <c r="Q50" s="28" t="n"/>
-      <c r="R50" s="29" t="n"/>
-      <c r="S50" s="28" t="n"/>
-      <c r="T50" s="29" t="n"/>
-      <c r="U50" s="28" t="n"/>
-      <c r="V50" s="29" t="n"/>
-      <c r="W50" s="28" t="n"/>
-      <c r="X50" s="29" t="n"/>
-      <c r="Y50" s="28" t="n"/>
-      <c r="Z50" s="29" t="n"/>
-      <c r="AA50" s="28" t="n"/>
-      <c r="AB50" s="29" t="n"/>
-      <c r="AC50" s="28" t="n"/>
-      <c r="AD50" s="29" t="n"/>
+      <c r="I50" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="J50" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K50" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="L50" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="M50" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="N50" s="29" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="O50" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="P50" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="Q50" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="R50" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="S50" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="T50" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="U50" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="V50" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="W50" s="28" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="X50" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="Y50" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="Z50" s="29" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="AA50" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="AB50" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AC50" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="AD50" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="AE50" s="10" t="n"/>
       <c r="AF50" s="10" t="n"/>
       <c r="AG50" s="10" t="n"/>
@@ -38148,7 +39793,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-43801</t>
         </is>
       </c>
-      <c r="D51" s="26" t="n"/>
+      <c r="D51" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E51" s="27" t="n"/>
       <c r="F51" s="28" t="n"/>
       <c r="G51" s="29" t="inlineStr">
@@ -38157,28 +39806,116 @@
         </is>
       </c>
       <c r="H51" s="27" t="n"/>
-      <c r="I51" s="28" t="n"/>
-      <c r="J51" s="29" t="n"/>
-      <c r="K51" s="28" t="n"/>
-      <c r="L51" s="29" t="n"/>
-      <c r="M51" s="28" t="n"/>
-      <c r="N51" s="29" t="n"/>
-      <c r="O51" s="28" t="n"/>
-      <c r="P51" s="29" t="n"/>
-      <c r="Q51" s="28" t="n"/>
-      <c r="R51" s="29" t="n"/>
-      <c r="S51" s="28" t="n"/>
-      <c r="T51" s="29" t="n"/>
-      <c r="U51" s="28" t="n"/>
-      <c r="V51" s="29" t="n"/>
-      <c r="W51" s="28" t="n"/>
-      <c r="X51" s="29" t="n"/>
-      <c r="Y51" s="28" t="n"/>
-      <c r="Z51" s="29" t="n"/>
-      <c r="AA51" s="28" t="n"/>
-      <c r="AB51" s="29" t="n"/>
-      <c r="AC51" s="28" t="n"/>
-      <c r="AD51" s="29" t="n"/>
+      <c r="I51" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="J51" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="K51" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="L51" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="M51" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="N51" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="O51" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="P51" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="Q51" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="R51" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="S51" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="T51" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="U51" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="V51" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="W51" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="X51" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="Y51" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="Z51" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="AA51" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="AB51" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AC51" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="AD51" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="AE51" s="10" t="n"/>
       <c r="AF51" s="10" t="n"/>
       <c r="AG51" s="10" t="n"/>
@@ -38211,7 +39948,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-43901</t>
         </is>
       </c>
-      <c r="D52" s="26" t="n"/>
+      <c r="D52" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E52" s="27" t="n"/>
       <c r="F52" s="28" t="n"/>
       <c r="G52" s="29" t="inlineStr">
@@ -38220,28 +39961,116 @@
         </is>
       </c>
       <c r="H52" s="27" t="n"/>
-      <c r="I52" s="28" t="n"/>
-      <c r="J52" s="29" t="n"/>
-      <c r="K52" s="28" t="n"/>
-      <c r="L52" s="29" t="n"/>
-      <c r="M52" s="28" t="n"/>
-      <c r="N52" s="29" t="n"/>
-      <c r="O52" s="28" t="n"/>
-      <c r="P52" s="29" t="n"/>
-      <c r="Q52" s="28" t="n"/>
-      <c r="R52" s="29" t="n"/>
-      <c r="S52" s="28" t="n"/>
-      <c r="T52" s="29" t="n"/>
-      <c r="U52" s="28" t="n"/>
-      <c r="V52" s="29" t="n"/>
-      <c r="W52" s="28" t="n"/>
-      <c r="X52" s="29" t="n"/>
-      <c r="Y52" s="28" t="n"/>
-      <c r="Z52" s="29" t="n"/>
-      <c r="AA52" s="28" t="n"/>
-      <c r="AB52" s="29" t="n"/>
-      <c r="AC52" s="28" t="n"/>
-      <c r="AD52" s="29" t="n"/>
+      <c r="I52" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="J52" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="K52" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="L52" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="M52" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="N52" s="29" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="O52" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="P52" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="Q52" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="R52" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="S52" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="T52" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="U52" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="V52" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="W52" s="28" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="X52" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="Y52" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="Z52" s="29" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="AA52" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="AB52" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AC52" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="AD52" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="AE52" s="10" t="n"/>
       <c r="AF52" s="10" t="n"/>
       <c r="AG52" s="10" t="n"/>
@@ -38274,7 +40103,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-44001</t>
         </is>
       </c>
-      <c r="D53" s="26" t="n"/>
+      <c r="D53" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E53" s="27" t="n"/>
       <c r="F53" s="28" t="n"/>
       <c r="G53" s="29" t="inlineStr">
@@ -38284,27 +40117,83 @@
       </c>
       <c r="H53" s="27" t="n"/>
       <c r="I53" s="28" t="n"/>
-      <c r="J53" s="29" t="n"/>
+      <c r="J53" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K53" s="28" t="n"/>
-      <c r="L53" s="29" t="n"/>
+      <c r="L53" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M53" s="28" t="n"/>
-      <c r="N53" s="29" t="n"/>
+      <c r="N53" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O53" s="28" t="n"/>
-      <c r="P53" s="29" t="n"/>
+      <c r="P53" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q53" s="28" t="n"/>
-      <c r="R53" s="29" t="n"/>
+      <c r="R53" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S53" s="28" t="n"/>
-      <c r="T53" s="29" t="n"/>
+      <c r="T53" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U53" s="28" t="n"/>
-      <c r="V53" s="29" t="n"/>
-      <c r="W53" s="28" t="n"/>
-      <c r="X53" s="29" t="n"/>
+      <c r="V53" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="W53" s="28" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="X53" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="Y53" s="28" t="n"/>
-      <c r="Z53" s="29" t="n"/>
-      <c r="AA53" s="28" t="n"/>
-      <c r="AB53" s="29" t="n"/>
-      <c r="AC53" s="28" t="n"/>
-      <c r="AD53" s="29" t="n"/>
+      <c r="Z53" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="AA53" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="AB53" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AC53" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="AD53" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="AE53" s="10" t="n"/>
       <c r="AF53" s="10" t="n"/>
       <c r="AG53" s="10" t="n"/>
@@ -38337,7 +40226,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-44101</t>
         </is>
       </c>
-      <c r="D54" s="26" t="n"/>
+      <c r="D54" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E54" s="27" t="n"/>
       <c r="F54" s="28" t="n"/>
       <c r="G54" s="29" t="inlineStr">
@@ -38347,27 +40240,83 @@
       </c>
       <c r="H54" s="27" t="n"/>
       <c r="I54" s="28" t="n"/>
-      <c r="J54" s="29" t="n"/>
+      <c r="J54" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K54" s="28" t="n"/>
-      <c r="L54" s="29" t="n"/>
+      <c r="L54" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M54" s="28" t="n"/>
-      <c r="N54" s="29" t="n"/>
+      <c r="N54" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O54" s="28" t="n"/>
-      <c r="P54" s="29" t="n"/>
+      <c r="P54" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q54" s="28" t="n"/>
-      <c r="R54" s="29" t="n"/>
+      <c r="R54" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S54" s="28" t="n"/>
-      <c r="T54" s="29" t="n"/>
+      <c r="T54" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U54" s="28" t="n"/>
-      <c r="V54" s="29" t="n"/>
-      <c r="W54" s="28" t="n"/>
-      <c r="X54" s="29" t="n"/>
+      <c r="V54" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="W54" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="X54" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="Y54" s="28" t="n"/>
-      <c r="Z54" s="29" t="n"/>
-      <c r="AA54" s="28" t="n"/>
-      <c r="AB54" s="29" t="n"/>
-      <c r="AC54" s="28" t="n"/>
-      <c r="AD54" s="29" t="n"/>
+      <c r="Z54" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="AA54" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="AB54" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AC54" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="AD54" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="AE54" s="10" t="n"/>
       <c r="AF54" s="10" t="n"/>
       <c r="AG54" s="10" t="n"/>
@@ -38400,7 +40349,11 @@
           <t>(no drawing number in legend)</t>
         </is>
       </c>
-      <c r="D55" s="26" t="n"/>
+      <c r="D55" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E55" s="27" t="n"/>
       <c r="F55" s="28" t="n"/>
       <c r="G55" s="29" t="inlineStr">
@@ -38410,27 +40363,75 @@
       </c>
       <c r="H55" s="27" t="n"/>
       <c r="I55" s="28" t="n"/>
-      <c r="J55" s="29" t="n"/>
+      <c r="J55" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K55" s="28" t="n"/>
-      <c r="L55" s="29" t="n"/>
+      <c r="L55" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M55" s="28" t="n"/>
-      <c r="N55" s="29" t="n"/>
+      <c r="N55" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O55" s="28" t="n"/>
-      <c r="P55" s="29" t="n"/>
+      <c r="P55" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q55" s="28" t="n"/>
-      <c r="R55" s="29" t="n"/>
+      <c r="R55" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S55" s="28" t="n"/>
-      <c r="T55" s="29" t="n"/>
+      <c r="T55" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U55" s="28" t="n"/>
-      <c r="V55" s="29" t="n"/>
-      <c r="W55" s="28" t="n"/>
-      <c r="X55" s="29" t="n"/>
+      <c r="V55" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="W55" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="X55" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="Y55" s="28" t="n"/>
-      <c r="Z55" s="29" t="n"/>
+      <c r="Z55" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA55" s="28" t="n"/>
-      <c r="AB55" s="29" t="n"/>
+      <c r="AB55" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC55" s="28" t="n"/>
-      <c r="AD55" s="29" t="n"/>
+      <c r="AD55" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE55" s="10" t="n"/>
       <c r="AF55" s="10" t="n"/>
       <c r="AG55" s="10" t="n"/>
@@ -38463,7 +40464,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-44301</t>
         </is>
       </c>
-      <c r="D56" s="26" t="n"/>
+      <c r="D56" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E56" s="27" t="n"/>
       <c r="F56" s="28" t="n"/>
       <c r="G56" s="29" t="inlineStr">
@@ -38473,27 +40478,79 @@
       </c>
       <c r="H56" s="27" t="n"/>
       <c r="I56" s="28" t="n"/>
-      <c r="J56" s="29" t="n"/>
+      <c r="J56" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K56" s="28" t="n"/>
-      <c r="L56" s="29" t="n"/>
+      <c r="L56" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M56" s="28" t="n"/>
-      <c r="N56" s="29" t="n"/>
+      <c r="N56" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O56" s="28" t="n"/>
-      <c r="P56" s="29" t="n"/>
+      <c r="P56" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q56" s="28" t="n"/>
-      <c r="R56" s="29" t="n"/>
+      <c r="R56" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S56" s="28" t="n"/>
-      <c r="T56" s="29" t="n"/>
+      <c r="T56" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U56" s="28" t="n"/>
-      <c r="V56" s="29" t="n"/>
+      <c r="V56" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W56" s="28" t="n"/>
-      <c r="X56" s="29" t="n"/>
+      <c r="X56" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y56" s="28" t="n"/>
-      <c r="Z56" s="29" t="n"/>
-      <c r="AA56" s="28" t="n"/>
-      <c r="AB56" s="29" t="n"/>
-      <c r="AC56" s="28" t="n"/>
-      <c r="AD56" s="29" t="n"/>
+      <c r="Z56" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="AA56" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="AB56" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AC56" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="AD56" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="AE56" s="10" t="n"/>
       <c r="AF56" s="10" t="n"/>
       <c r="AG56" s="10" t="n"/>
@@ -38526,7 +40583,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-44401</t>
         </is>
       </c>
-      <c r="D57" s="26" t="n"/>
+      <c r="D57" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E57" s="27" t="n"/>
       <c r="F57" s="28" t="n"/>
       <c r="G57" s="29" t="inlineStr">
@@ -38536,27 +40597,83 @@
       </c>
       <c r="H57" s="27" t="n"/>
       <c r="I57" s="28" t="n"/>
-      <c r="J57" s="29" t="n"/>
+      <c r="J57" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K57" s="28" t="n"/>
-      <c r="L57" s="29" t="n"/>
+      <c r="L57" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M57" s="28" t="n"/>
-      <c r="N57" s="29" t="n"/>
+      <c r="N57" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O57" s="28" t="n"/>
-      <c r="P57" s="29" t="n"/>
+      <c r="P57" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q57" s="28" t="n"/>
-      <c r="R57" s="29" t="n"/>
+      <c r="R57" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S57" s="28" t="n"/>
-      <c r="T57" s="29" t="n"/>
+      <c r="T57" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U57" s="28" t="n"/>
-      <c r="V57" s="29" t="n"/>
-      <c r="W57" s="28" t="n"/>
-      <c r="X57" s="29" t="n"/>
+      <c r="V57" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="W57" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="X57" s="29" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="Y57" s="28" t="n"/>
-      <c r="Z57" s="29" t="n"/>
-      <c r="AA57" s="28" t="n"/>
-      <c r="AB57" s="29" t="n"/>
-      <c r="AC57" s="28" t="n"/>
-      <c r="AD57" s="29" t="n"/>
+      <c r="Z57" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="AA57" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="AB57" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AC57" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="AD57" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="AE57" s="10" t="n"/>
       <c r="AF57" s="10" t="n"/>
       <c r="AG57" s="10" t="n"/>
@@ -38589,7 +40706,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-44501</t>
         </is>
       </c>
-      <c r="D58" s="26" t="n"/>
+      <c r="D58" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E58" s="27" t="n"/>
       <c r="F58" s="28" t="n"/>
       <c r="G58" s="29" t="inlineStr">
@@ -38599,27 +40720,87 @@
       </c>
       <c r="H58" s="27" t="n"/>
       <c r="I58" s="28" t="n"/>
-      <c r="J58" s="29" t="n"/>
+      <c r="J58" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K58" s="28" t="n"/>
-      <c r="L58" s="29" t="n"/>
-      <c r="M58" s="28" t="n"/>
-      <c r="N58" s="29" t="n"/>
+      <c r="L58" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="M58" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="N58" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="O58" s="28" t="n"/>
-      <c r="P58" s="29" t="n"/>
+      <c r="P58" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q58" s="28" t="n"/>
-      <c r="R58" s="29" t="n"/>
+      <c r="R58" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S58" s="28" t="n"/>
-      <c r="T58" s="29" t="n"/>
+      <c r="T58" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U58" s="28" t="n"/>
-      <c r="V58" s="29" t="n"/>
-      <c r="W58" s="28" t="n"/>
-      <c r="X58" s="29" t="n"/>
+      <c r="V58" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="W58" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="X58" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="Y58" s="28" t="n"/>
-      <c r="Z58" s="29" t="n"/>
-      <c r="AA58" s="28" t="n"/>
-      <c r="AB58" s="29" t="n"/>
-      <c r="AC58" s="28" t="n"/>
-      <c r="AD58" s="29" t="n"/>
+      <c r="Z58" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="AA58" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="AB58" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AC58" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="AD58" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="AE58" s="10" t="n"/>
       <c r="AF58" s="10" t="n"/>
       <c r="AG58" s="10" t="n"/>
@@ -38652,7 +40833,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-44901</t>
         </is>
       </c>
-      <c r="D59" s="26" t="n"/>
+      <c r="D59" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E59" s="27" t="n"/>
       <c r="F59" s="28" t="n"/>
       <c r="G59" s="29" t="inlineStr">
@@ -38661,28 +40846,116 @@
         </is>
       </c>
       <c r="H59" s="27" t="n"/>
-      <c r="I59" s="28" t="n"/>
-      <c r="J59" s="29" t="n"/>
-      <c r="K59" s="28" t="n"/>
-      <c r="L59" s="29" t="n"/>
-      <c r="M59" s="28" t="n"/>
-      <c r="N59" s="29" t="n"/>
-      <c r="O59" s="28" t="n"/>
-      <c r="P59" s="29" t="n"/>
-      <c r="Q59" s="28" t="n"/>
-      <c r="R59" s="29" t="n"/>
-      <c r="S59" s="28" t="n"/>
-      <c r="T59" s="29" t="n"/>
-      <c r="U59" s="28" t="n"/>
-      <c r="V59" s="29" t="n"/>
-      <c r="W59" s="28" t="n"/>
-      <c r="X59" s="29" t="n"/>
-      <c r="Y59" s="28" t="n"/>
-      <c r="Z59" s="29" t="n"/>
-      <c r="AA59" s="28" t="n"/>
-      <c r="AB59" s="29" t="n"/>
-      <c r="AC59" s="28" t="n"/>
-      <c r="AD59" s="29" t="n"/>
+      <c r="I59" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="J59" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K59" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="L59" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="M59" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="N59" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="O59" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="P59" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="Q59" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="R59" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="S59" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="T59" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="U59" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="V59" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="W59" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="X59" s="29" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Y59" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="Z59" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AA59" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="AB59" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AC59" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="AD59" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="AE59" s="10" t="n"/>
       <c r="AF59" s="10" t="n"/>
       <c r="AG59" s="10" t="n"/>
@@ -38715,7 +40988,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-44601</t>
         </is>
       </c>
-      <c r="D60" s="26" t="n"/>
+      <c r="D60" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E60" s="27" t="n"/>
       <c r="F60" s="28" t="n"/>
       <c r="G60" s="29" t="inlineStr">
@@ -38725,27 +41002,83 @@
       </c>
       <c r="H60" s="27" t="n"/>
       <c r="I60" s="28" t="n"/>
-      <c r="J60" s="29" t="n"/>
+      <c r="J60" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K60" s="28" t="n"/>
-      <c r="L60" s="29" t="n"/>
+      <c r="L60" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M60" s="28" t="n"/>
-      <c r="N60" s="29" t="n"/>
+      <c r="N60" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O60" s="28" t="n"/>
-      <c r="P60" s="29" t="n"/>
+      <c r="P60" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q60" s="28" t="n"/>
-      <c r="R60" s="29" t="n"/>
+      <c r="R60" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S60" s="28" t="n"/>
-      <c r="T60" s="29" t="n"/>
+      <c r="T60" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U60" s="28" t="n"/>
-      <c r="V60" s="29" t="n"/>
-      <c r="W60" s="28" t="n"/>
-      <c r="X60" s="29" t="n"/>
+      <c r="V60" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="W60" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="X60" s="29" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="Y60" s="28" t="n"/>
-      <c r="Z60" s="29" t="n"/>
-      <c r="AA60" s="28" t="n"/>
-      <c r="AB60" s="29" t="n"/>
-      <c r="AC60" s="28" t="n"/>
-      <c r="AD60" s="29" t="n"/>
+      <c r="Z60" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="AA60" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="AB60" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AC60" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="AD60" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="AE60" s="10" t="n"/>
       <c r="AF60" s="10" t="n"/>
       <c r="AG60" s="10" t="n"/>
@@ -38778,7 +41111,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-44701</t>
         </is>
       </c>
-      <c r="D61" s="26" t="n"/>
+      <c r="D61" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E61" s="27" t="n"/>
       <c r="F61" s="28" t="n"/>
       <c r="G61" s="29" t="inlineStr">
@@ -38788,27 +41125,79 @@
       </c>
       <c r="H61" s="27" t="n"/>
       <c r="I61" s="28" t="n"/>
-      <c r="J61" s="29" t="n"/>
+      <c r="J61" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K61" s="28" t="n"/>
-      <c r="L61" s="29" t="n"/>
+      <c r="L61" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M61" s="28" t="n"/>
-      <c r="N61" s="29" t="n"/>
+      <c r="N61" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O61" s="28" t="n"/>
-      <c r="P61" s="29" t="n"/>
+      <c r="P61" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q61" s="28" t="n"/>
-      <c r="R61" s="29" t="n"/>
+      <c r="R61" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S61" s="28" t="n"/>
-      <c r="T61" s="29" t="n"/>
+      <c r="T61" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U61" s="28" t="n"/>
-      <c r="V61" s="29" t="n"/>
+      <c r="V61" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W61" s="28" t="n"/>
-      <c r="X61" s="29" t="n"/>
+      <c r="X61" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y61" s="28" t="n"/>
-      <c r="Z61" s="29" t="n"/>
-      <c r="AA61" s="28" t="n"/>
-      <c r="AB61" s="29" t="n"/>
-      <c r="AC61" s="28" t="n"/>
-      <c r="AD61" s="29" t="n"/>
+      <c r="Z61" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="AA61" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="AB61" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AC61" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="AD61" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="AE61" s="10" t="n"/>
       <c r="AF61" s="10" t="n"/>
       <c r="AG61" s="10" t="n"/>
@@ -38841,7 +41230,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-44801</t>
         </is>
       </c>
-      <c r="D62" s="26" t="n"/>
+      <c r="D62" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E62" s="27" t="n"/>
       <c r="F62" s="28" t="n"/>
       <c r="G62" s="29" t="inlineStr">
@@ -38851,27 +41244,79 @@
       </c>
       <c r="H62" s="27" t="n"/>
       <c r="I62" s="28" t="n"/>
-      <c r="J62" s="29" t="n"/>
+      <c r="J62" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K62" s="28" t="n"/>
-      <c r="L62" s="29" t="n"/>
+      <c r="L62" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M62" s="28" t="n"/>
-      <c r="N62" s="29" t="n"/>
+      <c r="N62" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O62" s="28" t="n"/>
-      <c r="P62" s="29" t="n"/>
+      <c r="P62" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q62" s="28" t="n"/>
-      <c r="R62" s="29" t="n"/>
+      <c r="R62" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S62" s="28" t="n"/>
-      <c r="T62" s="29" t="n"/>
+      <c r="T62" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U62" s="28" t="n"/>
-      <c r="V62" s="29" t="n"/>
+      <c r="V62" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W62" s="28" t="n"/>
-      <c r="X62" s="29" t="n"/>
+      <c r="X62" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y62" s="28" t="n"/>
-      <c r="Z62" s="29" t="n"/>
-      <c r="AA62" s="28" t="n"/>
-      <c r="AB62" s="29" t="n"/>
-      <c r="AC62" s="28" t="n"/>
-      <c r="AD62" s="29" t="n"/>
+      <c r="Z62" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="AA62" s="28" t="inlineStr">
+        <is>
+          <t>00</t>
+        </is>
+      </c>
+      <c r="AB62" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AC62" s="28" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="AD62" s="29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="AE62" s="10" t="n"/>
       <c r="AF62" s="10" t="n"/>
       <c r="AG62" s="10" t="n"/>

</xml_diff>

<commit_message>
Add FLS (Fire Life & Safety) per level: Civil and MEP items; shown on level page after room list
</commit_message>
<xml_diff>
--- a/WPH_Room_Register.xlsx
+++ b/WPH_Room_Register.xlsx
@@ -10,10 +10,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clearances" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shop Drawings" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fields" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FLS" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fields" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Clearances'!$A$1:$M$554</definedName>
@@ -30,7 +31,7 @@
     <numFmt numFmtId="165" formatCode="dd\-mmm\-yyyy"/>
     <numFmt numFmtId="166" formatCode="dd-mmm-yyyy"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -89,6 +90,11 @@
     </font>
     <font>
       <color rgb="FF000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF1F3A5F"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -189,7 +195,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -263,6 +269,7 @@
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -663,7 +670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A37"/>
+  <dimension ref="A1:A40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -884,6 +891,20 @@
       <c r="A37" s="9" t="inlineStr">
         <is>
           <t>A / B = Approved / Approved as Noted (dark green)  |  UR = Under Review (amber)  |  C = Revise &amp; Resubmit (red)  |  TBS = To Be Submitted (grey). Codes, colours and meanings are defined in the Lists sheet and are used by both Excel and the QR pages. When the Coordination Sketch is "Provided", every MEP/ELV item that is not A/B is shown as "Coordinated" (light green); A/B approvals always show dark green.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="31" t="inlineStr">
+        <is>
+          <t>FLS – FIRE LIFE &amp; SAFETY (FLS sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="9" t="inlineStr">
+        <is>
+          <t>One row per tower/level. Civil: Steel Doors, Wooden Doors, Fire Sealant, Hardware. MEP: Fire Sealant, Fire Alarm, Fire Fighting. Use the same codes A / B / UR / C / TBS and a date. Shown on the LEVEL QR page after the room list.</t>
         </is>
       </c>
     </row>
@@ -41564,6 +41585,1049 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:AF18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="45" customHeight="1">
+      <c r="A1" s="23" t="inlineStr">
+        <is>
+          <t>Tower</t>
+        </is>
+      </c>
+      <c r="B1" s="23" t="inlineStr">
+        <is>
+          <t>Level</t>
+        </is>
+      </c>
+      <c r="C1" s="23" t="inlineStr">
+        <is>
+          <t>Level Code</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Civil - Steel Doors</t>
+        </is>
+      </c>
+      <c r="E1" s="24" t="inlineStr">
+        <is>
+          <t>Civil - Steel Doors Date</t>
+        </is>
+      </c>
+      <c r="F1" s="24" t="inlineStr">
+        <is>
+          <t>Civil - Wooden Doors</t>
+        </is>
+      </c>
+      <c r="G1" s="24" t="inlineStr">
+        <is>
+          <t>Civil - Wooden Doors Date</t>
+        </is>
+      </c>
+      <c r="H1" s="24" t="inlineStr">
+        <is>
+          <t>Civil - Fire Sealant</t>
+        </is>
+      </c>
+      <c r="I1" s="24" t="inlineStr">
+        <is>
+          <t>Civil - Fire Sealant Date</t>
+        </is>
+      </c>
+      <c r="J1" s="24" t="inlineStr">
+        <is>
+          <t>Civil - Hardware</t>
+        </is>
+      </c>
+      <c r="K1" s="24" t="inlineStr">
+        <is>
+          <t>Civil - Hardware Date</t>
+        </is>
+      </c>
+      <c r="L1" s="24" t="inlineStr">
+        <is>
+          <t>MEP - Fire Sealant</t>
+        </is>
+      </c>
+      <c r="M1" s="24" t="inlineStr">
+        <is>
+          <t>MEP - Fire Sealant Date</t>
+        </is>
+      </c>
+      <c r="N1" s="24" t="inlineStr">
+        <is>
+          <t>MEP - Fire Alarm</t>
+        </is>
+      </c>
+      <c r="O1" s="24" t="inlineStr">
+        <is>
+          <t>MEP - Fire Alarm Date</t>
+        </is>
+      </c>
+      <c r="P1" s="24" t="inlineStr">
+        <is>
+          <t>MEP - Fire Fighting</t>
+        </is>
+      </c>
+      <c r="Q1" s="24" t="inlineStr">
+        <is>
+          <t>MEP - Fire Fighting Date</t>
+        </is>
+      </c>
+      <c r="R1" s="10" t="n"/>
+      <c r="S1" s="10" t="n"/>
+      <c r="T1" s="10" t="n"/>
+      <c r="U1" s="10" t="n"/>
+      <c r="V1" s="10" t="n"/>
+      <c r="W1" s="10" t="n"/>
+      <c r="X1" s="10" t="n"/>
+      <c r="Y1" s="10" t="n"/>
+      <c r="Z1" s="10" t="n"/>
+      <c r="AA1" s="10" t="n"/>
+      <c r="AB1" s="10" t="n"/>
+      <c r="AC1" s="10" t="n"/>
+      <c r="AD1" s="10" t="n"/>
+      <c r="AE1" s="10" t="n"/>
+      <c r="AF1" s="10" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="25" t="inlineStr">
+        <is>
+          <t>Tower A</t>
+        </is>
+      </c>
+      <c r="B2" s="25" t="inlineStr">
+        <is>
+          <t>L02</t>
+        </is>
+      </c>
+      <c r="C2" s="25" t="inlineStr">
+        <is>
+          <t>AL02</t>
+        </is>
+      </c>
+      <c r="D2" s="29" t="n"/>
+      <c r="E2" s="27" t="n"/>
+      <c r="F2" s="29" t="n"/>
+      <c r="G2" s="27" t="n"/>
+      <c r="H2" s="29" t="n"/>
+      <c r="I2" s="27" t="n"/>
+      <c r="J2" s="29" t="n"/>
+      <c r="K2" s="27" t="n"/>
+      <c r="L2" s="29" t="n"/>
+      <c r="M2" s="27" t="n"/>
+      <c r="N2" s="29" t="n"/>
+      <c r="O2" s="27" t="n"/>
+      <c r="P2" s="29" t="n"/>
+      <c r="Q2" s="27" t="n"/>
+      <c r="R2" s="10" t="n"/>
+      <c r="S2" s="10" t="n"/>
+      <c r="T2" s="10" t="n"/>
+      <c r="U2" s="10" t="n"/>
+      <c r="V2" s="10" t="n"/>
+      <c r="W2" s="10" t="n"/>
+      <c r="X2" s="10" t="n"/>
+      <c r="Y2" s="10" t="n"/>
+      <c r="Z2" s="10" t="n"/>
+      <c r="AA2" s="10" t="n"/>
+      <c r="AB2" s="10" t="n"/>
+      <c r="AC2" s="10" t="n"/>
+      <c r="AD2" s="10" t="n"/>
+      <c r="AE2" s="10" t="n"/>
+      <c r="AF2" s="10" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="25" t="inlineStr">
+        <is>
+          <t>Tower A</t>
+        </is>
+      </c>
+      <c r="B3" s="25" t="inlineStr">
+        <is>
+          <t>L03</t>
+        </is>
+      </c>
+      <c r="C3" s="25" t="inlineStr">
+        <is>
+          <t>AL03</t>
+        </is>
+      </c>
+      <c r="D3" s="29" t="n"/>
+      <c r="E3" s="27" t="n"/>
+      <c r="F3" s="29" t="n"/>
+      <c r="G3" s="27" t="n"/>
+      <c r="H3" s="29" t="n"/>
+      <c r="I3" s="27" t="n"/>
+      <c r="J3" s="29" t="n"/>
+      <c r="K3" s="27" t="n"/>
+      <c r="L3" s="29" t="n"/>
+      <c r="M3" s="27" t="n"/>
+      <c r="N3" s="29" t="n"/>
+      <c r="O3" s="27" t="n"/>
+      <c r="P3" s="29" t="n"/>
+      <c r="Q3" s="27" t="n"/>
+      <c r="R3" s="10" t="n"/>
+      <c r="S3" s="10" t="n"/>
+      <c r="T3" s="10" t="n"/>
+      <c r="U3" s="10" t="n"/>
+      <c r="V3" s="10" t="n"/>
+      <c r="W3" s="10" t="n"/>
+      <c r="X3" s="10" t="n"/>
+      <c r="Y3" s="10" t="n"/>
+      <c r="Z3" s="10" t="n"/>
+      <c r="AA3" s="10" t="n"/>
+      <c r="AB3" s="10" t="n"/>
+      <c r="AC3" s="10" t="n"/>
+      <c r="AD3" s="10" t="n"/>
+      <c r="AE3" s="10" t="n"/>
+      <c r="AF3" s="10" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="25" t="inlineStr">
+        <is>
+          <t>Tower A</t>
+        </is>
+      </c>
+      <c r="B4" s="25" t="inlineStr">
+        <is>
+          <t>L04</t>
+        </is>
+      </c>
+      <c r="C4" s="25" t="inlineStr">
+        <is>
+          <t>AL04</t>
+        </is>
+      </c>
+      <c r="D4" s="29" t="n"/>
+      <c r="E4" s="27" t="n"/>
+      <c r="F4" s="29" t="n"/>
+      <c r="G4" s="27" t="n"/>
+      <c r="H4" s="29" t="n"/>
+      <c r="I4" s="27" t="n"/>
+      <c r="J4" s="29" t="n"/>
+      <c r="K4" s="27" t="n"/>
+      <c r="L4" s="29" t="n"/>
+      <c r="M4" s="27" t="n"/>
+      <c r="N4" s="29" t="n"/>
+      <c r="O4" s="27" t="n"/>
+      <c r="P4" s="29" t="n"/>
+      <c r="Q4" s="27" t="n"/>
+      <c r="R4" s="10" t="n"/>
+      <c r="S4" s="10" t="n"/>
+      <c r="T4" s="10" t="n"/>
+      <c r="U4" s="10" t="n"/>
+      <c r="V4" s="10" t="n"/>
+      <c r="W4" s="10" t="n"/>
+      <c r="X4" s="10" t="n"/>
+      <c r="Y4" s="10" t="n"/>
+      <c r="Z4" s="10" t="n"/>
+      <c r="AA4" s="10" t="n"/>
+      <c r="AB4" s="10" t="n"/>
+      <c r="AC4" s="10" t="n"/>
+      <c r="AD4" s="10" t="n"/>
+      <c r="AE4" s="10" t="n"/>
+      <c r="AF4" s="10" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="25" t="inlineStr">
+        <is>
+          <t>Tower A</t>
+        </is>
+      </c>
+      <c r="B5" s="25" t="inlineStr">
+        <is>
+          <t>L05</t>
+        </is>
+      </c>
+      <c r="C5" s="25" t="inlineStr">
+        <is>
+          <t>AL05</t>
+        </is>
+      </c>
+      <c r="D5" s="29" t="n"/>
+      <c r="E5" s="27" t="n"/>
+      <c r="F5" s="29" t="n"/>
+      <c r="G5" s="27" t="n"/>
+      <c r="H5" s="29" t="n"/>
+      <c r="I5" s="27" t="n"/>
+      <c r="J5" s="29" t="n"/>
+      <c r="K5" s="27" t="n"/>
+      <c r="L5" s="29" t="n"/>
+      <c r="M5" s="27" t="n"/>
+      <c r="N5" s="29" t="n"/>
+      <c r="O5" s="27" t="n"/>
+      <c r="P5" s="29" t="n"/>
+      <c r="Q5" s="27" t="n"/>
+      <c r="R5" s="10" t="n"/>
+      <c r="S5" s="10" t="n"/>
+      <c r="T5" s="10" t="n"/>
+      <c r="U5" s="10" t="n"/>
+      <c r="V5" s="10" t="n"/>
+      <c r="W5" s="10" t="n"/>
+      <c r="X5" s="10" t="n"/>
+      <c r="Y5" s="10" t="n"/>
+      <c r="Z5" s="10" t="n"/>
+      <c r="AA5" s="10" t="n"/>
+      <c r="AB5" s="10" t="n"/>
+      <c r="AC5" s="10" t="n"/>
+      <c r="AD5" s="10" t="n"/>
+      <c r="AE5" s="10" t="n"/>
+      <c r="AF5" s="10" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="25" t="inlineStr">
+        <is>
+          <t>Tower A</t>
+        </is>
+      </c>
+      <c r="B6" s="25" t="inlineStr">
+        <is>
+          <t>L06</t>
+        </is>
+      </c>
+      <c r="C6" s="25" t="inlineStr">
+        <is>
+          <t>AL06</t>
+        </is>
+      </c>
+      <c r="D6" s="29" t="n"/>
+      <c r="E6" s="27" t="n"/>
+      <c r="F6" s="29" t="n"/>
+      <c r="G6" s="27" t="n"/>
+      <c r="H6" s="29" t="n"/>
+      <c r="I6" s="27" t="n"/>
+      <c r="J6" s="29" t="n"/>
+      <c r="K6" s="27" t="n"/>
+      <c r="L6" s="29" t="n"/>
+      <c r="M6" s="27" t="n"/>
+      <c r="N6" s="29" t="n"/>
+      <c r="O6" s="27" t="n"/>
+      <c r="P6" s="29" t="n"/>
+      <c r="Q6" s="27" t="n"/>
+      <c r="R6" s="10" t="n"/>
+      <c r="S6" s="10" t="n"/>
+      <c r="T6" s="10" t="n"/>
+      <c r="U6" s="10" t="n"/>
+      <c r="V6" s="10" t="n"/>
+      <c r="W6" s="10" t="n"/>
+      <c r="X6" s="10" t="n"/>
+      <c r="Y6" s="10" t="n"/>
+      <c r="Z6" s="10" t="n"/>
+      <c r="AA6" s="10" t="n"/>
+      <c r="AB6" s="10" t="n"/>
+      <c r="AC6" s="10" t="n"/>
+      <c r="AD6" s="10" t="n"/>
+      <c r="AE6" s="10" t="n"/>
+      <c r="AF6" s="10" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="25" t="inlineStr">
+        <is>
+          <t>Tower A</t>
+        </is>
+      </c>
+      <c r="B7" s="25" t="inlineStr">
+        <is>
+          <t>L07</t>
+        </is>
+      </c>
+      <c r="C7" s="25" t="inlineStr">
+        <is>
+          <t>AL07</t>
+        </is>
+      </c>
+      <c r="D7" s="29" t="n"/>
+      <c r="E7" s="27" t="n"/>
+      <c r="F7" s="29" t="n"/>
+      <c r="G7" s="27" t="n"/>
+      <c r="H7" s="29" t="n"/>
+      <c r="I7" s="27" t="n"/>
+      <c r="J7" s="29" t="n"/>
+      <c r="K7" s="27" t="n"/>
+      <c r="L7" s="29" t="n"/>
+      <c r="M7" s="27" t="n"/>
+      <c r="N7" s="29" t="n"/>
+      <c r="O7" s="27" t="n"/>
+      <c r="P7" s="29" t="n"/>
+      <c r="Q7" s="27" t="n"/>
+      <c r="R7" s="10" t="n"/>
+      <c r="S7" s="10" t="n"/>
+      <c r="T7" s="10" t="n"/>
+      <c r="U7" s="10" t="n"/>
+      <c r="V7" s="10" t="n"/>
+      <c r="W7" s="10" t="n"/>
+      <c r="X7" s="10" t="n"/>
+      <c r="Y7" s="10" t="n"/>
+      <c r="Z7" s="10" t="n"/>
+      <c r="AA7" s="10" t="n"/>
+      <c r="AB7" s="10" t="n"/>
+      <c r="AC7" s="10" t="n"/>
+      <c r="AD7" s="10" t="n"/>
+      <c r="AE7" s="10" t="n"/>
+      <c r="AF7" s="10" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="25" t="inlineStr">
+        <is>
+          <t>Tower A</t>
+        </is>
+      </c>
+      <c r="B8" s="25" t="inlineStr">
+        <is>
+          <t>L08</t>
+        </is>
+      </c>
+      <c r="C8" s="25" t="inlineStr">
+        <is>
+          <t>AL08</t>
+        </is>
+      </c>
+      <c r="D8" s="29" t="n"/>
+      <c r="E8" s="27" t="n"/>
+      <c r="F8" s="29" t="n"/>
+      <c r="G8" s="27" t="n"/>
+      <c r="H8" s="29" t="n"/>
+      <c r="I8" s="27" t="n"/>
+      <c r="J8" s="29" t="n"/>
+      <c r="K8" s="27" t="n"/>
+      <c r="L8" s="29" t="n"/>
+      <c r="M8" s="27" t="n"/>
+      <c r="N8" s="29" t="n"/>
+      <c r="O8" s="27" t="n"/>
+      <c r="P8" s="29" t="n"/>
+      <c r="Q8" s="27" t="n"/>
+      <c r="R8" s="10" t="n"/>
+      <c r="S8" s="10" t="n"/>
+      <c r="T8" s="10" t="n"/>
+      <c r="U8" s="10" t="n"/>
+      <c r="V8" s="10" t="n"/>
+      <c r="W8" s="10" t="n"/>
+      <c r="X8" s="10" t="n"/>
+      <c r="Y8" s="10" t="n"/>
+      <c r="Z8" s="10" t="n"/>
+      <c r="AA8" s="10" t="n"/>
+      <c r="AB8" s="10" t="n"/>
+      <c r="AC8" s="10" t="n"/>
+      <c r="AD8" s="10" t="n"/>
+      <c r="AE8" s="10" t="n"/>
+      <c r="AF8" s="10" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="25" t="inlineStr">
+        <is>
+          <t>Tower A</t>
+        </is>
+      </c>
+      <c r="B9" s="25" t="inlineStr">
+        <is>
+          <t>L09</t>
+        </is>
+      </c>
+      <c r="C9" s="25" t="inlineStr">
+        <is>
+          <t>AL09</t>
+        </is>
+      </c>
+      <c r="D9" s="29" t="n"/>
+      <c r="E9" s="27" t="n"/>
+      <c r="F9" s="29" t="n"/>
+      <c r="G9" s="27" t="n"/>
+      <c r="H9" s="29" t="n"/>
+      <c r="I9" s="27" t="n"/>
+      <c r="J9" s="29" t="n"/>
+      <c r="K9" s="27" t="n"/>
+      <c r="L9" s="29" t="n"/>
+      <c r="M9" s="27" t="n"/>
+      <c r="N9" s="29" t="n"/>
+      <c r="O9" s="27" t="n"/>
+      <c r="P9" s="29" t="n"/>
+      <c r="Q9" s="27" t="n"/>
+      <c r="R9" s="10" t="n"/>
+      <c r="S9" s="10" t="n"/>
+      <c r="T9" s="10" t="n"/>
+      <c r="U9" s="10" t="n"/>
+      <c r="V9" s="10" t="n"/>
+      <c r="W9" s="10" t="n"/>
+      <c r="X9" s="10" t="n"/>
+      <c r="Y9" s="10" t="n"/>
+      <c r="Z9" s="10" t="n"/>
+      <c r="AA9" s="10" t="n"/>
+      <c r="AB9" s="10" t="n"/>
+      <c r="AC9" s="10" t="n"/>
+      <c r="AD9" s="10" t="n"/>
+      <c r="AE9" s="10" t="n"/>
+      <c r="AF9" s="10" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="25" t="inlineStr">
+        <is>
+          <t>Tower B</t>
+        </is>
+      </c>
+      <c r="B10" s="25" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="C10" s="25" t="inlineStr">
+        <is>
+          <t>BL01</t>
+        </is>
+      </c>
+      <c r="D10" s="29" t="n"/>
+      <c r="E10" s="27" t="n"/>
+      <c r="F10" s="29" t="n"/>
+      <c r="G10" s="27" t="n"/>
+      <c r="H10" s="29" t="n"/>
+      <c r="I10" s="27" t="n"/>
+      <c r="J10" s="29" t="n"/>
+      <c r="K10" s="27" t="n"/>
+      <c r="L10" s="29" t="n"/>
+      <c r="M10" s="27" t="n"/>
+      <c r="N10" s="29" t="n"/>
+      <c r="O10" s="27" t="n"/>
+      <c r="P10" s="29" t="n"/>
+      <c r="Q10" s="27" t="n"/>
+      <c r="R10" s="10" t="n"/>
+      <c r="S10" s="10" t="n"/>
+      <c r="T10" s="10" t="n"/>
+      <c r="U10" s="10" t="n"/>
+      <c r="V10" s="10" t="n"/>
+      <c r="W10" s="10" t="n"/>
+      <c r="X10" s="10" t="n"/>
+      <c r="Y10" s="10" t="n"/>
+      <c r="Z10" s="10" t="n"/>
+      <c r="AA10" s="10" t="n"/>
+      <c r="AB10" s="10" t="n"/>
+      <c r="AC10" s="10" t="n"/>
+      <c r="AD10" s="10" t="n"/>
+      <c r="AE10" s="10" t="n"/>
+      <c r="AF10" s="10" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="25" t="inlineStr">
+        <is>
+          <t>Tower B</t>
+        </is>
+      </c>
+      <c r="B11" s="25" t="inlineStr">
+        <is>
+          <t>L02</t>
+        </is>
+      </c>
+      <c r="C11" s="25" t="inlineStr">
+        <is>
+          <t>BL02</t>
+        </is>
+      </c>
+      <c r="D11" s="29" t="n"/>
+      <c r="E11" s="27" t="n"/>
+      <c r="F11" s="29" t="n"/>
+      <c r="G11" s="27" t="n"/>
+      <c r="H11" s="29" t="n"/>
+      <c r="I11" s="27" t="n"/>
+      <c r="J11" s="29" t="n"/>
+      <c r="K11" s="27" t="n"/>
+      <c r="L11" s="29" t="n"/>
+      <c r="M11" s="27" t="n"/>
+      <c r="N11" s="29" t="n"/>
+      <c r="O11" s="27" t="n"/>
+      <c r="P11" s="29" t="n"/>
+      <c r="Q11" s="27" t="n"/>
+      <c r="R11" s="10" t="n"/>
+      <c r="S11" s="10" t="n"/>
+      <c r="T11" s="10" t="n"/>
+      <c r="U11" s="10" t="n"/>
+      <c r="V11" s="10" t="n"/>
+      <c r="W11" s="10" t="n"/>
+      <c r="X11" s="10" t="n"/>
+      <c r="Y11" s="10" t="n"/>
+      <c r="Z11" s="10" t="n"/>
+      <c r="AA11" s="10" t="n"/>
+      <c r="AB11" s="10" t="n"/>
+      <c r="AC11" s="10" t="n"/>
+      <c r="AD11" s="10" t="n"/>
+      <c r="AE11" s="10" t="n"/>
+      <c r="AF11" s="10" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="25" t="inlineStr">
+        <is>
+          <t>Tower B</t>
+        </is>
+      </c>
+      <c r="B12" s="25" t="inlineStr">
+        <is>
+          <t>L03</t>
+        </is>
+      </c>
+      <c r="C12" s="25" t="inlineStr">
+        <is>
+          <t>BL03</t>
+        </is>
+      </c>
+      <c r="D12" s="29" t="n"/>
+      <c r="E12" s="27" t="n"/>
+      <c r="F12" s="29" t="n"/>
+      <c r="G12" s="27" t="n"/>
+      <c r="H12" s="29" t="n"/>
+      <c r="I12" s="27" t="n"/>
+      <c r="J12" s="29" t="n"/>
+      <c r="K12" s="27" t="n"/>
+      <c r="L12" s="29" t="n"/>
+      <c r="M12" s="27" t="n"/>
+      <c r="N12" s="29" t="n"/>
+      <c r="O12" s="27" t="n"/>
+      <c r="P12" s="29" t="n"/>
+      <c r="Q12" s="27" t="n"/>
+      <c r="R12" s="10" t="n"/>
+      <c r="S12" s="10" t="n"/>
+      <c r="T12" s="10" t="n"/>
+      <c r="U12" s="10" t="n"/>
+      <c r="V12" s="10" t="n"/>
+      <c r="W12" s="10" t="n"/>
+      <c r="X12" s="10" t="n"/>
+      <c r="Y12" s="10" t="n"/>
+      <c r="Z12" s="10" t="n"/>
+      <c r="AA12" s="10" t="n"/>
+      <c r="AB12" s="10" t="n"/>
+      <c r="AC12" s="10" t="n"/>
+      <c r="AD12" s="10" t="n"/>
+      <c r="AE12" s="10" t="n"/>
+      <c r="AF12" s="10" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="25" t="inlineStr">
+        <is>
+          <t>Tower B</t>
+        </is>
+      </c>
+      <c r="B13" s="25" t="inlineStr">
+        <is>
+          <t>L04</t>
+        </is>
+      </c>
+      <c r="C13" s="25" t="inlineStr">
+        <is>
+          <t>BL04</t>
+        </is>
+      </c>
+      <c r="D13" s="29" t="n"/>
+      <c r="E13" s="27" t="n"/>
+      <c r="F13" s="29" t="n"/>
+      <c r="G13" s="27" t="n"/>
+      <c r="H13" s="29" t="n"/>
+      <c r="I13" s="27" t="n"/>
+      <c r="J13" s="29" t="n"/>
+      <c r="K13" s="27" t="n"/>
+      <c r="L13" s="29" t="n"/>
+      <c r="M13" s="27" t="n"/>
+      <c r="N13" s="29" t="n"/>
+      <c r="O13" s="27" t="n"/>
+      <c r="P13" s="29" t="n"/>
+      <c r="Q13" s="27" t="n"/>
+      <c r="R13" s="10" t="n"/>
+      <c r="S13" s="10" t="n"/>
+      <c r="T13" s="10" t="n"/>
+      <c r="U13" s="10" t="n"/>
+      <c r="V13" s="10" t="n"/>
+      <c r="W13" s="10" t="n"/>
+      <c r="X13" s="10" t="n"/>
+      <c r="Y13" s="10" t="n"/>
+      <c r="Z13" s="10" t="n"/>
+      <c r="AA13" s="10" t="n"/>
+      <c r="AB13" s="10" t="n"/>
+      <c r="AC13" s="10" t="n"/>
+      <c r="AD13" s="10" t="n"/>
+      <c r="AE13" s="10" t="n"/>
+      <c r="AF13" s="10" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="25" t="inlineStr">
+        <is>
+          <t>Tower B</t>
+        </is>
+      </c>
+      <c r="B14" s="25" t="inlineStr">
+        <is>
+          <t>L05</t>
+        </is>
+      </c>
+      <c r="C14" s="25" t="inlineStr">
+        <is>
+          <t>BL05</t>
+        </is>
+      </c>
+      <c r="D14" s="29" t="n"/>
+      <c r="E14" s="27" t="n"/>
+      <c r="F14" s="29" t="n"/>
+      <c r="G14" s="27" t="n"/>
+      <c r="H14" s="29" t="n"/>
+      <c r="I14" s="27" t="n"/>
+      <c r="J14" s="29" t="n"/>
+      <c r="K14" s="27" t="n"/>
+      <c r="L14" s="29" t="n"/>
+      <c r="M14" s="27" t="n"/>
+      <c r="N14" s="29" t="n"/>
+      <c r="O14" s="27" t="n"/>
+      <c r="P14" s="29" t="n"/>
+      <c r="Q14" s="27" t="n"/>
+      <c r="R14" s="10" t="n"/>
+      <c r="S14" s="10" t="n"/>
+      <c r="T14" s="10" t="n"/>
+      <c r="U14" s="10" t="n"/>
+      <c r="V14" s="10" t="n"/>
+      <c r="W14" s="10" t="n"/>
+      <c r="X14" s="10" t="n"/>
+      <c r="Y14" s="10" t="n"/>
+      <c r="Z14" s="10" t="n"/>
+      <c r="AA14" s="10" t="n"/>
+      <c r="AB14" s="10" t="n"/>
+      <c r="AC14" s="10" t="n"/>
+      <c r="AD14" s="10" t="n"/>
+      <c r="AE14" s="10" t="n"/>
+      <c r="AF14" s="10" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="25" t="inlineStr">
+        <is>
+          <t>Tower B</t>
+        </is>
+      </c>
+      <c r="B15" s="25" t="inlineStr">
+        <is>
+          <t>L06</t>
+        </is>
+      </c>
+      <c r="C15" s="25" t="inlineStr">
+        <is>
+          <t>BL06</t>
+        </is>
+      </c>
+      <c r="D15" s="29" t="n"/>
+      <c r="E15" s="27" t="n"/>
+      <c r="F15" s="29" t="n"/>
+      <c r="G15" s="27" t="n"/>
+      <c r="H15" s="29" t="n"/>
+      <c r="I15" s="27" t="n"/>
+      <c r="J15" s="29" t="n"/>
+      <c r="K15" s="27" t="n"/>
+      <c r="L15" s="29" t="n"/>
+      <c r="M15" s="27" t="n"/>
+      <c r="N15" s="29" t="n"/>
+      <c r="O15" s="27" t="n"/>
+      <c r="P15" s="29" t="n"/>
+      <c r="Q15" s="27" t="n"/>
+      <c r="R15" s="10" t="n"/>
+      <c r="S15" s="10" t="n"/>
+      <c r="T15" s="10" t="n"/>
+      <c r="U15" s="10" t="n"/>
+      <c r="V15" s="10" t="n"/>
+      <c r="W15" s="10" t="n"/>
+      <c r="X15" s="10" t="n"/>
+      <c r="Y15" s="10" t="n"/>
+      <c r="Z15" s="10" t="n"/>
+      <c r="AA15" s="10" t="n"/>
+      <c r="AB15" s="10" t="n"/>
+      <c r="AC15" s="10" t="n"/>
+      <c r="AD15" s="10" t="n"/>
+      <c r="AE15" s="10" t="n"/>
+      <c r="AF15" s="10" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="25" t="inlineStr">
+        <is>
+          <t>Tower B</t>
+        </is>
+      </c>
+      <c r="B16" s="25" t="inlineStr">
+        <is>
+          <t>L07</t>
+        </is>
+      </c>
+      <c r="C16" s="25" t="inlineStr">
+        <is>
+          <t>BL07</t>
+        </is>
+      </c>
+      <c r="D16" s="29" t="n"/>
+      <c r="E16" s="27" t="n"/>
+      <c r="F16" s="29" t="n"/>
+      <c r="G16" s="27" t="n"/>
+      <c r="H16" s="29" t="n"/>
+      <c r="I16" s="27" t="n"/>
+      <c r="J16" s="29" t="n"/>
+      <c r="K16" s="27" t="n"/>
+      <c r="L16" s="29" t="n"/>
+      <c r="M16" s="27" t="n"/>
+      <c r="N16" s="29" t="n"/>
+      <c r="O16" s="27" t="n"/>
+      <c r="P16" s="29" t="n"/>
+      <c r="Q16" s="27" t="n"/>
+      <c r="R16" s="10" t="n"/>
+      <c r="S16" s="10" t="n"/>
+      <c r="T16" s="10" t="n"/>
+      <c r="U16" s="10" t="n"/>
+      <c r="V16" s="10" t="n"/>
+      <c r="W16" s="10" t="n"/>
+      <c r="X16" s="10" t="n"/>
+      <c r="Y16" s="10" t="n"/>
+      <c r="Z16" s="10" t="n"/>
+      <c r="AA16" s="10" t="n"/>
+      <c r="AB16" s="10" t="n"/>
+      <c r="AC16" s="10" t="n"/>
+      <c r="AD16" s="10" t="n"/>
+      <c r="AE16" s="10" t="n"/>
+      <c r="AF16" s="10" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="25" t="inlineStr">
+        <is>
+          <t>Tower B</t>
+        </is>
+      </c>
+      <c r="B17" s="25" t="inlineStr">
+        <is>
+          <t>L08</t>
+        </is>
+      </c>
+      <c r="C17" s="25" t="inlineStr">
+        <is>
+          <t>BL08</t>
+        </is>
+      </c>
+      <c r="D17" s="29" t="n"/>
+      <c r="E17" s="27" t="n"/>
+      <c r="F17" s="29" t="n"/>
+      <c r="G17" s="27" t="n"/>
+      <c r="H17" s="29" t="n"/>
+      <c r="I17" s="27" t="n"/>
+      <c r="J17" s="29" t="n"/>
+      <c r="K17" s="27" t="n"/>
+      <c r="L17" s="29" t="n"/>
+      <c r="M17" s="27" t="n"/>
+      <c r="N17" s="29" t="n"/>
+      <c r="O17" s="27" t="n"/>
+      <c r="P17" s="29" t="n"/>
+      <c r="Q17" s="27" t="n"/>
+      <c r="R17" s="10" t="n"/>
+      <c r="S17" s="10" t="n"/>
+      <c r="T17" s="10" t="n"/>
+      <c r="U17" s="10" t="n"/>
+      <c r="V17" s="10" t="n"/>
+      <c r="W17" s="10" t="n"/>
+      <c r="X17" s="10" t="n"/>
+      <c r="Y17" s="10" t="n"/>
+      <c r="Z17" s="10" t="n"/>
+      <c r="AA17" s="10" t="n"/>
+      <c r="AB17" s="10" t="n"/>
+      <c r="AC17" s="10" t="n"/>
+      <c r="AD17" s="10" t="n"/>
+      <c r="AE17" s="10" t="n"/>
+      <c r="AF17" s="10" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="25" t="inlineStr">
+        <is>
+          <t>Tower B</t>
+        </is>
+      </c>
+      <c r="B18" s="25" t="inlineStr">
+        <is>
+          <t>L09</t>
+        </is>
+      </c>
+      <c r="C18" s="25" t="inlineStr">
+        <is>
+          <t>BL09</t>
+        </is>
+      </c>
+      <c r="D18" s="29" t="n"/>
+      <c r="E18" s="27" t="n"/>
+      <c r="F18" s="29" t="n"/>
+      <c r="G18" s="27" t="n"/>
+      <c r="H18" s="29" t="n"/>
+      <c r="I18" s="27" t="n"/>
+      <c r="J18" s="29" t="n"/>
+      <c r="K18" s="27" t="n"/>
+      <c r="L18" s="29" t="n"/>
+      <c r="M18" s="27" t="n"/>
+      <c r="N18" s="29" t="n"/>
+      <c r="O18" s="27" t="n"/>
+      <c r="P18" s="29" t="n"/>
+      <c r="Q18" s="27" t="n"/>
+      <c r="R18" s="10" t="n"/>
+      <c r="S18" s="10" t="n"/>
+      <c r="T18" s="10" t="n"/>
+      <c r="U18" s="10" t="n"/>
+      <c r="V18" s="10" t="n"/>
+      <c r="W18" s="10" t="n"/>
+      <c r="X18" s="10" t="n"/>
+      <c r="Y18" s="10" t="n"/>
+      <c r="Z18" s="10" t="n"/>
+      <c r="AA18" s="10" t="n"/>
+      <c r="AB18" s="10" t="n"/>
+      <c r="AC18" s="10" t="n"/>
+      <c r="AD18" s="10" t="n"/>
+      <c r="AE18" s="10" t="n"/>
+      <c r="AF18" s="10" t="n"/>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="1" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="0" password="D6EA"/>
+  <conditionalFormatting sqref="D2:D18">
+    <cfRule type="expression" priority="1" dxfId="5" stopIfTrue="1">
+      <formula>TRIM(UPPER(D2))="A"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="5" stopIfTrue="1">
+      <formula>TRIM(UPPER(D2))="B"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="3" stopIfTrue="1">
+      <formula>TRIM(UPPER(D2))="UR"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="2" stopIfTrue="1">
+      <formula>TRIM(UPPER(D2))="C"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="1" stopIfTrue="1">
+      <formula>TRIM(UPPER(D2))="TBS"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F2:F18">
+    <cfRule type="expression" priority="6" dxfId="5" stopIfTrue="1">
+      <formula>TRIM(UPPER(F2))="A"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="7" dxfId="5" stopIfTrue="1">
+      <formula>TRIM(UPPER(F2))="B"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" dxfId="3" stopIfTrue="1">
+      <formula>TRIM(UPPER(F2))="UR"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="9" dxfId="2" stopIfTrue="1">
+      <formula>TRIM(UPPER(F2))="C"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="10" dxfId="1" stopIfTrue="1">
+      <formula>TRIM(UPPER(F2))="TBS"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2:H18">
+    <cfRule type="expression" priority="11" dxfId="5" stopIfTrue="1">
+      <formula>TRIM(UPPER(H2))="A"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="12" dxfId="5" stopIfTrue="1">
+      <formula>TRIM(UPPER(H2))="B"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="13" dxfId="3" stopIfTrue="1">
+      <formula>TRIM(UPPER(H2))="UR"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="14" dxfId="2" stopIfTrue="1">
+      <formula>TRIM(UPPER(H2))="C"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="15" dxfId="1" stopIfTrue="1">
+      <formula>TRIM(UPPER(H2))="TBS"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J2:J18">
+    <cfRule type="expression" priority="16" dxfId="5" stopIfTrue="1">
+      <formula>TRIM(UPPER(J2))="A"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="17" dxfId="5" stopIfTrue="1">
+      <formula>TRIM(UPPER(J2))="B"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="18" dxfId="3" stopIfTrue="1">
+      <formula>TRIM(UPPER(J2))="UR"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="19" dxfId="2" stopIfTrue="1">
+      <formula>TRIM(UPPER(J2))="C"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="20" dxfId="1" stopIfTrue="1">
+      <formula>TRIM(UPPER(J2))="TBS"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L2:L18">
+    <cfRule type="expression" priority="21" dxfId="5" stopIfTrue="1">
+      <formula>TRIM(UPPER(L2))="A"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="22" dxfId="5" stopIfTrue="1">
+      <formula>TRIM(UPPER(L2))="B"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="23" dxfId="3" stopIfTrue="1">
+      <formula>TRIM(UPPER(L2))="UR"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="24" dxfId="2" stopIfTrue="1">
+      <formula>TRIM(UPPER(L2))="C"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="25" dxfId="1" stopIfTrue="1">
+      <formula>TRIM(UPPER(L2))="TBS"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N2:N18">
+    <cfRule type="expression" priority="26" dxfId="5" stopIfTrue="1">
+      <formula>TRIM(UPPER(N2))="A"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="27" dxfId="5" stopIfTrue="1">
+      <formula>TRIM(UPPER(N2))="B"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="28" dxfId="3" stopIfTrue="1">
+      <formula>TRIM(UPPER(N2))="UR"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="29" dxfId="2" stopIfTrue="1">
+      <formula>TRIM(UPPER(N2))="C"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="30" dxfId="1" stopIfTrue="1">
+      <formula>TRIM(UPPER(N2))="TBS"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P2:P18">
+    <cfRule type="expression" priority="31" dxfId="5" stopIfTrue="1">
+      <formula>TRIM(UPPER(P2))="A"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="32" dxfId="5" stopIfTrue="1">
+      <formula>TRIM(UPPER(P2))="B"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="33" dxfId="3" stopIfTrue="1">
+      <formula>TRIM(UPPER(P2))="UR"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="34" dxfId="2" stopIfTrue="1">
+      <formula>TRIM(UPPER(P2))="C"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="35" dxfId="1" stopIfTrue="1">
+      <formula>TRIM(UPPER(P2))="TBS"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation sqref="D2:D18 F2:F18 H2:H18 J2:J18 L2:L18 N2:N18 P2:P18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Use A, B, UR, C or TBS" type="list">
+      <formula1>Lists!$A$2:$A$6</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E18 G2:G18 I2:I18 K2:K18 M2:M18 O2:O18 Q2:Q18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date"/>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F262"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
@@ -44491,7 +45555,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -46774,7 +47838,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -47504,7 +48568,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
FLS: Material and Shop Drawing status for every item
</commit_message>
<xml_diff>
--- a/WPH_Room_Register.xlsx
+++ b/WPH_Room_Register.xlsx
@@ -670,7 +670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A40"/>
+  <dimension ref="A1:A43"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -895,16 +895,22 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="31" t="inlineStr">
+      <c r="A39" s="31" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="9" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="31" t="inlineStr">
         <is>
           <t>FLS – FIRE LIFE &amp; SAFETY (FLS sheet)</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="9" t="inlineStr">
-        <is>
-          <t>One row per tower/level. Civil: Steel Doors, Wooden Doors, Fire Sealant, Hardware. MEP: Fire Sealant, Fire Alarm, Fire Fighting. Use the same codes A / B / UR / C / TBS and a date. Shown on the LEVEL QR page after the room list.</t>
+    <row r="43">
+      <c r="A43" s="9" t="inlineStr">
+        <is>
+          <t>One row per tower/level. Each item has a Material status and a Shop Drawing status (codes A / B / UR / C / TBS) with dates. Civil: Steel Doors, Wooden Doors, Fire Sealant, Hardware. MEP: Fire Sealant, Fire Alarm, Fire Fighting. Shown on the level QR page and on every room QR page of that level. A room can override its level by adding the same column header in Clearances.</t>
         </is>
       </c>
     </row>
@@ -41585,7 +41591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF18"/>
+  <dimension ref="A1:AT18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -41605,6 +41611,20 @@
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="12" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+    <col width="12" customWidth="1" min="27" max="27"/>
+    <col width="14" customWidth="1" min="28" max="28"/>
+    <col width="12" customWidth="1" min="29" max="29"/>
+    <col width="14" customWidth="1" min="30" max="30"/>
+    <col width="12" customWidth="1" min="31" max="31"/>
   </cols>
   <sheetData>
     <row r="1" ht="45" customHeight="1">
@@ -41625,89 +41645,159 @@
       </c>
       <c r="D1" s="24" t="inlineStr">
         <is>
-          <t>Civil - Steel Doors</t>
+          <t>Civil - Steel Doors - Material</t>
         </is>
       </c>
       <c r="E1" s="24" t="inlineStr">
         <is>
-          <t>Civil - Steel Doors Date</t>
+          <t>Civil - Steel Doors - Material Date</t>
         </is>
       </c>
       <c r="F1" s="24" t="inlineStr">
         <is>
-          <t>Civil - Wooden Doors</t>
+          <t>Civil - Steel Doors - Shop Drawing</t>
         </is>
       </c>
       <c r="G1" s="24" t="inlineStr">
         <is>
-          <t>Civil - Wooden Doors Date</t>
+          <t>Civil - Steel Doors - Shop Drawing Date</t>
         </is>
       </c>
       <c r="H1" s="24" t="inlineStr">
         <is>
-          <t>Civil - Fire Sealant</t>
+          <t>Civil - Wooden Doors - Material</t>
         </is>
       </c>
       <c r="I1" s="24" t="inlineStr">
         <is>
-          <t>Civil - Fire Sealant Date</t>
+          <t>Civil - Wooden Doors - Material Date</t>
         </is>
       </c>
       <c r="J1" s="24" t="inlineStr">
         <is>
-          <t>Civil - Hardware</t>
+          <t>Civil - Wooden Doors - Shop Drawing</t>
         </is>
       </c>
       <c r="K1" s="24" t="inlineStr">
         <is>
-          <t>Civil - Hardware Date</t>
+          <t>Civil - Wooden Doors - Shop Drawing Date</t>
         </is>
       </c>
       <c r="L1" s="24" t="inlineStr">
         <is>
-          <t>MEP - Fire Sealant</t>
+          <t>Civil - Fire Sealant - Material</t>
         </is>
       </c>
       <c r="M1" s="24" t="inlineStr">
         <is>
-          <t>MEP - Fire Sealant Date</t>
+          <t>Civil - Fire Sealant - Material Date</t>
         </is>
       </c>
       <c r="N1" s="24" t="inlineStr">
         <is>
-          <t>MEP - Fire Alarm</t>
+          <t>Civil - Fire Sealant - Shop Drawing</t>
         </is>
       </c>
       <c r="O1" s="24" t="inlineStr">
         <is>
-          <t>MEP - Fire Alarm Date</t>
+          <t>Civil - Fire Sealant - Shop Drawing Date</t>
         </is>
       </c>
       <c r="P1" s="24" t="inlineStr">
         <is>
-          <t>MEP - Fire Fighting</t>
+          <t>Civil - Hardware - Material</t>
         </is>
       </c>
       <c r="Q1" s="24" t="inlineStr">
         <is>
-          <t>MEP - Fire Fighting Date</t>
-        </is>
-      </c>
-      <c r="R1" s="10" t="n"/>
-      <c r="S1" s="10" t="n"/>
-      <c r="T1" s="10" t="n"/>
-      <c r="U1" s="10" t="n"/>
-      <c r="V1" s="10" t="n"/>
-      <c r="W1" s="10" t="n"/>
-      <c r="X1" s="10" t="n"/>
-      <c r="Y1" s="10" t="n"/>
-      <c r="Z1" s="10" t="n"/>
-      <c r="AA1" s="10" t="n"/>
-      <c r="AB1" s="10" t="n"/>
-      <c r="AC1" s="10" t="n"/>
-      <c r="AD1" s="10" t="n"/>
-      <c r="AE1" s="10" t="n"/>
+          <t>Civil - Hardware - Material Date</t>
+        </is>
+      </c>
+      <c r="R1" s="24" t="inlineStr">
+        <is>
+          <t>Civil - Hardware - Shop Drawing</t>
+        </is>
+      </c>
+      <c r="S1" s="24" t="inlineStr">
+        <is>
+          <t>Civil - Hardware - Shop Drawing Date</t>
+        </is>
+      </c>
+      <c r="T1" s="24" t="inlineStr">
+        <is>
+          <t>MEP - Fire Sealant - Material</t>
+        </is>
+      </c>
+      <c r="U1" s="24" t="inlineStr">
+        <is>
+          <t>MEP - Fire Sealant - Material Date</t>
+        </is>
+      </c>
+      <c r="V1" s="24" t="inlineStr">
+        <is>
+          <t>MEP - Fire Sealant - Shop Drawing</t>
+        </is>
+      </c>
+      <c r="W1" s="24" t="inlineStr">
+        <is>
+          <t>MEP - Fire Sealant - Shop Drawing Date</t>
+        </is>
+      </c>
+      <c r="X1" s="24" t="inlineStr">
+        <is>
+          <t>MEP - Fire Alarm - Material</t>
+        </is>
+      </c>
+      <c r="Y1" s="24" t="inlineStr">
+        <is>
+          <t>MEP - Fire Alarm - Material Date</t>
+        </is>
+      </c>
+      <c r="Z1" s="24" t="inlineStr">
+        <is>
+          <t>MEP - Fire Alarm - Shop Drawing</t>
+        </is>
+      </c>
+      <c r="AA1" s="24" t="inlineStr">
+        <is>
+          <t>MEP - Fire Alarm - Shop Drawing Date</t>
+        </is>
+      </c>
+      <c r="AB1" s="24" t="inlineStr">
+        <is>
+          <t>MEP - Fire Fighting - Material</t>
+        </is>
+      </c>
+      <c r="AC1" s="24" t="inlineStr">
+        <is>
+          <t>MEP - Fire Fighting - Material Date</t>
+        </is>
+      </c>
+      <c r="AD1" s="24" t="inlineStr">
+        <is>
+          <t>MEP - Fire Fighting - Shop Drawing</t>
+        </is>
+      </c>
+      <c r="AE1" s="24" t="inlineStr">
+        <is>
+          <t>MEP - Fire Fighting - Shop Drawing Date</t>
+        </is>
+      </c>
       <c r="AF1" s="10" t="n"/>
+      <c r="AG1" s="10" t="n"/>
+      <c r="AH1" s="10" t="n"/>
+      <c r="AI1" s="10" t="n"/>
+      <c r="AJ1" s="10" t="n"/>
+      <c r="AK1" s="10" t="n"/>
+      <c r="AL1" s="10" t="n"/>
+      <c r="AM1" s="10" t="n"/>
+      <c r="AN1" s="10" t="n"/>
+      <c r="AO1" s="10" t="n"/>
+      <c r="AP1" s="10" t="n"/>
+      <c r="AQ1" s="10" t="n"/>
+      <c r="AR1" s="10" t="n"/>
+      <c r="AS1" s="10" t="n"/>
+      <c r="AT1" s="10" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="25" t="inlineStr">
@@ -41739,21 +41829,35 @@
       <c r="O2" s="27" t="n"/>
       <c r="P2" s="29" t="n"/>
       <c r="Q2" s="27" t="n"/>
-      <c r="R2" s="10" t="n"/>
-      <c r="S2" s="10" t="n"/>
-      <c r="T2" s="10" t="n"/>
-      <c r="U2" s="10" t="n"/>
-      <c r="V2" s="10" t="n"/>
-      <c r="W2" s="10" t="n"/>
-      <c r="X2" s="10" t="n"/>
-      <c r="Y2" s="10" t="n"/>
-      <c r="Z2" s="10" t="n"/>
-      <c r="AA2" s="10" t="n"/>
-      <c r="AB2" s="10" t="n"/>
-      <c r="AC2" s="10" t="n"/>
-      <c r="AD2" s="10" t="n"/>
-      <c r="AE2" s="10" t="n"/>
+      <c r="R2" s="29" t="n"/>
+      <c r="S2" s="27" t="n"/>
+      <c r="T2" s="29" t="n"/>
+      <c r="U2" s="27" t="n"/>
+      <c r="V2" s="29" t="n"/>
+      <c r="W2" s="27" t="n"/>
+      <c r="X2" s="29" t="n"/>
+      <c r="Y2" s="27" t="n"/>
+      <c r="Z2" s="29" t="n"/>
+      <c r="AA2" s="27" t="n"/>
+      <c r="AB2" s="29" t="n"/>
+      <c r="AC2" s="27" t="n"/>
+      <c r="AD2" s="29" t="n"/>
+      <c r="AE2" s="27" t="n"/>
       <c r="AF2" s="10" t="n"/>
+      <c r="AG2" s="10" t="n"/>
+      <c r="AH2" s="10" t="n"/>
+      <c r="AI2" s="10" t="n"/>
+      <c r="AJ2" s="10" t="n"/>
+      <c r="AK2" s="10" t="n"/>
+      <c r="AL2" s="10" t="n"/>
+      <c r="AM2" s="10" t="n"/>
+      <c r="AN2" s="10" t="n"/>
+      <c r="AO2" s="10" t="n"/>
+      <c r="AP2" s="10" t="n"/>
+      <c r="AQ2" s="10" t="n"/>
+      <c r="AR2" s="10" t="n"/>
+      <c r="AS2" s="10" t="n"/>
+      <c r="AT2" s="10" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -41785,21 +41889,35 @@
       <c r="O3" s="27" t="n"/>
       <c r="P3" s="29" t="n"/>
       <c r="Q3" s="27" t="n"/>
-      <c r="R3" s="10" t="n"/>
-      <c r="S3" s="10" t="n"/>
-      <c r="T3" s="10" t="n"/>
-      <c r="U3" s="10" t="n"/>
-      <c r="V3" s="10" t="n"/>
-      <c r="W3" s="10" t="n"/>
-      <c r="X3" s="10" t="n"/>
-      <c r="Y3" s="10" t="n"/>
-      <c r="Z3" s="10" t="n"/>
-      <c r="AA3" s="10" t="n"/>
-      <c r="AB3" s="10" t="n"/>
-      <c r="AC3" s="10" t="n"/>
-      <c r="AD3" s="10" t="n"/>
-      <c r="AE3" s="10" t="n"/>
+      <c r="R3" s="29" t="n"/>
+      <c r="S3" s="27" t="n"/>
+      <c r="T3" s="29" t="n"/>
+      <c r="U3" s="27" t="n"/>
+      <c r="V3" s="29" t="n"/>
+      <c r="W3" s="27" t="n"/>
+      <c r="X3" s="29" t="n"/>
+      <c r="Y3" s="27" t="n"/>
+      <c r="Z3" s="29" t="n"/>
+      <c r="AA3" s="27" t="n"/>
+      <c r="AB3" s="29" t="n"/>
+      <c r="AC3" s="27" t="n"/>
+      <c r="AD3" s="29" t="n"/>
+      <c r="AE3" s="27" t="n"/>
       <c r="AF3" s="10" t="n"/>
+      <c r="AG3" s="10" t="n"/>
+      <c r="AH3" s="10" t="n"/>
+      <c r="AI3" s="10" t="n"/>
+      <c r="AJ3" s="10" t="n"/>
+      <c r="AK3" s="10" t="n"/>
+      <c r="AL3" s="10" t="n"/>
+      <c r="AM3" s="10" t="n"/>
+      <c r="AN3" s="10" t="n"/>
+      <c r="AO3" s="10" t="n"/>
+      <c r="AP3" s="10" t="n"/>
+      <c r="AQ3" s="10" t="n"/>
+      <c r="AR3" s="10" t="n"/>
+      <c r="AS3" s="10" t="n"/>
+      <c r="AT3" s="10" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="25" t="inlineStr">
@@ -41831,21 +41949,35 @@
       <c r="O4" s="27" t="n"/>
       <c r="P4" s="29" t="n"/>
       <c r="Q4" s="27" t="n"/>
-      <c r="R4" s="10" t="n"/>
-      <c r="S4" s="10" t="n"/>
-      <c r="T4" s="10" t="n"/>
-      <c r="U4" s="10" t="n"/>
-      <c r="V4" s="10" t="n"/>
-      <c r="W4" s="10" t="n"/>
-      <c r="X4" s="10" t="n"/>
-      <c r="Y4" s="10" t="n"/>
-      <c r="Z4" s="10" t="n"/>
-      <c r="AA4" s="10" t="n"/>
-      <c r="AB4" s="10" t="n"/>
-      <c r="AC4" s="10" t="n"/>
-      <c r="AD4" s="10" t="n"/>
-      <c r="AE4" s="10" t="n"/>
+      <c r="R4" s="29" t="n"/>
+      <c r="S4" s="27" t="n"/>
+      <c r="T4" s="29" t="n"/>
+      <c r="U4" s="27" t="n"/>
+      <c r="V4" s="29" t="n"/>
+      <c r="W4" s="27" t="n"/>
+      <c r="X4" s="29" t="n"/>
+      <c r="Y4" s="27" t="n"/>
+      <c r="Z4" s="29" t="n"/>
+      <c r="AA4" s="27" t="n"/>
+      <c r="AB4" s="29" t="n"/>
+      <c r="AC4" s="27" t="n"/>
+      <c r="AD4" s="29" t="n"/>
+      <c r="AE4" s="27" t="n"/>
       <c r="AF4" s="10" t="n"/>
+      <c r="AG4" s="10" t="n"/>
+      <c r="AH4" s="10" t="n"/>
+      <c r="AI4" s="10" t="n"/>
+      <c r="AJ4" s="10" t="n"/>
+      <c r="AK4" s="10" t="n"/>
+      <c r="AL4" s="10" t="n"/>
+      <c r="AM4" s="10" t="n"/>
+      <c r="AN4" s="10" t="n"/>
+      <c r="AO4" s="10" t="n"/>
+      <c r="AP4" s="10" t="n"/>
+      <c r="AQ4" s="10" t="n"/>
+      <c r="AR4" s="10" t="n"/>
+      <c r="AS4" s="10" t="n"/>
+      <c r="AT4" s="10" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="25" t="inlineStr">
@@ -41877,21 +42009,35 @@
       <c r="O5" s="27" t="n"/>
       <c r="P5" s="29" t="n"/>
       <c r="Q5" s="27" t="n"/>
-      <c r="R5" s="10" t="n"/>
-      <c r="S5" s="10" t="n"/>
-      <c r="T5" s="10" t="n"/>
-      <c r="U5" s="10" t="n"/>
-      <c r="V5" s="10" t="n"/>
-      <c r="W5" s="10" t="n"/>
-      <c r="X5" s="10" t="n"/>
-      <c r="Y5" s="10" t="n"/>
-      <c r="Z5" s="10" t="n"/>
-      <c r="AA5" s="10" t="n"/>
-      <c r="AB5" s="10" t="n"/>
-      <c r="AC5" s="10" t="n"/>
-      <c r="AD5" s="10" t="n"/>
-      <c r="AE5" s="10" t="n"/>
+      <c r="R5" s="29" t="n"/>
+      <c r="S5" s="27" t="n"/>
+      <c r="T5" s="29" t="n"/>
+      <c r="U5" s="27" t="n"/>
+      <c r="V5" s="29" t="n"/>
+      <c r="W5" s="27" t="n"/>
+      <c r="X5" s="29" t="n"/>
+      <c r="Y5" s="27" t="n"/>
+      <c r="Z5" s="29" t="n"/>
+      <c r="AA5" s="27" t="n"/>
+      <c r="AB5" s="29" t="n"/>
+      <c r="AC5" s="27" t="n"/>
+      <c r="AD5" s="29" t="n"/>
+      <c r="AE5" s="27" t="n"/>
       <c r="AF5" s="10" t="n"/>
+      <c r="AG5" s="10" t="n"/>
+      <c r="AH5" s="10" t="n"/>
+      <c r="AI5" s="10" t="n"/>
+      <c r="AJ5" s="10" t="n"/>
+      <c r="AK5" s="10" t="n"/>
+      <c r="AL5" s="10" t="n"/>
+      <c r="AM5" s="10" t="n"/>
+      <c r="AN5" s="10" t="n"/>
+      <c r="AO5" s="10" t="n"/>
+      <c r="AP5" s="10" t="n"/>
+      <c r="AQ5" s="10" t="n"/>
+      <c r="AR5" s="10" t="n"/>
+      <c r="AS5" s="10" t="n"/>
+      <c r="AT5" s="10" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="25" t="inlineStr">
@@ -41923,21 +42069,35 @@
       <c r="O6" s="27" t="n"/>
       <c r="P6" s="29" t="n"/>
       <c r="Q6" s="27" t="n"/>
-      <c r="R6" s="10" t="n"/>
-      <c r="S6" s="10" t="n"/>
-      <c r="T6" s="10" t="n"/>
-      <c r="U6" s="10" t="n"/>
-      <c r="V6" s="10" t="n"/>
-      <c r="W6" s="10" t="n"/>
-      <c r="X6" s="10" t="n"/>
-      <c r="Y6" s="10" t="n"/>
-      <c r="Z6" s="10" t="n"/>
-      <c r="AA6" s="10" t="n"/>
-      <c r="AB6" s="10" t="n"/>
-      <c r="AC6" s="10" t="n"/>
-      <c r="AD6" s="10" t="n"/>
-      <c r="AE6" s="10" t="n"/>
+      <c r="R6" s="29" t="n"/>
+      <c r="S6" s="27" t="n"/>
+      <c r="T6" s="29" t="n"/>
+      <c r="U6" s="27" t="n"/>
+      <c r="V6" s="29" t="n"/>
+      <c r="W6" s="27" t="n"/>
+      <c r="X6" s="29" t="n"/>
+      <c r="Y6" s="27" t="n"/>
+      <c r="Z6" s="29" t="n"/>
+      <c r="AA6" s="27" t="n"/>
+      <c r="AB6" s="29" t="n"/>
+      <c r="AC6" s="27" t="n"/>
+      <c r="AD6" s="29" t="n"/>
+      <c r="AE6" s="27" t="n"/>
       <c r="AF6" s="10" t="n"/>
+      <c r="AG6" s="10" t="n"/>
+      <c r="AH6" s="10" t="n"/>
+      <c r="AI6" s="10" t="n"/>
+      <c r="AJ6" s="10" t="n"/>
+      <c r="AK6" s="10" t="n"/>
+      <c r="AL6" s="10" t="n"/>
+      <c r="AM6" s="10" t="n"/>
+      <c r="AN6" s="10" t="n"/>
+      <c r="AO6" s="10" t="n"/>
+      <c r="AP6" s="10" t="n"/>
+      <c r="AQ6" s="10" t="n"/>
+      <c r="AR6" s="10" t="n"/>
+      <c r="AS6" s="10" t="n"/>
+      <c r="AT6" s="10" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="25" t="inlineStr">
@@ -41969,21 +42129,35 @@
       <c r="O7" s="27" t="n"/>
       <c r="P7" s="29" t="n"/>
       <c r="Q7" s="27" t="n"/>
-      <c r="R7" s="10" t="n"/>
-      <c r="S7" s="10" t="n"/>
-      <c r="T7" s="10" t="n"/>
-      <c r="U7" s="10" t="n"/>
-      <c r="V7" s="10" t="n"/>
-      <c r="W7" s="10" t="n"/>
-      <c r="X7" s="10" t="n"/>
-      <c r="Y7" s="10" t="n"/>
-      <c r="Z7" s="10" t="n"/>
-      <c r="AA7" s="10" t="n"/>
-      <c r="AB7" s="10" t="n"/>
-      <c r="AC7" s="10" t="n"/>
-      <c r="AD7" s="10" t="n"/>
-      <c r="AE7" s="10" t="n"/>
+      <c r="R7" s="29" t="n"/>
+      <c r="S7" s="27" t="n"/>
+      <c r="T7" s="29" t="n"/>
+      <c r="U7" s="27" t="n"/>
+      <c r="V7" s="29" t="n"/>
+      <c r="W7" s="27" t="n"/>
+      <c r="X7" s="29" t="n"/>
+      <c r="Y7" s="27" t="n"/>
+      <c r="Z7" s="29" t="n"/>
+      <c r="AA7" s="27" t="n"/>
+      <c r="AB7" s="29" t="n"/>
+      <c r="AC7" s="27" t="n"/>
+      <c r="AD7" s="29" t="n"/>
+      <c r="AE7" s="27" t="n"/>
       <c r="AF7" s="10" t="n"/>
+      <c r="AG7" s="10" t="n"/>
+      <c r="AH7" s="10" t="n"/>
+      <c r="AI7" s="10" t="n"/>
+      <c r="AJ7" s="10" t="n"/>
+      <c r="AK7" s="10" t="n"/>
+      <c r="AL7" s="10" t="n"/>
+      <c r="AM7" s="10" t="n"/>
+      <c r="AN7" s="10" t="n"/>
+      <c r="AO7" s="10" t="n"/>
+      <c r="AP7" s="10" t="n"/>
+      <c r="AQ7" s="10" t="n"/>
+      <c r="AR7" s="10" t="n"/>
+      <c r="AS7" s="10" t="n"/>
+      <c r="AT7" s="10" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="25" t="inlineStr">
@@ -42015,21 +42189,35 @@
       <c r="O8" s="27" t="n"/>
       <c r="P8" s="29" t="n"/>
       <c r="Q8" s="27" t="n"/>
-      <c r="R8" s="10" t="n"/>
-      <c r="S8" s="10" t="n"/>
-      <c r="T8" s="10" t="n"/>
-      <c r="U8" s="10" t="n"/>
-      <c r="V8" s="10" t="n"/>
-      <c r="W8" s="10" t="n"/>
-      <c r="X8" s="10" t="n"/>
-      <c r="Y8" s="10" t="n"/>
-      <c r="Z8" s="10" t="n"/>
-      <c r="AA8" s="10" t="n"/>
-      <c r="AB8" s="10" t="n"/>
-      <c r="AC8" s="10" t="n"/>
-      <c r="AD8" s="10" t="n"/>
-      <c r="AE8" s="10" t="n"/>
+      <c r="R8" s="29" t="n"/>
+      <c r="S8" s="27" t="n"/>
+      <c r="T8" s="29" t="n"/>
+      <c r="U8" s="27" t="n"/>
+      <c r="V8" s="29" t="n"/>
+      <c r="W8" s="27" t="n"/>
+      <c r="X8" s="29" t="n"/>
+      <c r="Y8" s="27" t="n"/>
+      <c r="Z8" s="29" t="n"/>
+      <c r="AA8" s="27" t="n"/>
+      <c r="AB8" s="29" t="n"/>
+      <c r="AC8" s="27" t="n"/>
+      <c r="AD8" s="29" t="n"/>
+      <c r="AE8" s="27" t="n"/>
       <c r="AF8" s="10" t="n"/>
+      <c r="AG8" s="10" t="n"/>
+      <c r="AH8" s="10" t="n"/>
+      <c r="AI8" s="10" t="n"/>
+      <c r="AJ8" s="10" t="n"/>
+      <c r="AK8" s="10" t="n"/>
+      <c r="AL8" s="10" t="n"/>
+      <c r="AM8" s="10" t="n"/>
+      <c r="AN8" s="10" t="n"/>
+      <c r="AO8" s="10" t="n"/>
+      <c r="AP8" s="10" t="n"/>
+      <c r="AQ8" s="10" t="n"/>
+      <c r="AR8" s="10" t="n"/>
+      <c r="AS8" s="10" t="n"/>
+      <c r="AT8" s="10" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="25" t="inlineStr">
@@ -42061,21 +42249,35 @@
       <c r="O9" s="27" t="n"/>
       <c r="P9" s="29" t="n"/>
       <c r="Q9" s="27" t="n"/>
-      <c r="R9" s="10" t="n"/>
-      <c r="S9" s="10" t="n"/>
-      <c r="T9" s="10" t="n"/>
-      <c r="U9" s="10" t="n"/>
-      <c r="V9" s="10" t="n"/>
-      <c r="W9" s="10" t="n"/>
-      <c r="X9" s="10" t="n"/>
-      <c r="Y9" s="10" t="n"/>
-      <c r="Z9" s="10" t="n"/>
-      <c r="AA9" s="10" t="n"/>
-      <c r="AB9" s="10" t="n"/>
-      <c r="AC9" s="10" t="n"/>
-      <c r="AD9" s="10" t="n"/>
-      <c r="AE9" s="10" t="n"/>
+      <c r="R9" s="29" t="n"/>
+      <c r="S9" s="27" t="n"/>
+      <c r="T9" s="29" t="n"/>
+      <c r="U9" s="27" t="n"/>
+      <c r="V9" s="29" t="n"/>
+      <c r="W9" s="27" t="n"/>
+      <c r="X9" s="29" t="n"/>
+      <c r="Y9" s="27" t="n"/>
+      <c r="Z9" s="29" t="n"/>
+      <c r="AA9" s="27" t="n"/>
+      <c r="AB9" s="29" t="n"/>
+      <c r="AC9" s="27" t="n"/>
+      <c r="AD9" s="29" t="n"/>
+      <c r="AE9" s="27" t="n"/>
       <c r="AF9" s="10" t="n"/>
+      <c r="AG9" s="10" t="n"/>
+      <c r="AH9" s="10" t="n"/>
+      <c r="AI9" s="10" t="n"/>
+      <c r="AJ9" s="10" t="n"/>
+      <c r="AK9" s="10" t="n"/>
+      <c r="AL9" s="10" t="n"/>
+      <c r="AM9" s="10" t="n"/>
+      <c r="AN9" s="10" t="n"/>
+      <c r="AO9" s="10" t="n"/>
+      <c r="AP9" s="10" t="n"/>
+      <c r="AQ9" s="10" t="n"/>
+      <c r="AR9" s="10" t="n"/>
+      <c r="AS9" s="10" t="n"/>
+      <c r="AT9" s="10" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="25" t="inlineStr">
@@ -42107,21 +42309,35 @@
       <c r="O10" s="27" t="n"/>
       <c r="P10" s="29" t="n"/>
       <c r="Q10" s="27" t="n"/>
-      <c r="R10" s="10" t="n"/>
-      <c r="S10" s="10" t="n"/>
-      <c r="T10" s="10" t="n"/>
-      <c r="U10" s="10" t="n"/>
-      <c r="V10" s="10" t="n"/>
-      <c r="W10" s="10" t="n"/>
-      <c r="X10" s="10" t="n"/>
-      <c r="Y10" s="10" t="n"/>
-      <c r="Z10" s="10" t="n"/>
-      <c r="AA10" s="10" t="n"/>
-      <c r="AB10" s="10" t="n"/>
-      <c r="AC10" s="10" t="n"/>
-      <c r="AD10" s="10" t="n"/>
-      <c r="AE10" s="10" t="n"/>
+      <c r="R10" s="29" t="n"/>
+      <c r="S10" s="27" t="n"/>
+      <c r="T10" s="29" t="n"/>
+      <c r="U10" s="27" t="n"/>
+      <c r="V10" s="29" t="n"/>
+      <c r="W10" s="27" t="n"/>
+      <c r="X10" s="29" t="n"/>
+      <c r="Y10" s="27" t="n"/>
+      <c r="Z10" s="29" t="n"/>
+      <c r="AA10" s="27" t="n"/>
+      <c r="AB10" s="29" t="n"/>
+      <c r="AC10" s="27" t="n"/>
+      <c r="AD10" s="29" t="n"/>
+      <c r="AE10" s="27" t="n"/>
       <c r="AF10" s="10" t="n"/>
+      <c r="AG10" s="10" t="n"/>
+      <c r="AH10" s="10" t="n"/>
+      <c r="AI10" s="10" t="n"/>
+      <c r="AJ10" s="10" t="n"/>
+      <c r="AK10" s="10" t="n"/>
+      <c r="AL10" s="10" t="n"/>
+      <c r="AM10" s="10" t="n"/>
+      <c r="AN10" s="10" t="n"/>
+      <c r="AO10" s="10" t="n"/>
+      <c r="AP10" s="10" t="n"/>
+      <c r="AQ10" s="10" t="n"/>
+      <c r="AR10" s="10" t="n"/>
+      <c r="AS10" s="10" t="n"/>
+      <c r="AT10" s="10" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="25" t="inlineStr">
@@ -42153,21 +42369,35 @@
       <c r="O11" s="27" t="n"/>
       <c r="P11" s="29" t="n"/>
       <c r="Q11" s="27" t="n"/>
-      <c r="R11" s="10" t="n"/>
-      <c r="S11" s="10" t="n"/>
-      <c r="T11" s="10" t="n"/>
-      <c r="U11" s="10" t="n"/>
-      <c r="V11" s="10" t="n"/>
-      <c r="W11" s="10" t="n"/>
-      <c r="X11" s="10" t="n"/>
-      <c r="Y11" s="10" t="n"/>
-      <c r="Z11" s="10" t="n"/>
-      <c r="AA11" s="10" t="n"/>
-      <c r="AB11" s="10" t="n"/>
-      <c r="AC11" s="10" t="n"/>
-      <c r="AD11" s="10" t="n"/>
-      <c r="AE11" s="10" t="n"/>
+      <c r="R11" s="29" t="n"/>
+      <c r="S11" s="27" t="n"/>
+      <c r="T11" s="29" t="n"/>
+      <c r="U11" s="27" t="n"/>
+      <c r="V11" s="29" t="n"/>
+      <c r="W11" s="27" t="n"/>
+      <c r="X11" s="29" t="n"/>
+      <c r="Y11" s="27" t="n"/>
+      <c r="Z11" s="29" t="n"/>
+      <c r="AA11" s="27" t="n"/>
+      <c r="AB11" s="29" t="n"/>
+      <c r="AC11" s="27" t="n"/>
+      <c r="AD11" s="29" t="n"/>
+      <c r="AE11" s="27" t="n"/>
       <c r="AF11" s="10" t="n"/>
+      <c r="AG11" s="10" t="n"/>
+      <c r="AH11" s="10" t="n"/>
+      <c r="AI11" s="10" t="n"/>
+      <c r="AJ11" s="10" t="n"/>
+      <c r="AK11" s="10" t="n"/>
+      <c r="AL11" s="10" t="n"/>
+      <c r="AM11" s="10" t="n"/>
+      <c r="AN11" s="10" t="n"/>
+      <c r="AO11" s="10" t="n"/>
+      <c r="AP11" s="10" t="n"/>
+      <c r="AQ11" s="10" t="n"/>
+      <c r="AR11" s="10" t="n"/>
+      <c r="AS11" s="10" t="n"/>
+      <c r="AT11" s="10" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="25" t="inlineStr">
@@ -42199,21 +42429,35 @@
       <c r="O12" s="27" t="n"/>
       <c r="P12" s="29" t="n"/>
       <c r="Q12" s="27" t="n"/>
-      <c r="R12" s="10" t="n"/>
-      <c r="S12" s="10" t="n"/>
-      <c r="T12" s="10" t="n"/>
-      <c r="U12" s="10" t="n"/>
-      <c r="V12" s="10" t="n"/>
-      <c r="W12" s="10" t="n"/>
-      <c r="X12" s="10" t="n"/>
-      <c r="Y12" s="10" t="n"/>
-      <c r="Z12" s="10" t="n"/>
-      <c r="AA12" s="10" t="n"/>
-      <c r="AB12" s="10" t="n"/>
-      <c r="AC12" s="10" t="n"/>
-      <c r="AD12" s="10" t="n"/>
-      <c r="AE12" s="10" t="n"/>
+      <c r="R12" s="29" t="n"/>
+      <c r="S12" s="27" t="n"/>
+      <c r="T12" s="29" t="n"/>
+      <c r="U12" s="27" t="n"/>
+      <c r="V12" s="29" t="n"/>
+      <c r="W12" s="27" t="n"/>
+      <c r="X12" s="29" t="n"/>
+      <c r="Y12" s="27" t="n"/>
+      <c r="Z12" s="29" t="n"/>
+      <c r="AA12" s="27" t="n"/>
+      <c r="AB12" s="29" t="n"/>
+      <c r="AC12" s="27" t="n"/>
+      <c r="AD12" s="29" t="n"/>
+      <c r="AE12" s="27" t="n"/>
       <c r="AF12" s="10" t="n"/>
+      <c r="AG12" s="10" t="n"/>
+      <c r="AH12" s="10" t="n"/>
+      <c r="AI12" s="10" t="n"/>
+      <c r="AJ12" s="10" t="n"/>
+      <c r="AK12" s="10" t="n"/>
+      <c r="AL12" s="10" t="n"/>
+      <c r="AM12" s="10" t="n"/>
+      <c r="AN12" s="10" t="n"/>
+      <c r="AO12" s="10" t="n"/>
+      <c r="AP12" s="10" t="n"/>
+      <c r="AQ12" s="10" t="n"/>
+      <c r="AR12" s="10" t="n"/>
+      <c r="AS12" s="10" t="n"/>
+      <c r="AT12" s="10" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="25" t="inlineStr">
@@ -42245,21 +42489,35 @@
       <c r="O13" s="27" t="n"/>
       <c r="P13" s="29" t="n"/>
       <c r="Q13" s="27" t="n"/>
-      <c r="R13" s="10" t="n"/>
-      <c r="S13" s="10" t="n"/>
-      <c r="T13" s="10" t="n"/>
-      <c r="U13" s="10" t="n"/>
-      <c r="V13" s="10" t="n"/>
-      <c r="W13" s="10" t="n"/>
-      <c r="X13" s="10" t="n"/>
-      <c r="Y13" s="10" t="n"/>
-      <c r="Z13" s="10" t="n"/>
-      <c r="AA13" s="10" t="n"/>
-      <c r="AB13" s="10" t="n"/>
-      <c r="AC13" s="10" t="n"/>
-      <c r="AD13" s="10" t="n"/>
-      <c r="AE13" s="10" t="n"/>
+      <c r="R13" s="29" t="n"/>
+      <c r="S13" s="27" t="n"/>
+      <c r="T13" s="29" t="n"/>
+      <c r="U13" s="27" t="n"/>
+      <c r="V13" s="29" t="n"/>
+      <c r="W13" s="27" t="n"/>
+      <c r="X13" s="29" t="n"/>
+      <c r="Y13" s="27" t="n"/>
+      <c r="Z13" s="29" t="n"/>
+      <c r="AA13" s="27" t="n"/>
+      <c r="AB13" s="29" t="n"/>
+      <c r="AC13" s="27" t="n"/>
+      <c r="AD13" s="29" t="n"/>
+      <c r="AE13" s="27" t="n"/>
       <c r="AF13" s="10" t="n"/>
+      <c r="AG13" s="10" t="n"/>
+      <c r="AH13" s="10" t="n"/>
+      <c r="AI13" s="10" t="n"/>
+      <c r="AJ13" s="10" t="n"/>
+      <c r="AK13" s="10" t="n"/>
+      <c r="AL13" s="10" t="n"/>
+      <c r="AM13" s="10" t="n"/>
+      <c r="AN13" s="10" t="n"/>
+      <c r="AO13" s="10" t="n"/>
+      <c r="AP13" s="10" t="n"/>
+      <c r="AQ13" s="10" t="n"/>
+      <c r="AR13" s="10" t="n"/>
+      <c r="AS13" s="10" t="n"/>
+      <c r="AT13" s="10" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="25" t="inlineStr">
@@ -42291,21 +42549,35 @@
       <c r="O14" s="27" t="n"/>
       <c r="P14" s="29" t="n"/>
       <c r="Q14" s="27" t="n"/>
-      <c r="R14" s="10" t="n"/>
-      <c r="S14" s="10" t="n"/>
-      <c r="T14" s="10" t="n"/>
-      <c r="U14" s="10" t="n"/>
-      <c r="V14" s="10" t="n"/>
-      <c r="W14" s="10" t="n"/>
-      <c r="X14" s="10" t="n"/>
-      <c r="Y14" s="10" t="n"/>
-      <c r="Z14" s="10" t="n"/>
-      <c r="AA14" s="10" t="n"/>
-      <c r="AB14" s="10" t="n"/>
-      <c r="AC14" s="10" t="n"/>
-      <c r="AD14" s="10" t="n"/>
-      <c r="AE14" s="10" t="n"/>
+      <c r="R14" s="29" t="n"/>
+      <c r="S14" s="27" t="n"/>
+      <c r="T14" s="29" t="n"/>
+      <c r="U14" s="27" t="n"/>
+      <c r="V14" s="29" t="n"/>
+      <c r="W14" s="27" t="n"/>
+      <c r="X14" s="29" t="n"/>
+      <c r="Y14" s="27" t="n"/>
+      <c r="Z14" s="29" t="n"/>
+      <c r="AA14" s="27" t="n"/>
+      <c r="AB14" s="29" t="n"/>
+      <c r="AC14" s="27" t="n"/>
+      <c r="AD14" s="29" t="n"/>
+      <c r="AE14" s="27" t="n"/>
       <c r="AF14" s="10" t="n"/>
+      <c r="AG14" s="10" t="n"/>
+      <c r="AH14" s="10" t="n"/>
+      <c r="AI14" s="10" t="n"/>
+      <c r="AJ14" s="10" t="n"/>
+      <c r="AK14" s="10" t="n"/>
+      <c r="AL14" s="10" t="n"/>
+      <c r="AM14" s="10" t="n"/>
+      <c r="AN14" s="10" t="n"/>
+      <c r="AO14" s="10" t="n"/>
+      <c r="AP14" s="10" t="n"/>
+      <c r="AQ14" s="10" t="n"/>
+      <c r="AR14" s="10" t="n"/>
+      <c r="AS14" s="10" t="n"/>
+      <c r="AT14" s="10" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="25" t="inlineStr">
@@ -42337,21 +42609,35 @@
       <c r="O15" s="27" t="n"/>
       <c r="P15" s="29" t="n"/>
       <c r="Q15" s="27" t="n"/>
-      <c r="R15" s="10" t="n"/>
-      <c r="S15" s="10" t="n"/>
-      <c r="T15" s="10" t="n"/>
-      <c r="U15" s="10" t="n"/>
-      <c r="V15" s="10" t="n"/>
-      <c r="W15" s="10" t="n"/>
-      <c r="X15" s="10" t="n"/>
-      <c r="Y15" s="10" t="n"/>
-      <c r="Z15" s="10" t="n"/>
-      <c r="AA15" s="10" t="n"/>
-      <c r="AB15" s="10" t="n"/>
-      <c r="AC15" s="10" t="n"/>
-      <c r="AD15" s="10" t="n"/>
-      <c r="AE15" s="10" t="n"/>
+      <c r="R15" s="29" t="n"/>
+      <c r="S15" s="27" t="n"/>
+      <c r="T15" s="29" t="n"/>
+      <c r="U15" s="27" t="n"/>
+      <c r="V15" s="29" t="n"/>
+      <c r="W15" s="27" t="n"/>
+      <c r="X15" s="29" t="n"/>
+      <c r="Y15" s="27" t="n"/>
+      <c r="Z15" s="29" t="n"/>
+      <c r="AA15" s="27" t="n"/>
+      <c r="AB15" s="29" t="n"/>
+      <c r="AC15" s="27" t="n"/>
+      <c r="AD15" s="29" t="n"/>
+      <c r="AE15" s="27" t="n"/>
       <c r="AF15" s="10" t="n"/>
+      <c r="AG15" s="10" t="n"/>
+      <c r="AH15" s="10" t="n"/>
+      <c r="AI15" s="10" t="n"/>
+      <c r="AJ15" s="10" t="n"/>
+      <c r="AK15" s="10" t="n"/>
+      <c r="AL15" s="10" t="n"/>
+      <c r="AM15" s="10" t="n"/>
+      <c r="AN15" s="10" t="n"/>
+      <c r="AO15" s="10" t="n"/>
+      <c r="AP15" s="10" t="n"/>
+      <c r="AQ15" s="10" t="n"/>
+      <c r="AR15" s="10" t="n"/>
+      <c r="AS15" s="10" t="n"/>
+      <c r="AT15" s="10" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="25" t="inlineStr">
@@ -42383,21 +42669,35 @@
       <c r="O16" s="27" t="n"/>
       <c r="P16" s="29" t="n"/>
       <c r="Q16" s="27" t="n"/>
-      <c r="R16" s="10" t="n"/>
-      <c r="S16" s="10" t="n"/>
-      <c r="T16" s="10" t="n"/>
-      <c r="U16" s="10" t="n"/>
-      <c r="V16" s="10" t="n"/>
-      <c r="W16" s="10" t="n"/>
-      <c r="X16" s="10" t="n"/>
-      <c r="Y16" s="10" t="n"/>
-      <c r="Z16" s="10" t="n"/>
-      <c r="AA16" s="10" t="n"/>
-      <c r="AB16" s="10" t="n"/>
-      <c r="AC16" s="10" t="n"/>
-      <c r="AD16" s="10" t="n"/>
-      <c r="AE16" s="10" t="n"/>
+      <c r="R16" s="29" t="n"/>
+      <c r="S16" s="27" t="n"/>
+      <c r="T16" s="29" t="n"/>
+      <c r="U16" s="27" t="n"/>
+      <c r="V16" s="29" t="n"/>
+      <c r="W16" s="27" t="n"/>
+      <c r="X16" s="29" t="n"/>
+      <c r="Y16" s="27" t="n"/>
+      <c r="Z16" s="29" t="n"/>
+      <c r="AA16" s="27" t="n"/>
+      <c r="AB16" s="29" t="n"/>
+      <c r="AC16" s="27" t="n"/>
+      <c r="AD16" s="29" t="n"/>
+      <c r="AE16" s="27" t="n"/>
       <c r="AF16" s="10" t="n"/>
+      <c r="AG16" s="10" t="n"/>
+      <c r="AH16" s="10" t="n"/>
+      <c r="AI16" s="10" t="n"/>
+      <c r="AJ16" s="10" t="n"/>
+      <c r="AK16" s="10" t="n"/>
+      <c r="AL16" s="10" t="n"/>
+      <c r="AM16" s="10" t="n"/>
+      <c r="AN16" s="10" t="n"/>
+      <c r="AO16" s="10" t="n"/>
+      <c r="AP16" s="10" t="n"/>
+      <c r="AQ16" s="10" t="n"/>
+      <c r="AR16" s="10" t="n"/>
+      <c r="AS16" s="10" t="n"/>
+      <c r="AT16" s="10" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="25" t="inlineStr">
@@ -42429,21 +42729,35 @@
       <c r="O17" s="27" t="n"/>
       <c r="P17" s="29" t="n"/>
       <c r="Q17" s="27" t="n"/>
-      <c r="R17" s="10" t="n"/>
-      <c r="S17" s="10" t="n"/>
-      <c r="T17" s="10" t="n"/>
-      <c r="U17" s="10" t="n"/>
-      <c r="V17" s="10" t="n"/>
-      <c r="W17" s="10" t="n"/>
-      <c r="X17" s="10" t="n"/>
-      <c r="Y17" s="10" t="n"/>
-      <c r="Z17" s="10" t="n"/>
-      <c r="AA17" s="10" t="n"/>
-      <c r="AB17" s="10" t="n"/>
-      <c r="AC17" s="10" t="n"/>
-      <c r="AD17" s="10" t="n"/>
-      <c r="AE17" s="10" t="n"/>
+      <c r="R17" s="29" t="n"/>
+      <c r="S17" s="27" t="n"/>
+      <c r="T17" s="29" t="n"/>
+      <c r="U17" s="27" t="n"/>
+      <c r="V17" s="29" t="n"/>
+      <c r="W17" s="27" t="n"/>
+      <c r="X17" s="29" t="n"/>
+      <c r="Y17" s="27" t="n"/>
+      <c r="Z17" s="29" t="n"/>
+      <c r="AA17" s="27" t="n"/>
+      <c r="AB17" s="29" t="n"/>
+      <c r="AC17" s="27" t="n"/>
+      <c r="AD17" s="29" t="n"/>
+      <c r="AE17" s="27" t="n"/>
       <c r="AF17" s="10" t="n"/>
+      <c r="AG17" s="10" t="n"/>
+      <c r="AH17" s="10" t="n"/>
+      <c r="AI17" s="10" t="n"/>
+      <c r="AJ17" s="10" t="n"/>
+      <c r="AK17" s="10" t="n"/>
+      <c r="AL17" s="10" t="n"/>
+      <c r="AM17" s="10" t="n"/>
+      <c r="AN17" s="10" t="n"/>
+      <c r="AO17" s="10" t="n"/>
+      <c r="AP17" s="10" t="n"/>
+      <c r="AQ17" s="10" t="n"/>
+      <c r="AR17" s="10" t="n"/>
+      <c r="AS17" s="10" t="n"/>
+      <c r="AT17" s="10" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="25" t="inlineStr">
@@ -42475,21 +42789,35 @@
       <c r="O18" s="27" t="n"/>
       <c r="P18" s="29" t="n"/>
       <c r="Q18" s="27" t="n"/>
-      <c r="R18" s="10" t="n"/>
-      <c r="S18" s="10" t="n"/>
-      <c r="T18" s="10" t="n"/>
-      <c r="U18" s="10" t="n"/>
-      <c r="V18" s="10" t="n"/>
-      <c r="W18" s="10" t="n"/>
-      <c r="X18" s="10" t="n"/>
-      <c r="Y18" s="10" t="n"/>
-      <c r="Z18" s="10" t="n"/>
-      <c r="AA18" s="10" t="n"/>
-      <c r="AB18" s="10" t="n"/>
-      <c r="AC18" s="10" t="n"/>
-      <c r="AD18" s="10" t="n"/>
-      <c r="AE18" s="10" t="n"/>
+      <c r="R18" s="29" t="n"/>
+      <c r="S18" s="27" t="n"/>
+      <c r="T18" s="29" t="n"/>
+      <c r="U18" s="27" t="n"/>
+      <c r="V18" s="29" t="n"/>
+      <c r="W18" s="27" t="n"/>
+      <c r="X18" s="29" t="n"/>
+      <c r="Y18" s="27" t="n"/>
+      <c r="Z18" s="29" t="n"/>
+      <c r="AA18" s="27" t="n"/>
+      <c r="AB18" s="29" t="n"/>
+      <c r="AC18" s="27" t="n"/>
+      <c r="AD18" s="29" t="n"/>
+      <c r="AE18" s="27" t="n"/>
       <c r="AF18" s="10" t="n"/>
+      <c r="AG18" s="10" t="n"/>
+      <c r="AH18" s="10" t="n"/>
+      <c r="AI18" s="10" t="n"/>
+      <c r="AJ18" s="10" t="n"/>
+      <c r="AK18" s="10" t="n"/>
+      <c r="AL18" s="10" t="n"/>
+      <c r="AM18" s="10" t="n"/>
+      <c r="AN18" s="10" t="n"/>
+      <c r="AO18" s="10" t="n"/>
+      <c r="AP18" s="10" t="n"/>
+      <c r="AQ18" s="10" t="n"/>
+      <c r="AR18" s="10" t="n"/>
+      <c r="AS18" s="10" t="n"/>
+      <c r="AT18" s="10" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="1" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="0" password="D6EA"/>
@@ -42612,11 +42940,130 @@
       <formula>TRIM(UPPER(P2))="TBS"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="R2:R18">
+    <cfRule type="expression" priority="36" dxfId="5" stopIfTrue="1">
+      <formula>TRIM(UPPER(R2))="A"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="37" dxfId="5" stopIfTrue="1">
+      <formula>TRIM(UPPER(R2))="B"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="38" dxfId="3" stopIfTrue="1">
+      <formula>TRIM(UPPER(R2))="UR"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="39" dxfId="2" stopIfTrue="1">
+      <formula>TRIM(UPPER(R2))="C"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="40" dxfId="1" stopIfTrue="1">
+      <formula>TRIM(UPPER(R2))="TBS"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T2:T18">
+    <cfRule type="expression" priority="41" dxfId="5" stopIfTrue="1">
+      <formula>TRIM(UPPER(T2))="A"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="42" dxfId="5" stopIfTrue="1">
+      <formula>TRIM(UPPER(T2))="B"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="43" dxfId="3" stopIfTrue="1">
+      <formula>TRIM(UPPER(T2))="UR"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="44" dxfId="2" stopIfTrue="1">
+      <formula>TRIM(UPPER(T2))="C"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="45" dxfId="1" stopIfTrue="1">
+      <formula>TRIM(UPPER(T2))="TBS"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="V2:V18">
+    <cfRule type="expression" priority="46" dxfId="5" stopIfTrue="1">
+      <formula>TRIM(UPPER(V2))="A"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="47" dxfId="5" stopIfTrue="1">
+      <formula>TRIM(UPPER(V2))="B"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="48" dxfId="3" stopIfTrue="1">
+      <formula>TRIM(UPPER(V2))="UR"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="49" dxfId="2" stopIfTrue="1">
+      <formula>TRIM(UPPER(V2))="C"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="50" dxfId="1" stopIfTrue="1">
+      <formula>TRIM(UPPER(V2))="TBS"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="X2:X18">
+    <cfRule type="expression" priority="51" dxfId="5" stopIfTrue="1">
+      <formula>TRIM(UPPER(X2))="A"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="52" dxfId="5" stopIfTrue="1">
+      <formula>TRIM(UPPER(X2))="B"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="53" dxfId="3" stopIfTrue="1">
+      <formula>TRIM(UPPER(X2))="UR"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="54" dxfId="2" stopIfTrue="1">
+      <formula>TRIM(UPPER(X2))="C"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="55" dxfId="1" stopIfTrue="1">
+      <formula>TRIM(UPPER(X2))="TBS"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Z2:Z18">
+    <cfRule type="expression" priority="56" dxfId="5" stopIfTrue="1">
+      <formula>TRIM(UPPER(Z2))="A"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="57" dxfId="5" stopIfTrue="1">
+      <formula>TRIM(UPPER(Z2))="B"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="58" dxfId="3" stopIfTrue="1">
+      <formula>TRIM(UPPER(Z2))="UR"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="59" dxfId="2" stopIfTrue="1">
+      <formula>TRIM(UPPER(Z2))="C"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="60" dxfId="1" stopIfTrue="1">
+      <formula>TRIM(UPPER(Z2))="TBS"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AB2:AB18">
+    <cfRule type="expression" priority="61" dxfId="5" stopIfTrue="1">
+      <formula>TRIM(UPPER(AB2))="A"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="62" dxfId="5" stopIfTrue="1">
+      <formula>TRIM(UPPER(AB2))="B"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="63" dxfId="3" stopIfTrue="1">
+      <formula>TRIM(UPPER(AB2))="UR"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="64" dxfId="2" stopIfTrue="1">
+      <formula>TRIM(UPPER(AB2))="C"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="65" dxfId="1" stopIfTrue="1">
+      <formula>TRIM(UPPER(AB2))="TBS"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AD2:AD18">
+    <cfRule type="expression" priority="66" dxfId="5" stopIfTrue="1">
+      <formula>TRIM(UPPER(AD2))="A"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="67" dxfId="5" stopIfTrue="1">
+      <formula>TRIM(UPPER(AD2))="B"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="68" dxfId="3" stopIfTrue="1">
+      <formula>TRIM(UPPER(AD2))="UR"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="69" dxfId="2" stopIfTrue="1">
+      <formula>TRIM(UPPER(AD2))="C"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="70" dxfId="1" stopIfTrue="1">
+      <formula>TRIM(UPPER(AD2))="TBS"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="D2:D18 F2:F18 H2:H18 J2:J18 L2:L18 N2:N18 P2:P18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Use A, B, UR, C or TBS" type="list">
+    <dataValidation sqref="D2:D18 F2:F18 H2:H18 J2:J18 L2:L18 N2:N18 P2:P18 R2:R18 T2:T18 V2:V18 X2:X18 Z2:Z18 AB2:AB18 AD2:AD18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Use A, B, UR, C or TBS" type="list">
       <formula1>Lists!$A$2:$A$6</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E18 G2:G18 I2:I18 K2:K18 M2:M18 O2:O18 Q2:Q18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date"/>
+    <dataValidation sqref="E2:E18 G2:G18 I2:I18 K2:K18 M2:M18 O2:O18 Q2:Q18 S2:S18 U2:U18 W2:W18 Y2:Y18 AA2:AA18 AC2:AC18 AE2:AE18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date"/>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Blank drawing statuses set to TBS (Shop Drawings and FLS)
</commit_message>
<xml_diff>
--- a/WPH_Room_Register.xlsx
+++ b/WPH_Room_Register.xlsx
@@ -35571,27 +35571,71 @@
       </c>
       <c r="H6" s="27" t="n"/>
       <c r="I6" s="28" t="n"/>
-      <c r="J6" s="29" t="n"/>
+      <c r="J6" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K6" s="28" t="n"/>
-      <c r="L6" s="29" t="n"/>
+      <c r="L6" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M6" s="28" t="n"/>
-      <c r="N6" s="29" t="n"/>
+      <c r="N6" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O6" s="28" t="n"/>
-      <c r="P6" s="29" t="n"/>
+      <c r="P6" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q6" s="28" t="n"/>
-      <c r="R6" s="29" t="n"/>
+      <c r="R6" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S6" s="28" t="n"/>
-      <c r="T6" s="29" t="n"/>
+      <c r="T6" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U6" s="28" t="n"/>
-      <c r="V6" s="29" t="n"/>
+      <c r="V6" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W6" s="28" t="n"/>
-      <c r="X6" s="29" t="n"/>
+      <c r="X6" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y6" s="28" t="n"/>
-      <c r="Z6" s="29" t="n"/>
+      <c r="Z6" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA6" s="28" t="n"/>
-      <c r="AB6" s="29" t="n"/>
+      <c r="AB6" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC6" s="28" t="n"/>
-      <c r="AD6" s="29" t="n"/>
+      <c r="AD6" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE6" s="10" t="n"/>
       <c r="AF6" s="10" t="n"/>
       <c r="AG6" s="10" t="n"/>
@@ -36452,27 +36496,71 @@
       </c>
       <c r="H13" s="27" t="n"/>
       <c r="I13" s="28" t="n"/>
-      <c r="J13" s="29" t="n"/>
+      <c r="J13" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K13" s="28" t="n"/>
-      <c r="L13" s="29" t="n"/>
+      <c r="L13" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M13" s="28" t="n"/>
-      <c r="N13" s="29" t="n"/>
+      <c r="N13" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O13" s="28" t="n"/>
-      <c r="P13" s="29" t="n"/>
+      <c r="P13" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q13" s="28" t="n"/>
-      <c r="R13" s="29" t="n"/>
+      <c r="R13" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S13" s="28" t="n"/>
-      <c r="T13" s="29" t="n"/>
+      <c r="T13" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U13" s="28" t="n"/>
-      <c r="V13" s="29" t="n"/>
+      <c r="V13" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W13" s="28" t="n"/>
-      <c r="X13" s="29" t="n"/>
+      <c r="X13" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y13" s="28" t="n"/>
-      <c r="Z13" s="29" t="n"/>
+      <c r="Z13" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA13" s="28" t="n"/>
-      <c r="AB13" s="29" t="n"/>
+      <c r="AB13" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC13" s="28" t="n"/>
-      <c r="AD13" s="29" t="n"/>
+      <c r="AD13" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE13" s="10" t="n"/>
       <c r="AF13" s="10" t="n"/>
       <c r="AG13" s="10" t="n"/>
@@ -36515,27 +36603,71 @@
       </c>
       <c r="H14" s="27" t="n"/>
       <c r="I14" s="28" t="n"/>
-      <c r="J14" s="29" t="n"/>
+      <c r="J14" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K14" s="28" t="n"/>
-      <c r="L14" s="29" t="n"/>
+      <c r="L14" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M14" s="28" t="n"/>
-      <c r="N14" s="29" t="n"/>
+      <c r="N14" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O14" s="28" t="n"/>
-      <c r="P14" s="29" t="n"/>
+      <c r="P14" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q14" s="28" t="n"/>
-      <c r="R14" s="29" t="n"/>
+      <c r="R14" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S14" s="28" t="n"/>
-      <c r="T14" s="29" t="n"/>
+      <c r="T14" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U14" s="28" t="n"/>
-      <c r="V14" s="29" t="n"/>
+      <c r="V14" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W14" s="28" t="n"/>
-      <c r="X14" s="29" t="n"/>
+      <c r="X14" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y14" s="28" t="n"/>
-      <c r="Z14" s="29" t="n"/>
+      <c r="Z14" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA14" s="28" t="n"/>
-      <c r="AB14" s="29" t="n"/>
+      <c r="AB14" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC14" s="28" t="n"/>
-      <c r="AD14" s="29" t="n"/>
+      <c r="AD14" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE14" s="10" t="n"/>
       <c r="AF14" s="10" t="n"/>
       <c r="AG14" s="10" t="n"/>
@@ -36578,27 +36710,71 @@
       </c>
       <c r="H15" s="27" t="n"/>
       <c r="I15" s="28" t="n"/>
-      <c r="J15" s="29" t="n"/>
+      <c r="J15" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K15" s="28" t="n"/>
-      <c r="L15" s="29" t="n"/>
+      <c r="L15" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M15" s="28" t="n"/>
-      <c r="N15" s="29" t="n"/>
+      <c r="N15" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O15" s="28" t="n"/>
-      <c r="P15" s="29" t="n"/>
+      <c r="P15" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q15" s="28" t="n"/>
-      <c r="R15" s="29" t="n"/>
+      <c r="R15" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S15" s="28" t="n"/>
-      <c r="T15" s="29" t="n"/>
+      <c r="T15" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U15" s="28" t="n"/>
-      <c r="V15" s="29" t="n"/>
+      <c r="V15" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W15" s="28" t="n"/>
-      <c r="X15" s="29" t="n"/>
+      <c r="X15" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y15" s="28" t="n"/>
-      <c r="Z15" s="29" t="n"/>
+      <c r="Z15" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA15" s="28" t="n"/>
-      <c r="AB15" s="29" t="n"/>
+      <c r="AB15" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC15" s="28" t="n"/>
-      <c r="AD15" s="29" t="n"/>
+      <c r="AD15" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE15" s="10" t="n"/>
       <c r="AF15" s="10" t="n"/>
       <c r="AG15" s="10" t="n"/>
@@ -36641,27 +36817,71 @@
       </c>
       <c r="H16" s="27" t="n"/>
       <c r="I16" s="28" t="n"/>
-      <c r="J16" s="29" t="n"/>
+      <c r="J16" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K16" s="28" t="n"/>
-      <c r="L16" s="29" t="n"/>
+      <c r="L16" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M16" s="28" t="n"/>
-      <c r="N16" s="29" t="n"/>
+      <c r="N16" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O16" s="28" t="n"/>
-      <c r="P16" s="29" t="n"/>
+      <c r="P16" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q16" s="28" t="n"/>
-      <c r="R16" s="29" t="n"/>
+      <c r="R16" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S16" s="28" t="n"/>
-      <c r="T16" s="29" t="n"/>
+      <c r="T16" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U16" s="28" t="n"/>
-      <c r="V16" s="29" t="n"/>
+      <c r="V16" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W16" s="28" t="n"/>
-      <c r="X16" s="29" t="n"/>
+      <c r="X16" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y16" s="28" t="n"/>
-      <c r="Z16" s="29" t="n"/>
+      <c r="Z16" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA16" s="28" t="n"/>
-      <c r="AB16" s="29" t="n"/>
+      <c r="AB16" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC16" s="28" t="n"/>
-      <c r="AD16" s="29" t="n"/>
+      <c r="AD16" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE16" s="10" t="n"/>
       <c r="AF16" s="10" t="n"/>
       <c r="AG16" s="10" t="n"/>
@@ -36704,27 +36924,71 @@
       </c>
       <c r="H17" s="27" t="n"/>
       <c r="I17" s="28" t="n"/>
-      <c r="J17" s="29" t="n"/>
+      <c r="J17" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K17" s="28" t="n"/>
-      <c r="L17" s="29" t="n"/>
+      <c r="L17" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M17" s="28" t="n"/>
-      <c r="N17" s="29" t="n"/>
+      <c r="N17" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O17" s="28" t="n"/>
-      <c r="P17" s="29" t="n"/>
+      <c r="P17" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q17" s="28" t="n"/>
-      <c r="R17" s="29" t="n"/>
+      <c r="R17" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S17" s="28" t="n"/>
-      <c r="T17" s="29" t="n"/>
+      <c r="T17" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U17" s="28" t="n"/>
-      <c r="V17" s="29" t="n"/>
+      <c r="V17" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W17" s="28" t="n"/>
-      <c r="X17" s="29" t="n"/>
+      <c r="X17" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y17" s="28" t="n"/>
-      <c r="Z17" s="29" t="n"/>
+      <c r="Z17" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA17" s="28" t="n"/>
-      <c r="AB17" s="29" t="n"/>
+      <c r="AB17" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC17" s="28" t="n"/>
-      <c r="AD17" s="29" t="n"/>
+      <c r="AD17" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE17" s="10" t="n"/>
       <c r="AF17" s="10" t="n"/>
       <c r="AG17" s="10" t="n"/>
@@ -36767,27 +37031,71 @@
       </c>
       <c r="H18" s="27" t="n"/>
       <c r="I18" s="28" t="n"/>
-      <c r="J18" s="29" t="n"/>
+      <c r="J18" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K18" s="28" t="n"/>
-      <c r="L18" s="29" t="n"/>
+      <c r="L18" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M18" s="28" t="n"/>
-      <c r="N18" s="29" t="n"/>
+      <c r="N18" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O18" s="28" t="n"/>
-      <c r="P18" s="29" t="n"/>
+      <c r="P18" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q18" s="28" t="n"/>
-      <c r="R18" s="29" t="n"/>
+      <c r="R18" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S18" s="28" t="n"/>
-      <c r="T18" s="29" t="n"/>
+      <c r="T18" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U18" s="28" t="n"/>
-      <c r="V18" s="29" t="n"/>
+      <c r="V18" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W18" s="28" t="n"/>
-      <c r="X18" s="29" t="n"/>
+      <c r="X18" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y18" s="28" t="n"/>
-      <c r="Z18" s="29" t="n"/>
+      <c r="Z18" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA18" s="28" t="n"/>
-      <c r="AB18" s="29" t="n"/>
+      <c r="AB18" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC18" s="28" t="n"/>
-      <c r="AD18" s="29" t="n"/>
+      <c r="AD18" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE18" s="10" t="n"/>
       <c r="AF18" s="10" t="n"/>
       <c r="AG18" s="10" t="n"/>
@@ -36830,27 +37138,71 @@
       </c>
       <c r="H19" s="27" t="n"/>
       <c r="I19" s="28" t="n"/>
-      <c r="J19" s="29" t="n"/>
+      <c r="J19" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K19" s="28" t="n"/>
-      <c r="L19" s="29" t="n"/>
+      <c r="L19" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M19" s="28" t="n"/>
-      <c r="N19" s="29" t="n"/>
+      <c r="N19" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O19" s="28" t="n"/>
-      <c r="P19" s="29" t="n"/>
+      <c r="P19" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q19" s="28" t="n"/>
-      <c r="R19" s="29" t="n"/>
+      <c r="R19" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S19" s="28" t="n"/>
-      <c r="T19" s="29" t="n"/>
+      <c r="T19" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U19" s="28" t="n"/>
-      <c r="V19" s="29" t="n"/>
+      <c r="V19" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W19" s="28" t="n"/>
-      <c r="X19" s="29" t="n"/>
+      <c r="X19" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y19" s="28" t="n"/>
-      <c r="Z19" s="29" t="n"/>
+      <c r="Z19" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA19" s="28" t="n"/>
-      <c r="AB19" s="29" t="n"/>
+      <c r="AB19" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC19" s="28" t="n"/>
-      <c r="AD19" s="29" t="n"/>
+      <c r="AD19" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE19" s="10" t="n"/>
       <c r="AF19" s="10" t="n"/>
       <c r="AG19" s="10" t="n"/>
@@ -36893,27 +37245,71 @@
       </c>
       <c r="H20" s="27" t="n"/>
       <c r="I20" s="28" t="n"/>
-      <c r="J20" s="29" t="n"/>
+      <c r="J20" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K20" s="28" t="n"/>
-      <c r="L20" s="29" t="n"/>
+      <c r="L20" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M20" s="28" t="n"/>
-      <c r="N20" s="29" t="n"/>
+      <c r="N20" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O20" s="28" t="n"/>
-      <c r="P20" s="29" t="n"/>
+      <c r="P20" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q20" s="28" t="n"/>
-      <c r="R20" s="29" t="n"/>
+      <c r="R20" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S20" s="28" t="n"/>
-      <c r="T20" s="29" t="n"/>
+      <c r="T20" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U20" s="28" t="n"/>
-      <c r="V20" s="29" t="n"/>
+      <c r="V20" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W20" s="28" t="n"/>
-      <c r="X20" s="29" t="n"/>
+      <c r="X20" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y20" s="28" t="n"/>
-      <c r="Z20" s="29" t="n"/>
+      <c r="Z20" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA20" s="28" t="n"/>
-      <c r="AB20" s="29" t="n"/>
+      <c r="AB20" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC20" s="28" t="n"/>
-      <c r="AD20" s="29" t="n"/>
+      <c r="AD20" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE20" s="10" t="n"/>
       <c r="AF20" s="10" t="n"/>
       <c r="AG20" s="10" t="n"/>
@@ -36956,27 +37352,71 @@
       </c>
       <c r="H21" s="27" t="n"/>
       <c r="I21" s="28" t="n"/>
-      <c r="J21" s="29" t="n"/>
+      <c r="J21" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K21" s="28" t="n"/>
-      <c r="L21" s="29" t="n"/>
+      <c r="L21" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M21" s="28" t="n"/>
-      <c r="N21" s="29" t="n"/>
+      <c r="N21" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O21" s="28" t="n"/>
-      <c r="P21" s="29" t="n"/>
+      <c r="P21" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q21" s="28" t="n"/>
-      <c r="R21" s="29" t="n"/>
+      <c r="R21" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S21" s="28" t="n"/>
-      <c r="T21" s="29" t="n"/>
+      <c r="T21" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U21" s="28" t="n"/>
-      <c r="V21" s="29" t="n"/>
+      <c r="V21" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W21" s="28" t="n"/>
-      <c r="X21" s="29" t="n"/>
+      <c r="X21" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y21" s="28" t="n"/>
-      <c r="Z21" s="29" t="n"/>
+      <c r="Z21" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA21" s="28" t="n"/>
-      <c r="AB21" s="29" t="n"/>
+      <c r="AB21" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC21" s="28" t="n"/>
-      <c r="AD21" s="29" t="n"/>
+      <c r="AD21" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE21" s="10" t="n"/>
       <c r="AF21" s="10" t="n"/>
       <c r="AG21" s="10" t="n"/>
@@ -37019,27 +37459,71 @@
       </c>
       <c r="H22" s="27" t="n"/>
       <c r="I22" s="28" t="n"/>
-      <c r="J22" s="29" t="n"/>
+      <c r="J22" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K22" s="28" t="n"/>
-      <c r="L22" s="29" t="n"/>
+      <c r="L22" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M22" s="28" t="n"/>
-      <c r="N22" s="29" t="n"/>
+      <c r="N22" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O22" s="28" t="n"/>
-      <c r="P22" s="29" t="n"/>
+      <c r="P22" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q22" s="28" t="n"/>
-      <c r="R22" s="29" t="n"/>
+      <c r="R22" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S22" s="28" t="n"/>
-      <c r="T22" s="29" t="n"/>
+      <c r="T22" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U22" s="28" t="n"/>
-      <c r="V22" s="29" t="n"/>
+      <c r="V22" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W22" s="28" t="n"/>
-      <c r="X22" s="29" t="n"/>
+      <c r="X22" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y22" s="28" t="n"/>
-      <c r="Z22" s="29" t="n"/>
+      <c r="Z22" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA22" s="28" t="n"/>
-      <c r="AB22" s="29" t="n"/>
+      <c r="AB22" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC22" s="28" t="n"/>
-      <c r="AD22" s="29" t="n"/>
+      <c r="AD22" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE22" s="10" t="n"/>
       <c r="AF22" s="10" t="n"/>
       <c r="AG22" s="10" t="n"/>
@@ -37082,27 +37566,71 @@
       </c>
       <c r="H23" s="27" t="n"/>
       <c r="I23" s="28" t="n"/>
-      <c r="J23" s="29" t="n"/>
+      <c r="J23" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K23" s="28" t="n"/>
-      <c r="L23" s="29" t="n"/>
+      <c r="L23" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M23" s="28" t="n"/>
-      <c r="N23" s="29" t="n"/>
+      <c r="N23" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O23" s="28" t="n"/>
-      <c r="P23" s="29" t="n"/>
+      <c r="P23" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q23" s="28" t="n"/>
-      <c r="R23" s="29" t="n"/>
+      <c r="R23" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S23" s="28" t="n"/>
-      <c r="T23" s="29" t="n"/>
+      <c r="T23" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U23" s="28" t="n"/>
-      <c r="V23" s="29" t="n"/>
+      <c r="V23" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W23" s="28" t="n"/>
-      <c r="X23" s="29" t="n"/>
+      <c r="X23" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y23" s="28" t="n"/>
-      <c r="Z23" s="29" t="n"/>
+      <c r="Z23" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA23" s="28" t="n"/>
-      <c r="AB23" s="29" t="n"/>
+      <c r="AB23" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC23" s="28" t="n"/>
-      <c r="AD23" s="29" t="n"/>
+      <c r="AD23" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE23" s="10" t="n"/>
       <c r="AF23" s="10" t="n"/>
       <c r="AG23" s="10" t="n"/>
@@ -37145,27 +37673,71 @@
       </c>
       <c r="H24" s="27" t="n"/>
       <c r="I24" s="28" t="n"/>
-      <c r="J24" s="29" t="n"/>
+      <c r="J24" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K24" s="28" t="n"/>
-      <c r="L24" s="29" t="n"/>
+      <c r="L24" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M24" s="28" t="n"/>
-      <c r="N24" s="29" t="n"/>
+      <c r="N24" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O24" s="28" t="n"/>
-      <c r="P24" s="29" t="n"/>
+      <c r="P24" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q24" s="28" t="n"/>
-      <c r="R24" s="29" t="n"/>
+      <c r="R24" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S24" s="28" t="n"/>
-      <c r="T24" s="29" t="n"/>
+      <c r="T24" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U24" s="28" t="n"/>
-      <c r="V24" s="29" t="n"/>
+      <c r="V24" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W24" s="28" t="n"/>
-      <c r="X24" s="29" t="n"/>
+      <c r="X24" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y24" s="28" t="n"/>
-      <c r="Z24" s="29" t="n"/>
+      <c r="Z24" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA24" s="28" t="n"/>
-      <c r="AB24" s="29" t="n"/>
+      <c r="AB24" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC24" s="28" t="n"/>
-      <c r="AD24" s="29" t="n"/>
+      <c r="AD24" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE24" s="10" t="n"/>
       <c r="AF24" s="10" t="n"/>
       <c r="AG24" s="10" t="n"/>
@@ -37208,27 +37780,71 @@
       </c>
       <c r="H25" s="27" t="n"/>
       <c r="I25" s="28" t="n"/>
-      <c r="J25" s="29" t="n"/>
+      <c r="J25" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K25" s="28" t="n"/>
-      <c r="L25" s="29" t="n"/>
+      <c r="L25" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M25" s="28" t="n"/>
-      <c r="N25" s="29" t="n"/>
+      <c r="N25" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O25" s="28" t="n"/>
-      <c r="P25" s="29" t="n"/>
+      <c r="P25" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q25" s="28" t="n"/>
-      <c r="R25" s="29" t="n"/>
+      <c r="R25" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S25" s="28" t="n"/>
-      <c r="T25" s="29" t="n"/>
+      <c r="T25" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U25" s="28" t="n"/>
-      <c r="V25" s="29" t="n"/>
+      <c r="V25" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W25" s="28" t="n"/>
-      <c r="X25" s="29" t="n"/>
+      <c r="X25" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y25" s="28" t="n"/>
-      <c r="Z25" s="29" t="n"/>
+      <c r="Z25" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA25" s="28" t="n"/>
-      <c r="AB25" s="29" t="n"/>
+      <c r="AB25" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC25" s="28" t="n"/>
-      <c r="AD25" s="29" t="n"/>
+      <c r="AD25" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE25" s="10" t="n"/>
       <c r="AF25" s="10" t="n"/>
       <c r="AG25" s="10" t="n"/>
@@ -37632,27 +38248,71 @@
       </c>
       <c r="H29" s="27" t="n"/>
       <c r="I29" s="28" t="n"/>
-      <c r="J29" s="29" t="n"/>
+      <c r="J29" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K29" s="28" t="n"/>
-      <c r="L29" s="29" t="n"/>
+      <c r="L29" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M29" s="28" t="n"/>
-      <c r="N29" s="29" t="n"/>
+      <c r="N29" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O29" s="28" t="n"/>
-      <c r="P29" s="29" t="n"/>
+      <c r="P29" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q29" s="28" t="n"/>
-      <c r="R29" s="29" t="n"/>
+      <c r="R29" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S29" s="28" t="n"/>
-      <c r="T29" s="29" t="n"/>
+      <c r="T29" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U29" s="28" t="n"/>
-      <c r="V29" s="29" t="n"/>
+      <c r="V29" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W29" s="28" t="n"/>
-      <c r="X29" s="29" t="n"/>
+      <c r="X29" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y29" s="28" t="n"/>
-      <c r="Z29" s="29" t="n"/>
+      <c r="Z29" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA29" s="28" t="n"/>
-      <c r="AB29" s="29" t="n"/>
+      <c r="AB29" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC29" s="28" t="n"/>
-      <c r="AD29" s="29" t="n"/>
+      <c r="AD29" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE29" s="10" t="n"/>
       <c r="AF29" s="10" t="n"/>
       <c r="AG29" s="10" t="n"/>
@@ -37695,27 +38355,71 @@
       </c>
       <c r="H30" s="27" t="n"/>
       <c r="I30" s="28" t="n"/>
-      <c r="J30" s="29" t="n"/>
+      <c r="J30" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K30" s="28" t="n"/>
-      <c r="L30" s="29" t="n"/>
+      <c r="L30" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M30" s="28" t="n"/>
-      <c r="N30" s="29" t="n"/>
+      <c r="N30" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O30" s="28" t="n"/>
-      <c r="P30" s="29" t="n"/>
+      <c r="P30" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q30" s="28" t="n"/>
-      <c r="R30" s="29" t="n"/>
+      <c r="R30" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S30" s="28" t="n"/>
-      <c r="T30" s="29" t="n"/>
+      <c r="T30" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U30" s="28" t="n"/>
-      <c r="V30" s="29" t="n"/>
+      <c r="V30" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W30" s="28" t="n"/>
-      <c r="X30" s="29" t="n"/>
+      <c r="X30" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y30" s="28" t="n"/>
-      <c r="Z30" s="29" t="n"/>
+      <c r="Z30" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA30" s="28" t="n"/>
-      <c r="AB30" s="29" t="n"/>
+      <c r="AB30" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC30" s="28" t="n"/>
-      <c r="AD30" s="29" t="n"/>
+      <c r="AD30" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE30" s="10" t="n"/>
       <c r="AF30" s="10" t="n"/>
       <c r="AG30" s="10" t="n"/>
@@ -37758,27 +38462,71 @@
       </c>
       <c r="H31" s="27" t="n"/>
       <c r="I31" s="28" t="n"/>
-      <c r="J31" s="29" t="n"/>
+      <c r="J31" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K31" s="28" t="n"/>
-      <c r="L31" s="29" t="n"/>
+      <c r="L31" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M31" s="28" t="n"/>
-      <c r="N31" s="29" t="n"/>
+      <c r="N31" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O31" s="28" t="n"/>
-      <c r="P31" s="29" t="n"/>
+      <c r="P31" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q31" s="28" t="n"/>
-      <c r="R31" s="29" t="n"/>
+      <c r="R31" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S31" s="28" t="n"/>
-      <c r="T31" s="29" t="n"/>
+      <c r="T31" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U31" s="28" t="n"/>
-      <c r="V31" s="29" t="n"/>
+      <c r="V31" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W31" s="28" t="n"/>
-      <c r="X31" s="29" t="n"/>
+      <c r="X31" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y31" s="28" t="n"/>
-      <c r="Z31" s="29" t="n"/>
+      <c r="Z31" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA31" s="28" t="n"/>
-      <c r="AB31" s="29" t="n"/>
+      <c r="AB31" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC31" s="28" t="n"/>
-      <c r="AD31" s="29" t="n"/>
+      <c r="AD31" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE31" s="10" t="n"/>
       <c r="AF31" s="10" t="n"/>
       <c r="AG31" s="10" t="n"/>
@@ -37821,27 +38569,71 @@
       </c>
       <c r="H32" s="27" t="n"/>
       <c r="I32" s="28" t="n"/>
-      <c r="J32" s="29" t="n"/>
+      <c r="J32" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K32" s="28" t="n"/>
-      <c r="L32" s="29" t="n"/>
+      <c r="L32" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M32" s="28" t="n"/>
-      <c r="N32" s="29" t="n"/>
+      <c r="N32" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O32" s="28" t="n"/>
-      <c r="P32" s="29" t="n"/>
+      <c r="P32" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q32" s="28" t="n"/>
-      <c r="R32" s="29" t="n"/>
+      <c r="R32" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S32" s="28" t="n"/>
-      <c r="T32" s="29" t="n"/>
+      <c r="T32" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U32" s="28" t="n"/>
-      <c r="V32" s="29" t="n"/>
+      <c r="V32" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W32" s="28" t="n"/>
-      <c r="X32" s="29" t="n"/>
+      <c r="X32" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y32" s="28" t="n"/>
-      <c r="Z32" s="29" t="n"/>
+      <c r="Z32" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA32" s="28" t="n"/>
-      <c r="AB32" s="29" t="n"/>
+      <c r="AB32" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC32" s="28" t="n"/>
-      <c r="AD32" s="29" t="n"/>
+      <c r="AD32" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE32" s="10" t="n"/>
       <c r="AF32" s="10" t="n"/>
       <c r="AG32" s="10" t="n"/>
@@ -37884,27 +38676,71 @@
       </c>
       <c r="H33" s="27" t="n"/>
       <c r="I33" s="28" t="n"/>
-      <c r="J33" s="29" t="n"/>
+      <c r="J33" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K33" s="28" t="n"/>
-      <c r="L33" s="29" t="n"/>
+      <c r="L33" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M33" s="28" t="n"/>
-      <c r="N33" s="29" t="n"/>
+      <c r="N33" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O33" s="28" t="n"/>
-      <c r="P33" s="29" t="n"/>
+      <c r="P33" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q33" s="28" t="n"/>
-      <c r="R33" s="29" t="n"/>
+      <c r="R33" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S33" s="28" t="n"/>
-      <c r="T33" s="29" t="n"/>
+      <c r="T33" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U33" s="28" t="n"/>
-      <c r="V33" s="29" t="n"/>
+      <c r="V33" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W33" s="28" t="n"/>
-      <c r="X33" s="29" t="n"/>
+      <c r="X33" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y33" s="28" t="n"/>
-      <c r="Z33" s="29" t="n"/>
+      <c r="Z33" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA33" s="28" t="n"/>
-      <c r="AB33" s="29" t="n"/>
+      <c r="AB33" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC33" s="28" t="n"/>
-      <c r="AD33" s="29" t="n"/>
+      <c r="AD33" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE33" s="10" t="n"/>
       <c r="AF33" s="10" t="n"/>
       <c r="AG33" s="10" t="n"/>
@@ -37947,27 +38783,71 @@
       </c>
       <c r="H34" s="27" t="n"/>
       <c r="I34" s="28" t="n"/>
-      <c r="J34" s="29" t="n"/>
+      <c r="J34" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K34" s="28" t="n"/>
-      <c r="L34" s="29" t="n"/>
+      <c r="L34" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M34" s="28" t="n"/>
-      <c r="N34" s="29" t="n"/>
+      <c r="N34" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O34" s="28" t="n"/>
-      <c r="P34" s="29" t="n"/>
+      <c r="P34" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q34" s="28" t="n"/>
-      <c r="R34" s="29" t="n"/>
+      <c r="R34" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S34" s="28" t="n"/>
-      <c r="T34" s="29" t="n"/>
+      <c r="T34" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U34" s="28" t="n"/>
-      <c r="V34" s="29" t="n"/>
+      <c r="V34" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W34" s="28" t="n"/>
-      <c r="X34" s="29" t="n"/>
+      <c r="X34" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y34" s="28" t="n"/>
-      <c r="Z34" s="29" t="n"/>
+      <c r="Z34" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA34" s="28" t="n"/>
-      <c r="AB34" s="29" t="n"/>
+      <c r="AB34" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC34" s="28" t="n"/>
-      <c r="AD34" s="29" t="n"/>
+      <c r="AD34" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE34" s="10" t="n"/>
       <c r="AF34" s="10" t="n"/>
       <c r="AG34" s="10" t="n"/>
@@ -38010,27 +38890,71 @@
       </c>
       <c r="H35" s="27" t="n"/>
       <c r="I35" s="28" t="n"/>
-      <c r="J35" s="29" t="n"/>
+      <c r="J35" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K35" s="28" t="n"/>
-      <c r="L35" s="29" t="n"/>
+      <c r="L35" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M35" s="28" t="n"/>
-      <c r="N35" s="29" t="n"/>
+      <c r="N35" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O35" s="28" t="n"/>
-      <c r="P35" s="29" t="n"/>
+      <c r="P35" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q35" s="28" t="n"/>
-      <c r="R35" s="29" t="n"/>
+      <c r="R35" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S35" s="28" t="n"/>
-      <c r="T35" s="29" t="n"/>
+      <c r="T35" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U35" s="28" t="n"/>
-      <c r="V35" s="29" t="n"/>
+      <c r="V35" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W35" s="28" t="n"/>
-      <c r="X35" s="29" t="n"/>
+      <c r="X35" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y35" s="28" t="n"/>
-      <c r="Z35" s="29" t="n"/>
+      <c r="Z35" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA35" s="28" t="n"/>
-      <c r="AB35" s="29" t="n"/>
+      <c r="AB35" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC35" s="28" t="n"/>
-      <c r="AD35" s="29" t="n"/>
+      <c r="AD35" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE35" s="10" t="n"/>
       <c r="AF35" s="10" t="n"/>
       <c r="AG35" s="10" t="n"/>
@@ -38073,27 +38997,71 @@
       </c>
       <c r="H36" s="27" t="n"/>
       <c r="I36" s="28" t="n"/>
-      <c r="J36" s="29" t="n"/>
+      <c r="J36" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K36" s="28" t="n"/>
-      <c r="L36" s="29" t="n"/>
+      <c r="L36" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M36" s="28" t="n"/>
-      <c r="N36" s="29" t="n"/>
+      <c r="N36" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O36" s="28" t="n"/>
-      <c r="P36" s="29" t="n"/>
+      <c r="P36" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q36" s="28" t="n"/>
-      <c r="R36" s="29" t="n"/>
+      <c r="R36" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S36" s="28" t="n"/>
-      <c r="T36" s="29" t="n"/>
+      <c r="T36" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U36" s="28" t="n"/>
-      <c r="V36" s="29" t="n"/>
+      <c r="V36" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W36" s="28" t="n"/>
-      <c r="X36" s="29" t="n"/>
+      <c r="X36" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y36" s="28" t="n"/>
-      <c r="Z36" s="29" t="n"/>
+      <c r="Z36" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA36" s="28" t="n"/>
-      <c r="AB36" s="29" t="n"/>
+      <c r="AB36" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC36" s="28" t="n"/>
-      <c r="AD36" s="29" t="n"/>
+      <c r="AD36" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE36" s="10" t="n"/>
       <c r="AF36" s="10" t="n"/>
       <c r="AG36" s="10" t="n"/>
@@ -38136,27 +39104,71 @@
       </c>
       <c r="H37" s="27" t="n"/>
       <c r="I37" s="28" t="n"/>
-      <c r="J37" s="29" t="n"/>
+      <c r="J37" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K37" s="28" t="n"/>
-      <c r="L37" s="29" t="n"/>
+      <c r="L37" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M37" s="28" t="n"/>
-      <c r="N37" s="29" t="n"/>
+      <c r="N37" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O37" s="28" t="n"/>
-      <c r="P37" s="29" t="n"/>
+      <c r="P37" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q37" s="28" t="n"/>
-      <c r="R37" s="29" t="n"/>
+      <c r="R37" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S37" s="28" t="n"/>
-      <c r="T37" s="29" t="n"/>
+      <c r="T37" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U37" s="28" t="n"/>
-      <c r="V37" s="29" t="n"/>
+      <c r="V37" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W37" s="28" t="n"/>
-      <c r="X37" s="29" t="n"/>
+      <c r="X37" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y37" s="28" t="n"/>
-      <c r="Z37" s="29" t="n"/>
+      <c r="Z37" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA37" s="28" t="n"/>
-      <c r="AB37" s="29" t="n"/>
+      <c r="AB37" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC37" s="28" t="n"/>
-      <c r="AD37" s="29" t="n"/>
+      <c r="AD37" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE37" s="10" t="n"/>
       <c r="AF37" s="10" t="n"/>
       <c r="AG37" s="10" t="n"/>
@@ -38489,27 +39501,71 @@
       </c>
       <c r="H40" s="27" t="n"/>
       <c r="I40" s="28" t="n"/>
-      <c r="J40" s="29" t="n"/>
+      <c r="J40" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K40" s="28" t="n"/>
-      <c r="L40" s="29" t="n"/>
+      <c r="L40" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M40" s="28" t="n"/>
-      <c r="N40" s="29" t="n"/>
+      <c r="N40" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O40" s="28" t="n"/>
-      <c r="P40" s="29" t="n"/>
+      <c r="P40" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q40" s="28" t="n"/>
-      <c r="R40" s="29" t="n"/>
+      <c r="R40" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S40" s="28" t="n"/>
-      <c r="T40" s="29" t="n"/>
+      <c r="T40" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U40" s="28" t="n"/>
-      <c r="V40" s="29" t="n"/>
+      <c r="V40" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W40" s="28" t="n"/>
-      <c r="X40" s="29" t="n"/>
+      <c r="X40" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y40" s="28" t="n"/>
-      <c r="Z40" s="29" t="n"/>
+      <c r="Z40" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA40" s="28" t="n"/>
-      <c r="AB40" s="29" t="n"/>
+      <c r="AB40" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC40" s="28" t="n"/>
-      <c r="AD40" s="29" t="n"/>
+      <c r="AD40" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE40" s="10" t="n"/>
       <c r="AF40" s="10" t="n"/>
       <c r="AG40" s="10" t="n"/>
@@ -38834,27 +39890,71 @@
       </c>
       <c r="H43" s="27" t="n"/>
       <c r="I43" s="28" t="n"/>
-      <c r="J43" s="29" t="n"/>
+      <c r="J43" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K43" s="28" t="n"/>
-      <c r="L43" s="29" t="n"/>
+      <c r="L43" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M43" s="28" t="n"/>
-      <c r="N43" s="29" t="n"/>
+      <c r="N43" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O43" s="28" t="n"/>
-      <c r="P43" s="29" t="n"/>
+      <c r="P43" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q43" s="28" t="n"/>
-      <c r="R43" s="29" t="n"/>
+      <c r="R43" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S43" s="28" t="n"/>
-      <c r="T43" s="29" t="n"/>
+      <c r="T43" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U43" s="28" t="n"/>
-      <c r="V43" s="29" t="n"/>
+      <c r="V43" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W43" s="28" t="n"/>
-      <c r="X43" s="29" t="n"/>
+      <c r="X43" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y43" s="28" t="n"/>
-      <c r="Z43" s="29" t="n"/>
+      <c r="Z43" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA43" s="28" t="n"/>
-      <c r="AB43" s="29" t="n"/>
+      <c r="AB43" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC43" s="28" t="n"/>
-      <c r="AD43" s="29" t="n"/>
+      <c r="AD43" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE43" s="10" t="n"/>
       <c r="AF43" s="10" t="n"/>
       <c r="AG43" s="10" t="n"/>
@@ -38897,27 +39997,71 @@
       </c>
       <c r="H44" s="27" t="n"/>
       <c r="I44" s="28" t="n"/>
-      <c r="J44" s="29" t="n"/>
+      <c r="J44" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K44" s="28" t="n"/>
-      <c r="L44" s="29" t="n"/>
+      <c r="L44" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M44" s="28" t="n"/>
-      <c r="N44" s="29" t="n"/>
+      <c r="N44" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O44" s="28" t="n"/>
-      <c r="P44" s="29" t="n"/>
+      <c r="P44" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q44" s="28" t="n"/>
-      <c r="R44" s="29" t="n"/>
+      <c r="R44" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S44" s="28" t="n"/>
-      <c r="T44" s="29" t="n"/>
+      <c r="T44" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U44" s="28" t="n"/>
-      <c r="V44" s="29" t="n"/>
+      <c r="V44" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W44" s="28" t="n"/>
-      <c r="X44" s="29" t="n"/>
+      <c r="X44" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y44" s="28" t="n"/>
-      <c r="Z44" s="29" t="n"/>
+      <c r="Z44" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA44" s="28" t="n"/>
-      <c r="AB44" s="29" t="n"/>
+      <c r="AB44" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC44" s="28" t="n"/>
-      <c r="AD44" s="29" t="n"/>
+      <c r="AD44" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE44" s="10" t="n"/>
       <c r="AF44" s="10" t="n"/>
       <c r="AG44" s="10" t="n"/>
@@ -41815,33 +42959,89 @@
           <t>AL02</t>
         </is>
       </c>
-      <c r="D2" s="29" t="n"/>
+      <c r="D2" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="E2" s="27" t="n"/>
-      <c r="F2" s="29" t="n"/>
+      <c r="F2" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="G2" s="27" t="n"/>
-      <c r="H2" s="29" t="n"/>
+      <c r="H2" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="I2" s="27" t="n"/>
-      <c r="J2" s="29" t="n"/>
+      <c r="J2" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K2" s="27" t="n"/>
-      <c r="L2" s="29" t="n"/>
+      <c r="L2" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M2" s="27" t="n"/>
-      <c r="N2" s="29" t="n"/>
+      <c r="N2" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O2" s="27" t="n"/>
-      <c r="P2" s="29" t="n"/>
+      <c r="P2" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q2" s="27" t="n"/>
-      <c r="R2" s="29" t="n"/>
+      <c r="R2" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S2" s="27" t="n"/>
-      <c r="T2" s="29" t="n"/>
+      <c r="T2" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U2" s="27" t="n"/>
-      <c r="V2" s="29" t="n"/>
+      <c r="V2" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W2" s="27" t="n"/>
-      <c r="X2" s="29" t="n"/>
+      <c r="X2" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y2" s="27" t="n"/>
-      <c r="Z2" s="29" t="n"/>
+      <c r="Z2" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA2" s="27" t="n"/>
-      <c r="AB2" s="29" t="n"/>
+      <c r="AB2" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC2" s="27" t="n"/>
-      <c r="AD2" s="29" t="n"/>
+      <c r="AD2" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE2" s="27" t="n"/>
       <c r="AF2" s="10" t="n"/>
       <c r="AG2" s="10" t="n"/>
@@ -41875,33 +43075,89 @@
           <t>AL03</t>
         </is>
       </c>
-      <c r="D3" s="29" t="n"/>
+      <c r="D3" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="E3" s="27" t="n"/>
-      <c r="F3" s="29" t="n"/>
+      <c r="F3" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="G3" s="27" t="n"/>
-      <c r="H3" s="29" t="n"/>
+      <c r="H3" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="I3" s="27" t="n"/>
-      <c r="J3" s="29" t="n"/>
+      <c r="J3" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K3" s="27" t="n"/>
-      <c r="L3" s="29" t="n"/>
+      <c r="L3" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M3" s="27" t="n"/>
-      <c r="N3" s="29" t="n"/>
+      <c r="N3" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O3" s="27" t="n"/>
-      <c r="P3" s="29" t="n"/>
+      <c r="P3" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q3" s="27" t="n"/>
-      <c r="R3" s="29" t="n"/>
+      <c r="R3" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S3" s="27" t="n"/>
-      <c r="T3" s="29" t="n"/>
+      <c r="T3" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U3" s="27" t="n"/>
-      <c r="V3" s="29" t="n"/>
+      <c r="V3" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W3" s="27" t="n"/>
-      <c r="X3" s="29" t="n"/>
+      <c r="X3" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y3" s="27" t="n"/>
-      <c r="Z3" s="29" t="n"/>
+      <c r="Z3" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA3" s="27" t="n"/>
-      <c r="AB3" s="29" t="n"/>
+      <c r="AB3" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC3" s="27" t="n"/>
-      <c r="AD3" s="29" t="n"/>
+      <c r="AD3" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE3" s="27" t="n"/>
       <c r="AF3" s="10" t="n"/>
       <c r="AG3" s="10" t="n"/>
@@ -41935,33 +43191,89 @@
           <t>AL04</t>
         </is>
       </c>
-      <c r="D4" s="29" t="n"/>
+      <c r="D4" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="E4" s="27" t="n"/>
-      <c r="F4" s="29" t="n"/>
+      <c r="F4" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="G4" s="27" t="n"/>
-      <c r="H4" s="29" t="n"/>
+      <c r="H4" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="I4" s="27" t="n"/>
-      <c r="J4" s="29" t="n"/>
+      <c r="J4" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K4" s="27" t="n"/>
-      <c r="L4" s="29" t="n"/>
+      <c r="L4" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M4" s="27" t="n"/>
-      <c r="N4" s="29" t="n"/>
+      <c r="N4" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O4" s="27" t="n"/>
-      <c r="P4" s="29" t="n"/>
+      <c r="P4" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q4" s="27" t="n"/>
-      <c r="R4" s="29" t="n"/>
+      <c r="R4" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S4" s="27" t="n"/>
-      <c r="T4" s="29" t="n"/>
+      <c r="T4" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U4" s="27" t="n"/>
-      <c r="V4" s="29" t="n"/>
+      <c r="V4" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W4" s="27" t="n"/>
-      <c r="X4" s="29" t="n"/>
+      <c r="X4" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y4" s="27" t="n"/>
-      <c r="Z4" s="29" t="n"/>
+      <c r="Z4" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA4" s="27" t="n"/>
-      <c r="AB4" s="29" t="n"/>
+      <c r="AB4" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC4" s="27" t="n"/>
-      <c r="AD4" s="29" t="n"/>
+      <c r="AD4" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE4" s="27" t="n"/>
       <c r="AF4" s="10" t="n"/>
       <c r="AG4" s="10" t="n"/>
@@ -41995,33 +43307,89 @@
           <t>AL05</t>
         </is>
       </c>
-      <c r="D5" s="29" t="n"/>
+      <c r="D5" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="E5" s="27" t="n"/>
-      <c r="F5" s="29" t="n"/>
+      <c r="F5" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="G5" s="27" t="n"/>
-      <c r="H5" s="29" t="n"/>
+      <c r="H5" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="I5" s="27" t="n"/>
-      <c r="J5" s="29" t="n"/>
+      <c r="J5" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K5" s="27" t="n"/>
-      <c r="L5" s="29" t="n"/>
+      <c r="L5" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M5" s="27" t="n"/>
-      <c r="N5" s="29" t="n"/>
+      <c r="N5" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O5" s="27" t="n"/>
-      <c r="P5" s="29" t="n"/>
+      <c r="P5" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q5" s="27" t="n"/>
-      <c r="R5" s="29" t="n"/>
+      <c r="R5" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S5" s="27" t="n"/>
-      <c r="T5" s="29" t="n"/>
+      <c r="T5" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U5" s="27" t="n"/>
-      <c r="V5" s="29" t="n"/>
+      <c r="V5" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W5" s="27" t="n"/>
-      <c r="X5" s="29" t="n"/>
+      <c r="X5" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y5" s="27" t="n"/>
-      <c r="Z5" s="29" t="n"/>
+      <c r="Z5" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA5" s="27" t="n"/>
-      <c r="AB5" s="29" t="n"/>
+      <c r="AB5" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC5" s="27" t="n"/>
-      <c r="AD5" s="29" t="n"/>
+      <c r="AD5" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE5" s="27" t="n"/>
       <c r="AF5" s="10" t="n"/>
       <c r="AG5" s="10" t="n"/>
@@ -42055,33 +43423,89 @@
           <t>AL06</t>
         </is>
       </c>
-      <c r="D6" s="29" t="n"/>
+      <c r="D6" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="E6" s="27" t="n"/>
-      <c r="F6" s="29" t="n"/>
+      <c r="F6" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="G6" s="27" t="n"/>
-      <c r="H6" s="29" t="n"/>
+      <c r="H6" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="I6" s="27" t="n"/>
-      <c r="J6" s="29" t="n"/>
+      <c r="J6" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K6" s="27" t="n"/>
-      <c r="L6" s="29" t="n"/>
+      <c r="L6" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M6" s="27" t="n"/>
-      <c r="N6" s="29" t="n"/>
+      <c r="N6" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O6" s="27" t="n"/>
-      <c r="P6" s="29" t="n"/>
+      <c r="P6" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q6" s="27" t="n"/>
-      <c r="R6" s="29" t="n"/>
+      <c r="R6" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S6" s="27" t="n"/>
-      <c r="T6" s="29" t="n"/>
+      <c r="T6" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U6" s="27" t="n"/>
-      <c r="V6" s="29" t="n"/>
+      <c r="V6" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W6" s="27" t="n"/>
-      <c r="X6" s="29" t="n"/>
+      <c r="X6" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y6" s="27" t="n"/>
-      <c r="Z6" s="29" t="n"/>
+      <c r="Z6" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA6" s="27" t="n"/>
-      <c r="AB6" s="29" t="n"/>
+      <c r="AB6" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC6" s="27" t="n"/>
-      <c r="AD6" s="29" t="n"/>
+      <c r="AD6" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE6" s="27" t="n"/>
       <c r="AF6" s="10" t="n"/>
       <c r="AG6" s="10" t="n"/>
@@ -42115,33 +43539,89 @@
           <t>AL07</t>
         </is>
       </c>
-      <c r="D7" s="29" t="n"/>
+      <c r="D7" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="E7" s="27" t="n"/>
-      <c r="F7" s="29" t="n"/>
+      <c r="F7" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="G7" s="27" t="n"/>
-      <c r="H7" s="29" t="n"/>
+      <c r="H7" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="I7" s="27" t="n"/>
-      <c r="J7" s="29" t="n"/>
+      <c r="J7" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K7" s="27" t="n"/>
-      <c r="L7" s="29" t="n"/>
+      <c r="L7" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M7" s="27" t="n"/>
-      <c r="N7" s="29" t="n"/>
+      <c r="N7" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O7" s="27" t="n"/>
-      <c r="P7" s="29" t="n"/>
+      <c r="P7" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q7" s="27" t="n"/>
-      <c r="R7" s="29" t="n"/>
+      <c r="R7" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S7" s="27" t="n"/>
-      <c r="T7" s="29" t="n"/>
+      <c r="T7" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U7" s="27" t="n"/>
-      <c r="V7" s="29" t="n"/>
+      <c r="V7" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W7" s="27" t="n"/>
-      <c r="X7" s="29" t="n"/>
+      <c r="X7" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y7" s="27" t="n"/>
-      <c r="Z7" s="29" t="n"/>
+      <c r="Z7" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA7" s="27" t="n"/>
-      <c r="AB7" s="29" t="n"/>
+      <c r="AB7" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC7" s="27" t="n"/>
-      <c r="AD7" s="29" t="n"/>
+      <c r="AD7" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE7" s="27" t="n"/>
       <c r="AF7" s="10" t="n"/>
       <c r="AG7" s="10" t="n"/>
@@ -42175,33 +43655,89 @@
           <t>AL08</t>
         </is>
       </c>
-      <c r="D8" s="29" t="n"/>
+      <c r="D8" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="E8" s="27" t="n"/>
-      <c r="F8" s="29" t="n"/>
+      <c r="F8" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="G8" s="27" t="n"/>
-      <c r="H8" s="29" t="n"/>
+      <c r="H8" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="I8" s="27" t="n"/>
-      <c r="J8" s="29" t="n"/>
+      <c r="J8" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K8" s="27" t="n"/>
-      <c r="L8" s="29" t="n"/>
+      <c r="L8" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M8" s="27" t="n"/>
-      <c r="N8" s="29" t="n"/>
+      <c r="N8" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O8" s="27" t="n"/>
-      <c r="P8" s="29" t="n"/>
+      <c r="P8" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q8" s="27" t="n"/>
-      <c r="R8" s="29" t="n"/>
+      <c r="R8" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S8" s="27" t="n"/>
-      <c r="T8" s="29" t="n"/>
+      <c r="T8" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U8" s="27" t="n"/>
-      <c r="V8" s="29" t="n"/>
+      <c r="V8" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W8" s="27" t="n"/>
-      <c r="X8" s="29" t="n"/>
+      <c r="X8" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y8" s="27" t="n"/>
-      <c r="Z8" s="29" t="n"/>
+      <c r="Z8" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA8" s="27" t="n"/>
-      <c r="AB8" s="29" t="n"/>
+      <c r="AB8" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC8" s="27" t="n"/>
-      <c r="AD8" s="29" t="n"/>
+      <c r="AD8" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE8" s="27" t="n"/>
       <c r="AF8" s="10" t="n"/>
       <c r="AG8" s="10" t="n"/>
@@ -42235,33 +43771,89 @@
           <t>AL09</t>
         </is>
       </c>
-      <c r="D9" s="29" t="n"/>
+      <c r="D9" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="E9" s="27" t="n"/>
-      <c r="F9" s="29" t="n"/>
+      <c r="F9" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="G9" s="27" t="n"/>
-      <c r="H9" s="29" t="n"/>
+      <c r="H9" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="I9" s="27" t="n"/>
-      <c r="J9" s="29" t="n"/>
+      <c r="J9" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K9" s="27" t="n"/>
-      <c r="L9" s="29" t="n"/>
+      <c r="L9" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M9" s="27" t="n"/>
-      <c r="N9" s="29" t="n"/>
+      <c r="N9" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O9" s="27" t="n"/>
-      <c r="P9" s="29" t="n"/>
+      <c r="P9" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q9" s="27" t="n"/>
-      <c r="R9" s="29" t="n"/>
+      <c r="R9" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S9" s="27" t="n"/>
-      <c r="T9" s="29" t="n"/>
+      <c r="T9" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U9" s="27" t="n"/>
-      <c r="V9" s="29" t="n"/>
+      <c r="V9" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W9" s="27" t="n"/>
-      <c r="X9" s="29" t="n"/>
+      <c r="X9" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y9" s="27" t="n"/>
-      <c r="Z9" s="29" t="n"/>
+      <c r="Z9" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA9" s="27" t="n"/>
-      <c r="AB9" s="29" t="n"/>
+      <c r="AB9" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC9" s="27" t="n"/>
-      <c r="AD9" s="29" t="n"/>
+      <c r="AD9" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE9" s="27" t="n"/>
       <c r="AF9" s="10" t="n"/>
       <c r="AG9" s="10" t="n"/>
@@ -42295,33 +43887,89 @@
           <t>BL01</t>
         </is>
       </c>
-      <c r="D10" s="29" t="n"/>
+      <c r="D10" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="E10" s="27" t="n"/>
-      <c r="F10" s="29" t="n"/>
+      <c r="F10" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="G10" s="27" t="n"/>
-      <c r="H10" s="29" t="n"/>
+      <c r="H10" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="I10" s="27" t="n"/>
-      <c r="J10" s="29" t="n"/>
+      <c r="J10" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K10" s="27" t="n"/>
-      <c r="L10" s="29" t="n"/>
+      <c r="L10" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M10" s="27" t="n"/>
-      <c r="N10" s="29" t="n"/>
+      <c r="N10" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O10" s="27" t="n"/>
-      <c r="P10" s="29" t="n"/>
+      <c r="P10" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q10" s="27" t="n"/>
-      <c r="R10" s="29" t="n"/>
+      <c r="R10" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S10" s="27" t="n"/>
-      <c r="T10" s="29" t="n"/>
+      <c r="T10" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U10" s="27" t="n"/>
-      <c r="V10" s="29" t="n"/>
+      <c r="V10" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W10" s="27" t="n"/>
-      <c r="X10" s="29" t="n"/>
+      <c r="X10" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y10" s="27" t="n"/>
-      <c r="Z10" s="29" t="n"/>
+      <c r="Z10" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA10" s="27" t="n"/>
-      <c r="AB10" s="29" t="n"/>
+      <c r="AB10" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC10" s="27" t="n"/>
-      <c r="AD10" s="29" t="n"/>
+      <c r="AD10" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE10" s="27" t="n"/>
       <c r="AF10" s="10" t="n"/>
       <c r="AG10" s="10" t="n"/>
@@ -42355,33 +44003,89 @@
           <t>BL02</t>
         </is>
       </c>
-      <c r="D11" s="29" t="n"/>
+      <c r="D11" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="E11" s="27" t="n"/>
-      <c r="F11" s="29" t="n"/>
+      <c r="F11" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="G11" s="27" t="n"/>
-      <c r="H11" s="29" t="n"/>
+      <c r="H11" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="I11" s="27" t="n"/>
-      <c r="J11" s="29" t="n"/>
+      <c r="J11" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K11" s="27" t="n"/>
-      <c r="L11" s="29" t="n"/>
+      <c r="L11" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M11" s="27" t="n"/>
-      <c r="N11" s="29" t="n"/>
+      <c r="N11" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O11" s="27" t="n"/>
-      <c r="P11" s="29" t="n"/>
+      <c r="P11" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q11" s="27" t="n"/>
-      <c r="R11" s="29" t="n"/>
+      <c r="R11" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S11" s="27" t="n"/>
-      <c r="T11" s="29" t="n"/>
+      <c r="T11" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U11" s="27" t="n"/>
-      <c r="V11" s="29" t="n"/>
+      <c r="V11" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W11" s="27" t="n"/>
-      <c r="X11" s="29" t="n"/>
+      <c r="X11" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y11" s="27" t="n"/>
-      <c r="Z11" s="29" t="n"/>
+      <c r="Z11" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA11" s="27" t="n"/>
-      <c r="AB11" s="29" t="n"/>
+      <c r="AB11" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC11" s="27" t="n"/>
-      <c r="AD11" s="29" t="n"/>
+      <c r="AD11" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE11" s="27" t="n"/>
       <c r="AF11" s="10" t="n"/>
       <c r="AG11" s="10" t="n"/>
@@ -42415,33 +44119,89 @@
           <t>BL03</t>
         </is>
       </c>
-      <c r="D12" s="29" t="n"/>
+      <c r="D12" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="E12" s="27" t="n"/>
-      <c r="F12" s="29" t="n"/>
+      <c r="F12" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="G12" s="27" t="n"/>
-      <c r="H12" s="29" t="n"/>
+      <c r="H12" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="I12" s="27" t="n"/>
-      <c r="J12" s="29" t="n"/>
+      <c r="J12" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K12" s="27" t="n"/>
-      <c r="L12" s="29" t="n"/>
+      <c r="L12" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M12" s="27" t="n"/>
-      <c r="N12" s="29" t="n"/>
+      <c r="N12" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O12" s="27" t="n"/>
-      <c r="P12" s="29" t="n"/>
+      <c r="P12" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q12" s="27" t="n"/>
-      <c r="R12" s="29" t="n"/>
+      <c r="R12" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S12" s="27" t="n"/>
-      <c r="T12" s="29" t="n"/>
+      <c r="T12" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U12" s="27" t="n"/>
-      <c r="V12" s="29" t="n"/>
+      <c r="V12" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W12" s="27" t="n"/>
-      <c r="X12" s="29" t="n"/>
+      <c r="X12" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y12" s="27" t="n"/>
-      <c r="Z12" s="29" t="n"/>
+      <c r="Z12" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA12" s="27" t="n"/>
-      <c r="AB12" s="29" t="n"/>
+      <c r="AB12" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC12" s="27" t="n"/>
-      <c r="AD12" s="29" t="n"/>
+      <c r="AD12" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE12" s="27" t="n"/>
       <c r="AF12" s="10" t="n"/>
       <c r="AG12" s="10" t="n"/>
@@ -42475,33 +44235,89 @@
           <t>BL04</t>
         </is>
       </c>
-      <c r="D13" s="29" t="n"/>
+      <c r="D13" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="E13" s="27" t="n"/>
-      <c r="F13" s="29" t="n"/>
+      <c r="F13" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="G13" s="27" t="n"/>
-      <c r="H13" s="29" t="n"/>
+      <c r="H13" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="I13" s="27" t="n"/>
-      <c r="J13" s="29" t="n"/>
+      <c r="J13" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K13" s="27" t="n"/>
-      <c r="L13" s="29" t="n"/>
+      <c r="L13" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M13" s="27" t="n"/>
-      <c r="N13" s="29" t="n"/>
+      <c r="N13" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O13" s="27" t="n"/>
-      <c r="P13" s="29" t="n"/>
+      <c r="P13" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q13" s="27" t="n"/>
-      <c r="R13" s="29" t="n"/>
+      <c r="R13" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S13" s="27" t="n"/>
-      <c r="T13" s="29" t="n"/>
+      <c r="T13" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U13" s="27" t="n"/>
-      <c r="V13" s="29" t="n"/>
+      <c r="V13" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W13" s="27" t="n"/>
-      <c r="X13" s="29" t="n"/>
+      <c r="X13" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y13" s="27" t="n"/>
-      <c r="Z13" s="29" t="n"/>
+      <c r="Z13" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA13" s="27" t="n"/>
-      <c r="AB13" s="29" t="n"/>
+      <c r="AB13" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC13" s="27" t="n"/>
-      <c r="AD13" s="29" t="n"/>
+      <c r="AD13" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE13" s="27" t="n"/>
       <c r="AF13" s="10" t="n"/>
       <c r="AG13" s="10" t="n"/>
@@ -42535,33 +44351,89 @@
           <t>BL05</t>
         </is>
       </c>
-      <c r="D14" s="29" t="n"/>
+      <c r="D14" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="E14" s="27" t="n"/>
-      <c r="F14" s="29" t="n"/>
+      <c r="F14" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="G14" s="27" t="n"/>
-      <c r="H14" s="29" t="n"/>
+      <c r="H14" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="I14" s="27" t="n"/>
-      <c r="J14" s="29" t="n"/>
+      <c r="J14" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K14" s="27" t="n"/>
-      <c r="L14" s="29" t="n"/>
+      <c r="L14" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M14" s="27" t="n"/>
-      <c r="N14" s="29" t="n"/>
+      <c r="N14" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O14" s="27" t="n"/>
-      <c r="P14" s="29" t="n"/>
+      <c r="P14" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q14" s="27" t="n"/>
-      <c r="R14" s="29" t="n"/>
+      <c r="R14" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S14" s="27" t="n"/>
-      <c r="T14" s="29" t="n"/>
+      <c r="T14" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U14" s="27" t="n"/>
-      <c r="V14" s="29" t="n"/>
+      <c r="V14" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W14" s="27" t="n"/>
-      <c r="X14" s="29" t="n"/>
+      <c r="X14" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y14" s="27" t="n"/>
-      <c r="Z14" s="29" t="n"/>
+      <c r="Z14" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA14" s="27" t="n"/>
-      <c r="AB14" s="29" t="n"/>
+      <c r="AB14" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC14" s="27" t="n"/>
-      <c r="AD14" s="29" t="n"/>
+      <c r="AD14" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE14" s="27" t="n"/>
       <c r="AF14" s="10" t="n"/>
       <c r="AG14" s="10" t="n"/>
@@ -42595,33 +44467,89 @@
           <t>BL06</t>
         </is>
       </c>
-      <c r="D15" s="29" t="n"/>
+      <c r="D15" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="E15" s="27" t="n"/>
-      <c r="F15" s="29" t="n"/>
+      <c r="F15" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="G15" s="27" t="n"/>
-      <c r="H15" s="29" t="n"/>
+      <c r="H15" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="I15" s="27" t="n"/>
-      <c r="J15" s="29" t="n"/>
+      <c r="J15" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K15" s="27" t="n"/>
-      <c r="L15" s="29" t="n"/>
+      <c r="L15" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M15" s="27" t="n"/>
-      <c r="N15" s="29" t="n"/>
+      <c r="N15" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O15" s="27" t="n"/>
-      <c r="P15" s="29" t="n"/>
+      <c r="P15" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q15" s="27" t="n"/>
-      <c r="R15" s="29" t="n"/>
+      <c r="R15" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S15" s="27" t="n"/>
-      <c r="T15" s="29" t="n"/>
+      <c r="T15" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U15" s="27" t="n"/>
-      <c r="V15" s="29" t="n"/>
+      <c r="V15" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W15" s="27" t="n"/>
-      <c r="X15" s="29" t="n"/>
+      <c r="X15" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y15" s="27" t="n"/>
-      <c r="Z15" s="29" t="n"/>
+      <c r="Z15" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA15" s="27" t="n"/>
-      <c r="AB15" s="29" t="n"/>
+      <c r="AB15" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC15" s="27" t="n"/>
-      <c r="AD15" s="29" t="n"/>
+      <c r="AD15" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE15" s="27" t="n"/>
       <c r="AF15" s="10" t="n"/>
       <c r="AG15" s="10" t="n"/>
@@ -42655,33 +44583,89 @@
           <t>BL07</t>
         </is>
       </c>
-      <c r="D16" s="29" t="n"/>
+      <c r="D16" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="E16" s="27" t="n"/>
-      <c r="F16" s="29" t="n"/>
+      <c r="F16" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="G16" s="27" t="n"/>
-      <c r="H16" s="29" t="n"/>
+      <c r="H16" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="I16" s="27" t="n"/>
-      <c r="J16" s="29" t="n"/>
+      <c r="J16" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K16" s="27" t="n"/>
-      <c r="L16" s="29" t="n"/>
+      <c r="L16" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M16" s="27" t="n"/>
-      <c r="N16" s="29" t="n"/>
+      <c r="N16" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O16" s="27" t="n"/>
-      <c r="P16" s="29" t="n"/>
+      <c r="P16" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q16" s="27" t="n"/>
-      <c r="R16" s="29" t="n"/>
+      <c r="R16" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S16" s="27" t="n"/>
-      <c r="T16" s="29" t="n"/>
+      <c r="T16" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U16" s="27" t="n"/>
-      <c r="V16" s="29" t="n"/>
+      <c r="V16" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W16" s="27" t="n"/>
-      <c r="X16" s="29" t="n"/>
+      <c r="X16" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y16" s="27" t="n"/>
-      <c r="Z16" s="29" t="n"/>
+      <c r="Z16" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA16" s="27" t="n"/>
-      <c r="AB16" s="29" t="n"/>
+      <c r="AB16" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC16" s="27" t="n"/>
-      <c r="AD16" s="29" t="n"/>
+      <c r="AD16" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE16" s="27" t="n"/>
       <c r="AF16" s="10" t="n"/>
       <c r="AG16" s="10" t="n"/>
@@ -42715,33 +44699,89 @@
           <t>BL08</t>
         </is>
       </c>
-      <c r="D17" s="29" t="n"/>
+      <c r="D17" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="E17" s="27" t="n"/>
-      <c r="F17" s="29" t="n"/>
+      <c r="F17" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="G17" s="27" t="n"/>
-      <c r="H17" s="29" t="n"/>
+      <c r="H17" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="I17" s="27" t="n"/>
-      <c r="J17" s="29" t="n"/>
+      <c r="J17" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K17" s="27" t="n"/>
-      <c r="L17" s="29" t="n"/>
+      <c r="L17" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M17" s="27" t="n"/>
-      <c r="N17" s="29" t="n"/>
+      <c r="N17" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O17" s="27" t="n"/>
-      <c r="P17" s="29" t="n"/>
+      <c r="P17" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q17" s="27" t="n"/>
-      <c r="R17" s="29" t="n"/>
+      <c r="R17" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S17" s="27" t="n"/>
-      <c r="T17" s="29" t="n"/>
+      <c r="T17" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U17" s="27" t="n"/>
-      <c r="V17" s="29" t="n"/>
+      <c r="V17" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W17" s="27" t="n"/>
-      <c r="X17" s="29" t="n"/>
+      <c r="X17" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y17" s="27" t="n"/>
-      <c r="Z17" s="29" t="n"/>
+      <c r="Z17" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA17" s="27" t="n"/>
-      <c r="AB17" s="29" t="n"/>
+      <c r="AB17" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC17" s="27" t="n"/>
-      <c r="AD17" s="29" t="n"/>
+      <c r="AD17" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE17" s="27" t="n"/>
       <c r="AF17" s="10" t="n"/>
       <c r="AG17" s="10" t="n"/>
@@ -42775,33 +44815,89 @@
           <t>BL09</t>
         </is>
       </c>
-      <c r="D18" s="29" t="n"/>
+      <c r="D18" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="E18" s="27" t="n"/>
-      <c r="F18" s="29" t="n"/>
+      <c r="F18" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="G18" s="27" t="n"/>
-      <c r="H18" s="29" t="n"/>
+      <c r="H18" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="I18" s="27" t="n"/>
-      <c r="J18" s="29" t="n"/>
+      <c r="J18" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="K18" s="27" t="n"/>
-      <c r="L18" s="29" t="n"/>
+      <c r="L18" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="M18" s="27" t="n"/>
-      <c r="N18" s="29" t="n"/>
+      <c r="N18" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="O18" s="27" t="n"/>
-      <c r="P18" s="29" t="n"/>
+      <c r="P18" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Q18" s="27" t="n"/>
-      <c r="R18" s="29" t="n"/>
+      <c r="R18" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="S18" s="27" t="n"/>
-      <c r="T18" s="29" t="n"/>
+      <c r="T18" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="U18" s="27" t="n"/>
-      <c r="V18" s="29" t="n"/>
+      <c r="V18" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="W18" s="27" t="n"/>
-      <c r="X18" s="29" t="n"/>
+      <c r="X18" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="Y18" s="27" t="n"/>
-      <c r="Z18" s="29" t="n"/>
+      <c r="Z18" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AA18" s="27" t="n"/>
-      <c r="AB18" s="29" t="n"/>
+      <c r="AB18" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AC18" s="27" t="n"/>
-      <c r="AD18" s="29" t="n"/>
+      <c r="AD18" s="29" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
       <c r="AE18" s="27" t="n"/>
       <c r="AF18" s="10" t="n"/>
       <c r="AG18" s="10" t="n"/>

</xml_diff>

<commit_message>
All coordination sketches set to Not Provided
</commit_message>
<xml_diff>
--- a/WPH_Room_Register.xlsx
+++ b/WPH_Room_Register.xlsx
@@ -35303,7 +35303,7 @@
       </c>
       <c r="D4" s="26" t="inlineStr">
         <is>
-          <t>Provided</t>
+          <t>Not Provided</t>
         </is>
       </c>
       <c r="E4" s="27" t="n"/>
@@ -35561,7 +35561,11 @@
           <t>(no drawing number in legend)</t>
         </is>
       </c>
-      <c r="D6" s="26" t="n"/>
+      <c r="D6" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E6" s="27" t="n"/>
       <c r="F6" s="28" t="n"/>
       <c r="G6" s="29" t="inlineStr">
@@ -36486,7 +36490,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-40301</t>
         </is>
       </c>
-      <c r="D13" s="26" t="n"/>
+      <c r="D13" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E13" s="27" t="n"/>
       <c r="F13" s="28" t="n"/>
       <c r="G13" s="29" t="inlineStr">
@@ -36593,7 +36601,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-40301</t>
         </is>
       </c>
-      <c r="D14" s="26" t="n"/>
+      <c r="D14" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E14" s="27" t="n"/>
       <c r="F14" s="28" t="n"/>
       <c r="G14" s="29" t="inlineStr">
@@ -36700,7 +36712,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-40301</t>
         </is>
       </c>
-      <c r="D15" s="26" t="n"/>
+      <c r="D15" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E15" s="27" t="n"/>
       <c r="F15" s="28" t="n"/>
       <c r="G15" s="29" t="inlineStr">
@@ -36807,7 +36823,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-40301</t>
         </is>
       </c>
-      <c r="D16" s="26" t="n"/>
+      <c r="D16" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E16" s="27" t="n"/>
       <c r="F16" s="28" t="n"/>
       <c r="G16" s="29" t="inlineStr">
@@ -36914,7 +36934,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-40301</t>
         </is>
       </c>
-      <c r="D17" s="26" t="n"/>
+      <c r="D17" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E17" s="27" t="n"/>
       <c r="F17" s="28" t="n"/>
       <c r="G17" s="29" t="inlineStr">
@@ -37021,7 +37045,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-40301</t>
         </is>
       </c>
-      <c r="D18" s="26" t="n"/>
+      <c r="D18" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E18" s="27" t="n"/>
       <c r="F18" s="28" t="n"/>
       <c r="G18" s="29" t="inlineStr">
@@ -37128,7 +37156,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-40701</t>
         </is>
       </c>
-      <c r="D19" s="26" t="n"/>
+      <c r="D19" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E19" s="27" t="n"/>
       <c r="F19" s="28" t="n"/>
       <c r="G19" s="29" t="inlineStr">
@@ -37235,7 +37267,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-40701</t>
         </is>
       </c>
-      <c r="D20" s="26" t="n"/>
+      <c r="D20" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E20" s="27" t="n"/>
       <c r="F20" s="28" t="n"/>
       <c r="G20" s="29" t="inlineStr">
@@ -37342,7 +37378,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-40701</t>
         </is>
       </c>
-      <c r="D21" s="26" t="n"/>
+      <c r="D21" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E21" s="27" t="n"/>
       <c r="F21" s="28" t="n"/>
       <c r="G21" s="29" t="inlineStr">
@@ -37449,7 +37489,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-40701</t>
         </is>
       </c>
-      <c r="D22" s="26" t="n"/>
+      <c r="D22" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E22" s="27" t="n"/>
       <c r="F22" s="28" t="n"/>
       <c r="G22" s="29" t="inlineStr">
@@ -37556,7 +37600,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-40701</t>
         </is>
       </c>
-      <c r="D23" s="26" t="n"/>
+      <c r="D23" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E23" s="27" t="n"/>
       <c r="F23" s="28" t="n"/>
       <c r="G23" s="29" t="inlineStr">
@@ -37663,7 +37711,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-40701</t>
         </is>
       </c>
-      <c r="D24" s="26" t="n"/>
+      <c r="D24" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E24" s="27" t="n"/>
       <c r="F24" s="28" t="n"/>
       <c r="G24" s="29" t="inlineStr">
@@ -37770,7 +37822,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-40701</t>
         </is>
       </c>
-      <c r="D25" s="26" t="n"/>
+      <c r="D25" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E25" s="27" t="n"/>
       <c r="F25" s="28" t="n"/>
       <c r="G25" s="29" t="inlineStr">
@@ -38238,7 +38294,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-41401</t>
         </is>
       </c>
-      <c r="D29" s="26" t="n"/>
+      <c r="D29" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E29" s="27" t="n"/>
       <c r="F29" s="28" t="n"/>
       <c r="G29" s="29" t="inlineStr">
@@ -38345,7 +38405,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-41401</t>
         </is>
       </c>
-      <c r="D30" s="26" t="n"/>
+      <c r="D30" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E30" s="27" t="n"/>
       <c r="F30" s="28" t="n"/>
       <c r="G30" s="29" t="inlineStr">
@@ -38452,7 +38516,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-41401</t>
         </is>
       </c>
-      <c r="D31" s="26" t="n"/>
+      <c r="D31" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E31" s="27" t="n"/>
       <c r="F31" s="28" t="n"/>
       <c r="G31" s="29" t="inlineStr">
@@ -38559,7 +38627,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-41601</t>
         </is>
       </c>
-      <c r="D32" s="26" t="n"/>
+      <c r="D32" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E32" s="27" t="n"/>
       <c r="F32" s="28" t="n"/>
       <c r="G32" s="29" t="inlineStr">
@@ -38666,7 +38738,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-41601</t>
         </is>
       </c>
-      <c r="D33" s="26" t="n"/>
+      <c r="D33" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E33" s="27" t="n"/>
       <c r="F33" s="28" t="n"/>
       <c r="G33" s="29" t="inlineStr">
@@ -38773,7 +38849,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-41601</t>
         </is>
       </c>
-      <c r="D34" s="26" t="n"/>
+      <c r="D34" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E34" s="27" t="n"/>
       <c r="F34" s="28" t="n"/>
       <c r="G34" s="29" t="inlineStr">
@@ -38880,7 +38960,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-41601</t>
         </is>
       </c>
-      <c r="D35" s="26" t="n"/>
+      <c r="D35" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E35" s="27" t="n"/>
       <c r="F35" s="28" t="n"/>
       <c r="G35" s="29" t="inlineStr">
@@ -38987,7 +39071,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-41601</t>
         </is>
       </c>
-      <c r="D36" s="26" t="n"/>
+      <c r="D36" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E36" s="27" t="n"/>
       <c r="F36" s="28" t="n"/>
       <c r="G36" s="29" t="inlineStr">
@@ -39094,7 +39182,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-41601</t>
         </is>
       </c>
-      <c r="D37" s="26" t="n"/>
+      <c r="D37" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E37" s="27" t="n"/>
       <c r="F37" s="28" t="n"/>
       <c r="G37" s="29" t="inlineStr">
@@ -39491,7 +39583,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-42101</t>
         </is>
       </c>
-      <c r="D40" s="26" t="n"/>
+      <c r="D40" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E40" s="27" t="n"/>
       <c r="F40" s="28" t="n"/>
       <c r="G40" s="29" t="inlineStr">
@@ -39880,7 +39976,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-41801</t>
         </is>
       </c>
-      <c r="D43" s="26" t="n"/>
+      <c r="D43" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E43" s="27" t="n"/>
       <c r="F43" s="28" t="n"/>
       <c r="G43" s="29" t="inlineStr">
@@ -39987,7 +40087,11 @@
           <t>WPH-ETC-DRW-SDW-IND-00-ZZZ-41801</t>
         </is>
       </c>
-      <c r="D44" s="26" t="n"/>
+      <c r="D44" s="26" t="inlineStr">
+        <is>
+          <t>Not Provided</t>
+        </is>
+      </c>
       <c r="E44" s="27" t="n"/>
       <c r="F44" s="28" t="n"/>
       <c r="G44" s="29" t="inlineStr">
@@ -40811,7 +40915,7 @@
       </c>
       <c r="D50" s="26" t="inlineStr">
         <is>
-          <t>Provided</t>
+          <t>Not Provided</t>
         </is>
       </c>
       <c r="E50" s="27" t="n"/>

</xml_diff>

<commit_message>
FLS Steel Doors material and shop drawing set to B
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AxwUpNTzQx5sXM23V5WdKL
</commit_message>
<xml_diff>
--- a/WPH_Room_Register.xlsx
+++ b/WPH_Room_Register.xlsx
@@ -43065,13 +43065,13 @@
       </c>
       <c r="D2" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E2" s="27" t="n"/>
       <c r="F2" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G2" s="27" t="n"/>
@@ -43181,13 +43181,13 @@
       </c>
       <c r="D3" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E3" s="27" t="n"/>
       <c r="F3" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G3" s="27" t="n"/>
@@ -43297,13 +43297,13 @@
       </c>
       <c r="D4" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E4" s="27" t="n"/>
       <c r="F4" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G4" s="27" t="n"/>
@@ -43413,13 +43413,13 @@
       </c>
       <c r="D5" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E5" s="27" t="n"/>
       <c r="F5" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G5" s="27" t="n"/>
@@ -43529,13 +43529,13 @@
       </c>
       <c r="D6" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E6" s="27" t="n"/>
       <c r="F6" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G6" s="27" t="n"/>
@@ -43645,13 +43645,13 @@
       </c>
       <c r="D7" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E7" s="27" t="n"/>
       <c r="F7" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G7" s="27" t="n"/>
@@ -43761,13 +43761,13 @@
       </c>
       <c r="D8" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E8" s="27" t="n"/>
       <c r="F8" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G8" s="27" t="n"/>
@@ -43877,13 +43877,13 @@
       </c>
       <c r="D9" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E9" s="27" t="n"/>
       <c r="F9" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G9" s="27" t="n"/>
@@ -43993,13 +43993,13 @@
       </c>
       <c r="D10" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E10" s="27" t="n"/>
       <c r="F10" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G10" s="27" t="n"/>
@@ -44109,13 +44109,13 @@
       </c>
       <c r="D11" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E11" s="27" t="n"/>
       <c r="F11" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G11" s="27" t="n"/>
@@ -44225,13 +44225,13 @@
       </c>
       <c r="D12" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E12" s="27" t="n"/>
       <c r="F12" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G12" s="27" t="n"/>
@@ -44341,13 +44341,13 @@
       </c>
       <c r="D13" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E13" s="27" t="n"/>
       <c r="F13" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G13" s="27" t="n"/>
@@ -44457,13 +44457,13 @@
       </c>
       <c r="D14" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E14" s="27" t="n"/>
       <c r="F14" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G14" s="27" t="n"/>
@@ -44573,13 +44573,13 @@
       </c>
       <c r="D15" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E15" s="27" t="n"/>
       <c r="F15" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G15" s="27" t="n"/>
@@ -44689,13 +44689,13 @@
       </c>
       <c r="D16" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E16" s="27" t="n"/>
       <c r="F16" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G16" s="27" t="n"/>
@@ -44805,13 +44805,13 @@
       </c>
       <c r="D17" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E17" s="27" t="n"/>
       <c r="F17" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G17" s="27" t="n"/>
@@ -44921,13 +44921,13 @@
       </c>
       <c r="D18" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E18" s="27" t="n"/>
       <c r="F18" s="29" t="inlineStr">
         <is>
-          <t>TBS</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G18" s="27" t="n"/>

</xml_diff>